<commit_message>
Ajout des éléments du premier atelier
</commit_message>
<xml_diff>
--- a/EBIOS_RM_Classeur.xlsx
+++ b/EBIOS_RM_Classeur.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fonda\Documents\1 - Portfolio\BACKUP\1 - Python script backup file tree\2 - Learning\4 - Cours\7 - Cours Cyber\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fonda\Documents\1 - Portfolio\BACKUP\1 - Python script backup file tree\2 - Learning\4 - Cours\7 - Cours Cyber\TP2_EBIOS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9077BE5-E20F-4491-9DC7-BCF67E1A5878}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{332F6E16-9D62-4B48-9FA5-028812EB880D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="992" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="992" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Organisation" sheetId="1" r:id="rId1"/>
@@ -2692,7 +2692,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="178">
+  <cellXfs count="184">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2924,16 +2924,10 @@
     <xf numFmtId="0" fontId="0" fillId="21" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2941,9 +2935,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="26" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3081,29 +3072,53 @@
     <xf numFmtId="0" fontId="1" fillId="37" borderId="0" xfId="5" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="34" borderId="0" xfId="5" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="5" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="24" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="21" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="23" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="24" borderId="26" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="15" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3132,16 +3147,52 @@
     <xf numFmtId="0" fontId="12" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="23" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="41" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="41" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="22" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="22" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="22" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="23" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="23" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="23" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3153,65 +3204,32 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="34" borderId="0" xfId="5" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="5" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="24" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="24" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="24" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="21" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="23" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="23" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="24" borderId="26" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="23" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="23" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="22" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="22" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="22" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="23" borderId="41" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="23" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="24" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="24" borderId="41" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="24" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -15803,7 +15821,7 @@
       <c r="A1" s="74" t="s">
         <v>132</v>
       </c>
-      <c r="B1" s="85" t="s">
+      <c r="B1" s="82" t="s">
         <v>133</v>
       </c>
     </row>
@@ -15811,7 +15829,7 @@
       <c r="A2" s="76" t="s">
         <v>290</v>
       </c>
-      <c r="B2" s="98" t="s">
+      <c r="B2" s="95" t="s">
         <v>291</v>
       </c>
     </row>
@@ -15945,40 +15963,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="114" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="99" t="s">
+      <c r="A1" s="96" t="s">
         <v>134</v>
       </c>
-      <c r="B1" s="100" t="s">
+      <c r="B1" s="97" t="s">
         <v>135</v>
       </c>
-      <c r="C1" s="101" t="s">
+      <c r="C1" s="98" t="s">
         <v>135</v>
       </c>
-      <c r="D1" s="101" t="s">
+      <c r="D1" s="98" t="s">
         <v>136</v>
       </c>
-      <c r="E1" s="102" t="s">
+      <c r="E1" s="99" t="s">
         <v>137</v>
       </c>
-      <c r="F1" s="102" t="s">
+      <c r="F1" s="99" t="s">
         <v>108</v>
       </c>
-      <c r="G1" s="103" t="s">
+      <c r="G1" s="100" t="s">
         <v>138</v>
       </c>
-      <c r="H1" s="104" t="s">
+      <c r="H1" s="101" t="s">
         <v>139</v>
       </c>
-      <c r="I1" s="104" t="s">
+      <c r="I1" s="101" t="s">
         <v>140</v>
       </c>
-      <c r="J1" s="104" t="s">
+      <c r="J1" s="101" t="s">
         <v>14</v>
       </c>
-      <c r="K1" s="105" t="s">
+      <c r="K1" s="102" t="s">
         <v>141</v>
       </c>
-      <c r="L1" s="105" t="s">
+      <c r="L1" s="102" t="s">
         <v>142</v>
       </c>
     </row>
@@ -15989,16 +16007,16 @@
       <c r="B2" s="75" t="s">
         <v>309</v>
       </c>
-      <c r="C2" s="78" t="s">
+      <c r="C2" s="77" t="s">
         <v>71</v>
       </c>
-      <c r="D2" s="106" t="s">
+      <c r="D2" s="103" t="s">
         <v>144</v>
       </c>
       <c r="E2" s="75" t="s">
         <v>296</v>
       </c>
-      <c r="F2" s="86" t="s">
+      <c r="F2" s="83" t="s">
         <v>297</v>
       </c>
       <c r="G2" s="75" t="s">
@@ -16010,13 +16028,13 @@
       <c r="I2" s="75" t="s">
         <v>508</v>
       </c>
-      <c r="J2" s="79">
+      <c r="J2" s="78">
         <v>4</v>
       </c>
       <c r="K2" s="75" t="s">
         <v>146</v>
       </c>
-      <c r="L2" s="107">
+      <c r="L2" s="104">
         <v>3</v>
       </c>
     </row>
@@ -16027,16 +16045,16 @@
       <c r="B3" s="75" t="s">
         <v>310</v>
       </c>
-      <c r="C3" s="79" t="s">
+      <c r="C3" s="78" t="s">
         <v>66</v>
       </c>
-      <c r="D3" s="106" t="s">
+      <c r="D3" s="103" t="s">
         <v>144</v>
       </c>
       <c r="E3" s="75" t="s">
         <v>296</v>
       </c>
-      <c r="F3" s="86" t="s">
+      <c r="F3" s="83" t="s">
         <v>297</v>
       </c>
       <c r="G3" s="75" t="s">
@@ -16048,13 +16066,13 @@
       <c r="I3" s="75" t="s">
         <v>509</v>
       </c>
-      <c r="J3" s="79">
+      <c r="J3" s="78">
         <v>3</v>
       </c>
       <c r="K3" s="75" t="s">
         <v>148</v>
       </c>
-      <c r="L3" s="108">
+      <c r="L3" s="105">
         <v>2</v>
       </c>
     </row>
@@ -16065,16 +16083,16 @@
       <c r="B4" s="75" t="s">
         <v>311</v>
       </c>
-      <c r="C4" s="78" t="s">
+      <c r="C4" s="77" t="s">
         <v>71</v>
       </c>
-      <c r="D4" s="106" t="s">
+      <c r="D4" s="103" t="s">
         <v>144</v>
       </c>
       <c r="E4" s="75" t="s">
         <v>296</v>
       </c>
-      <c r="F4" s="86" t="s">
+      <c r="F4" s="83" t="s">
         <v>297</v>
       </c>
       <c r="G4" s="75" t="s">
@@ -16086,13 +16104,13 @@
       <c r="I4" s="75" t="s">
         <v>510</v>
       </c>
-      <c r="J4" s="79">
+      <c r="J4" s="78">
         <v>4</v>
       </c>
       <c r="K4" s="75" t="s">
         <v>150</v>
       </c>
-      <c r="L4" s="109">
+      <c r="L4" s="106">
         <v>3</v>
       </c>
     </row>
@@ -16103,16 +16121,16 @@
       <c r="B5" s="75" t="s">
         <v>312</v>
       </c>
-      <c r="C5" s="79" t="s">
+      <c r="C5" s="78" t="s">
         <v>66</v>
       </c>
-      <c r="D5" s="106" t="s">
+      <c r="D5" s="103" t="s">
         <v>144</v>
       </c>
       <c r="E5" s="75" t="s">
         <v>301</v>
       </c>
-      <c r="F5" s="86" t="s">
+      <c r="F5" s="83" t="s">
         <v>302</v>
       </c>
       <c r="G5" s="75" t="s">
@@ -16124,13 +16142,13 @@
       <c r="I5" s="75" t="s">
         <v>543</v>
       </c>
-      <c r="J5" s="78">
+      <c r="J5" s="77">
         <v>3</v>
       </c>
       <c r="K5" s="75" t="s">
         <v>153</v>
       </c>
-      <c r="L5" s="108">
+      <c r="L5" s="105">
         <v>3</v>
       </c>
     </row>
@@ -16141,16 +16159,16 @@
       <c r="B6" s="75" t="s">
         <v>313</v>
       </c>
-      <c r="C6" s="79" t="s">
+      <c r="C6" s="78" t="s">
         <v>66</v>
       </c>
-      <c r="D6" s="106" t="s">
+      <c r="D6" s="103" t="s">
         <v>144</v>
       </c>
       <c r="E6" s="75" t="s">
         <v>305</v>
       </c>
-      <c r="F6" s="86" t="s">
+      <c r="F6" s="83" t="s">
         <v>306</v>
       </c>
       <c r="G6" s="75" t="s">
@@ -16162,13 +16180,13 @@
       <c r="I6" s="75" t="s">
         <v>511</v>
       </c>
-      <c r="J6" s="78">
+      <c r="J6" s="77">
         <v>3</v>
       </c>
       <c r="K6" s="75" t="s">
         <v>155</v>
       </c>
-      <c r="L6" s="110">
+      <c r="L6" s="107">
         <v>3</v>
       </c>
     </row>
@@ -16223,778 +16241,778 @@
   <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6" style="128" customWidth="1"/>
-    <col min="2" max="2" width="13" style="128" customWidth="1"/>
-    <col min="3" max="3" width="60" style="128" customWidth="1"/>
-    <col min="4" max="4" width="12" style="128" customWidth="1"/>
-    <col min="5" max="5" width="24" style="128" customWidth="1"/>
-    <col min="6" max="6" width="11" style="128" customWidth="1"/>
-    <col min="7" max="7" width="17.7109375" style="128" customWidth="1"/>
-    <col min="8" max="8" width="12" style="128" customWidth="1"/>
-    <col min="9" max="9" width="16" style="128" customWidth="1"/>
-    <col min="10" max="10" width="34" style="128" customWidth="1"/>
-    <col min="11" max="11" width="9" style="128" customWidth="1"/>
-    <col min="12" max="12" width="11" style="128" customWidth="1"/>
-    <col min="13" max="16384" width="8.85546875" style="128"/>
+    <col min="1" max="1" width="6" style="125" customWidth="1"/>
+    <col min="2" max="2" width="13" style="125" customWidth="1"/>
+    <col min="3" max="3" width="60" style="125" customWidth="1"/>
+    <col min="4" max="4" width="12" style="125" customWidth="1"/>
+    <col min="5" max="5" width="24" style="125" customWidth="1"/>
+    <col min="6" max="6" width="11" style="125" customWidth="1"/>
+    <col min="7" max="7" width="17.7109375" style="125" customWidth="1"/>
+    <col min="8" max="8" width="12" style="125" customWidth="1"/>
+    <col min="9" max="9" width="16" style="125" customWidth="1"/>
+    <col min="10" max="10" width="34" style="125" customWidth="1"/>
+    <col min="11" max="11" width="9" style="125" customWidth="1"/>
+    <col min="12" max="12" width="11" style="125" customWidth="1"/>
+    <col min="13" max="16384" width="8.85546875" style="125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="158" t="s">
+      <c r="A1" s="131" t="s">
         <v>314</v>
       </c>
-      <c r="B1" s="158" t="s">
+      <c r="B1" s="131" t="s">
         <v>315</v>
       </c>
-      <c r="C1" s="158" t="s">
+      <c r="C1" s="131" t="s">
         <v>316</v>
       </c>
-      <c r="D1" s="158" t="s">
+      <c r="D1" s="131" t="s">
         <v>317</v>
       </c>
-      <c r="E1" s="158" t="s">
+      <c r="E1" s="131" t="s">
         <v>318</v>
       </c>
-      <c r="F1" s="158" t="s">
+      <c r="F1" s="131" t="s">
         <v>319</v>
       </c>
-      <c r="G1" s="158" t="s">
+      <c r="G1" s="131" t="s">
         <v>320</v>
       </c>
-      <c r="H1" s="158" t="s">
+      <c r="H1" s="131" t="s">
         <v>321</v>
       </c>
-      <c r="I1" s="158" t="s">
+      <c r="I1" s="131" t="s">
         <v>322</v>
       </c>
-      <c r="J1" s="158" t="s">
+      <c r="J1" s="131" t="s">
         <v>323</v>
       </c>
-      <c r="K1" s="158" t="s">
+      <c r="K1" s="131" t="s">
         <v>110</v>
       </c>
-      <c r="L1" s="158" t="s">
+      <c r="L1" s="131" t="s">
         <v>324</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="159" t="s">
+      <c r="A2" s="132" t="s">
         <v>347</v>
       </c>
-      <c r="B2" s="159" t="s">
+      <c r="B2" s="132" t="s">
         <v>339</v>
       </c>
-      <c r="C2" s="159" t="s">
+      <c r="C2" s="132" t="s">
         <v>512</v>
       </c>
-      <c r="D2" s="159" t="s">
+      <c r="D2" s="132" t="s">
         <v>143</v>
       </c>
-      <c r="E2" s="159" t="s">
+      <c r="E2" s="132" t="s">
         <v>327</v>
       </c>
-      <c r="F2" s="159" t="s">
+      <c r="F2" s="132" t="s">
         <v>113</v>
       </c>
-      <c r="G2" s="159">
-        <v>3</v>
-      </c>
-      <c r="H2" s="159" t="s">
+      <c r="G2" s="132">
+        <v>3</v>
+      </c>
+      <c r="H2" s="132" t="s">
         <v>348</v>
       </c>
-      <c r="I2" s="159" t="s">
+      <c r="I2" s="132" t="s">
         <v>349</v>
       </c>
-      <c r="J2" s="159" t="s">
+      <c r="J2" s="132" t="s">
         <v>350</v>
       </c>
-      <c r="K2" s="159" t="s">
+      <c r="K2" s="132" t="s">
         <v>330</v>
       </c>
-      <c r="L2" s="159" t="s">
+      <c r="L2" s="132" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="159" t="s">
+      <c r="A3" s="132" t="s">
         <v>357</v>
       </c>
-      <c r="B3" s="159" t="s">
+      <c r="B3" s="132" t="s">
         <v>339</v>
       </c>
-      <c r="C3" s="159" t="s">
+      <c r="C3" s="132" t="s">
         <v>358</v>
       </c>
-      <c r="D3" s="159" t="s">
+      <c r="D3" s="132" t="s">
         <v>359</v>
       </c>
-      <c r="E3" s="159" t="s">
+      <c r="E3" s="132" t="s">
         <v>334</v>
       </c>
-      <c r="F3" s="159" t="s">
+      <c r="F3" s="132" t="s">
         <v>41</v>
       </c>
-      <c r="G3" s="159">
-        <v>3</v>
-      </c>
-      <c r="H3" s="159" t="s">
+      <c r="G3" s="132">
+        <v>3</v>
+      </c>
+      <c r="H3" s="132" t="s">
         <v>348</v>
       </c>
-      <c r="I3" s="159" t="s">
+      <c r="I3" s="132" t="s">
         <v>360</v>
       </c>
-      <c r="J3" s="159" t="s">
+      <c r="J3" s="132" t="s">
         <v>361</v>
       </c>
-      <c r="K3" s="159" t="s">
+      <c r="K3" s="132" t="s">
         <v>330</v>
       </c>
-      <c r="L3" s="159" t="s">
+      <c r="L3" s="132" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="159" t="s">
+      <c r="A4" s="132" t="s">
         <v>325</v>
       </c>
-      <c r="B4" s="159" t="s">
+      <c r="B4" s="132" t="s">
         <v>339</v>
       </c>
-      <c r="C4" s="159" t="s">
+      <c r="C4" s="132" t="s">
         <v>513</v>
       </c>
-      <c r="D4" s="159" t="s">
+      <c r="D4" s="132" t="s">
         <v>151</v>
       </c>
-      <c r="E4" s="159" t="s">
+      <c r="E4" s="132" t="s">
         <v>327</v>
       </c>
-      <c r="F4" s="159" t="s">
+      <c r="F4" s="132" t="s">
         <v>41</v>
       </c>
-      <c r="G4" s="159">
-        <v>1</v>
-      </c>
-      <c r="H4" s="159" t="s">
+      <c r="G4" s="132">
+        <v>1</v>
+      </c>
+      <c r="H4" s="132" t="s">
         <v>328</v>
       </c>
-      <c r="I4" s="159" t="s">
+      <c r="I4" s="132" t="s">
         <v>329</v>
       </c>
-      <c r="J4" s="159" t="s">
+      <c r="J4" s="132" t="s">
         <v>514</v>
       </c>
-      <c r="K4" s="159" t="s">
+      <c r="K4" s="132" t="s">
         <v>330</v>
       </c>
-      <c r="L4" s="159" t="s">
+      <c r="L4" s="132" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="159" t="s">
+      <c r="A5" s="132" t="s">
         <v>372</v>
       </c>
-      <c r="B5" s="159" t="s">
+      <c r="B5" s="132" t="s">
         <v>339</v>
       </c>
-      <c r="C5" s="159" t="s">
+      <c r="C5" s="132" t="s">
         <v>373</v>
       </c>
-      <c r="D5" s="159" t="s">
+      <c r="D5" s="132" t="s">
         <v>374</v>
       </c>
-      <c r="E5" s="159" t="s">
+      <c r="E5" s="132" t="s">
         <v>375</v>
       </c>
-      <c r="F5" s="159" t="s">
+      <c r="F5" s="132" t="s">
         <v>113</v>
       </c>
-      <c r="G5" s="159">
+      <c r="G5" s="132">
         <v>6</v>
       </c>
-      <c r="H5" s="159" t="s">
+      <c r="H5" s="132" t="s">
         <v>376</v>
       </c>
-      <c r="I5" s="159" t="s">
+      <c r="I5" s="132" t="s">
         <v>377</v>
       </c>
-      <c r="J5" s="159" t="s">
+      <c r="J5" s="132" t="s">
         <v>378</v>
       </c>
-      <c r="K5" s="159" t="s">
+      <c r="K5" s="132" t="s">
         <v>362</v>
       </c>
-      <c r="L5" s="159" t="s">
+      <c r="L5" s="132" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="159" t="s">
+      <c r="A6" s="132" t="s">
         <v>363</v>
       </c>
-      <c r="B6" s="159" t="s">
+      <c r="B6" s="132" t="s">
         <v>339</v>
       </c>
-      <c r="C6" s="159" t="s">
+      <c r="C6" s="132" t="s">
         <v>364</v>
       </c>
-      <c r="D6" s="159" t="s">
+      <c r="D6" s="132" t="s">
         <v>154</v>
       </c>
-      <c r="E6" s="159" t="s">
+      <c r="E6" s="132" t="s">
         <v>327</v>
       </c>
-      <c r="F6" s="159" t="s">
+      <c r="F6" s="132" t="s">
         <v>41</v>
       </c>
-      <c r="G6" s="159">
-        <v>3</v>
-      </c>
-      <c r="H6" s="159" t="s">
+      <c r="G6" s="132">
+        <v>3</v>
+      </c>
+      <c r="H6" s="132" t="s">
         <v>348</v>
       </c>
-      <c r="I6" s="159" t="s">
+      <c r="I6" s="132" t="s">
         <v>329</v>
       </c>
-      <c r="J6" s="159" t="s">
+      <c r="J6" s="132" t="s">
         <v>365</v>
       </c>
-      <c r="K6" s="159" t="s">
+      <c r="K6" s="132" t="s">
         <v>362</v>
       </c>
-      <c r="L6" s="159" t="s">
+      <c r="L6" s="132" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="159" t="s">
+      <c r="A7" s="132" t="s">
         <v>338</v>
       </c>
-      <c r="B7" s="159" t="s">
+      <c r="B7" s="132" t="s">
         <v>339</v>
       </c>
-      <c r="C7" s="159" t="s">
+      <c r="C7" s="132" t="s">
         <v>340</v>
       </c>
-      <c r="D7" s="159" t="s">
+      <c r="D7" s="132" t="s">
         <v>143</v>
       </c>
-      <c r="E7" s="159" t="s">
+      <c r="E7" s="132" t="s">
         <v>327</v>
       </c>
-      <c r="F7" s="159" t="s">
+      <c r="F7" s="132" t="s">
         <v>41</v>
       </c>
-      <c r="G7" s="159">
-        <v>2</v>
-      </c>
-      <c r="H7" s="159" t="s">
+      <c r="G7" s="132">
+        <v>2</v>
+      </c>
+      <c r="H7" s="132" t="s">
         <v>335</v>
       </c>
-      <c r="I7" s="159" t="s">
+      <c r="I7" s="132" t="s">
         <v>329</v>
       </c>
-      <c r="J7" s="159" t="s">
+      <c r="J7" s="132" t="s">
         <v>341</v>
       </c>
-      <c r="K7" s="159" t="s">
+      <c r="K7" s="132" t="s">
         <v>362</v>
       </c>
-      <c r="L7" s="159" t="s">
+      <c r="L7" s="132" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="159" t="s">
+      <c r="A8" s="132" t="s">
         <v>332</v>
       </c>
-      <c r="B8" s="159" t="s">
+      <c r="B8" s="132" t="s">
         <v>326</v>
       </c>
-      <c r="C8" s="159" t="s">
+      <c r="C8" s="132" t="s">
         <v>544</v>
       </c>
-      <c r="D8" s="159" t="s">
+      <c r="D8" s="132" t="s">
         <v>333</v>
       </c>
-      <c r="E8" s="159" t="s">
+      <c r="E8" s="132" t="s">
         <v>334</v>
       </c>
-      <c r="F8" s="159" t="s">
+      <c r="F8" s="132" t="s">
         <v>113</v>
       </c>
-      <c r="G8" s="159">
-        <v>2</v>
-      </c>
-      <c r="H8" s="159" t="s">
+      <c r="G8" s="132">
+        <v>2</v>
+      </c>
+      <c r="H8" s="132" t="s">
         <v>335</v>
       </c>
-      <c r="I8" s="159" t="s">
+      <c r="I8" s="132" t="s">
         <v>336</v>
       </c>
-      <c r="J8" s="159" t="s">
+      <c r="J8" s="132" t="s">
         <v>337</v>
       </c>
-      <c r="K8" s="159" t="s">
+      <c r="K8" s="132" t="s">
         <v>330</v>
       </c>
-      <c r="L8" s="159" t="s">
+      <c r="L8" s="132" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="159" t="s">
+      <c r="A9" s="132" t="s">
         <v>379</v>
       </c>
-      <c r="B9" s="159" t="s">
+      <c r="B9" s="132" t="s">
         <v>326</v>
       </c>
-      <c r="C9" s="159" t="s">
+      <c r="C9" s="132" t="s">
         <v>380</v>
       </c>
-      <c r="D9" s="159" t="s">
+      <c r="D9" s="132" t="s">
         <v>381</v>
       </c>
-      <c r="E9" s="159" t="s">
+      <c r="E9" s="132" t="s">
         <v>382</v>
       </c>
-      <c r="F9" s="159" t="s">
+      <c r="F9" s="132" t="s">
         <v>383</v>
       </c>
-      <c r="G9" s="159">
+      <c r="G9" s="132">
         <v>6</v>
       </c>
-      <c r="H9" s="159" t="s">
+      <c r="H9" s="132" t="s">
         <v>376</v>
       </c>
-      <c r="I9" s="159" t="s">
+      <c r="I9" s="132" t="s">
         <v>384</v>
       </c>
-      <c r="J9" s="159" t="s">
+      <c r="J9" s="132" t="s">
         <v>385</v>
       </c>
-      <c r="K9" s="159" t="s">
+      <c r="K9" s="132" t="s">
         <v>330</v>
       </c>
-      <c r="L9" s="159" t="s">
+      <c r="L9" s="132" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="159" t="s">
+      <c r="A10" s="132" t="s">
         <v>342</v>
       </c>
-      <c r="B10" s="159" t="s">
+      <c r="B10" s="132" t="s">
         <v>326</v>
       </c>
-      <c r="C10" s="159" t="s">
+      <c r="C10" s="132" t="s">
         <v>343</v>
       </c>
-      <c r="D10" s="159" t="s">
+      <c r="D10" s="132" t="s">
         <v>154</v>
       </c>
-      <c r="E10" s="159" t="s">
+      <c r="E10" s="132" t="s">
         <v>344</v>
       </c>
-      <c r="F10" s="159" t="s">
+      <c r="F10" s="132" t="s">
         <v>41</v>
       </c>
-      <c r="G10" s="159">
-        <v>2</v>
-      </c>
-      <c r="H10" s="159" t="s">
+      <c r="G10" s="132">
+        <v>2</v>
+      </c>
+      <c r="H10" s="132" t="s">
         <v>335</v>
       </c>
-      <c r="I10" s="159" t="s">
+      <c r="I10" s="132" t="s">
         <v>345</v>
       </c>
-      <c r="J10" s="159" t="s">
+      <c r="J10" s="132" t="s">
         <v>346</v>
       </c>
-      <c r="K10" s="159" t="s">
+      <c r="K10" s="132" t="s">
         <v>330</v>
       </c>
-      <c r="L10" s="159" t="s">
+      <c r="L10" s="132" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="159" t="s">
+      <c r="A11" s="132" t="s">
         <v>515</v>
       </c>
-      <c r="B11" s="159" t="s">
+      <c r="B11" s="132" t="s">
         <v>326</v>
       </c>
-      <c r="C11" s="159" t="s">
+      <c r="C11" s="132" t="s">
         <v>516</v>
       </c>
-      <c r="D11" s="159" t="s">
+      <c r="D11" s="132" t="s">
         <v>151</v>
       </c>
-      <c r="E11" s="159" t="s">
+      <c r="E11" s="132" t="s">
         <v>327</v>
       </c>
-      <c r="F11" s="159" t="s">
+      <c r="F11" s="132" t="s">
         <v>41</v>
       </c>
-      <c r="G11" s="159">
-        <v>1</v>
-      </c>
-      <c r="H11" s="159" t="s">
+      <c r="G11" s="132">
+        <v>1</v>
+      </c>
+      <c r="H11" s="132" t="s">
         <v>328</v>
       </c>
-      <c r="I11" s="159" t="s">
+      <c r="I11" s="132" t="s">
         <v>329</v>
       </c>
-      <c r="J11" s="159" t="s">
+      <c r="J11" s="132" t="s">
         <v>517</v>
       </c>
-      <c r="K11" s="159" t="s">
+      <c r="K11" s="132" t="s">
         <v>330</v>
       </c>
-      <c r="L11" s="159" t="s">
+      <c r="L11" s="132" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="159" t="s">
+      <c r="A12" s="132" t="s">
         <v>396</v>
       </c>
-      <c r="B12" s="159" t="s">
+      <c r="B12" s="132" t="s">
         <v>326</v>
       </c>
-      <c r="C12" s="159" t="s">
+      <c r="C12" s="132" t="s">
         <v>397</v>
       </c>
-      <c r="D12" s="159" t="s">
+      <c r="D12" s="132" t="s">
         <v>147</v>
       </c>
-      <c r="E12" s="159" t="s">
+      <c r="E12" s="132" t="s">
         <v>334</v>
       </c>
-      <c r="F12" s="159" t="s">
+      <c r="F12" s="132" t="s">
         <v>41</v>
       </c>
-      <c r="G12" s="159">
+      <c r="G12" s="132">
         <v>7</v>
       </c>
-      <c r="H12" s="159" t="s">
+      <c r="H12" s="132" t="s">
         <v>398</v>
       </c>
-      <c r="I12" s="159" t="s">
+      <c r="I12" s="132" t="s">
         <v>329</v>
       </c>
-      <c r="J12" s="159" t="s">
+      <c r="J12" s="132" t="s">
         <v>399</v>
       </c>
-      <c r="K12" s="159" t="s">
+      <c r="K12" s="132" t="s">
         <v>362</v>
       </c>
-      <c r="L12" s="159" t="s">
+      <c r="L12" s="132" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="159" t="s">
+      <c r="A13" s="132" t="s">
         <v>400</v>
       </c>
-      <c r="B13" s="159" t="s">
+      <c r="B13" s="132" t="s">
         <v>326</v>
       </c>
-      <c r="C13" s="159" t="s">
+      <c r="C13" s="132" t="s">
         <v>401</v>
       </c>
-      <c r="D13" s="159" t="s">
+      <c r="D13" s="132" t="s">
         <v>402</v>
       </c>
-      <c r="E13" s="159" t="s">
+      <c r="E13" s="132" t="s">
         <v>403</v>
       </c>
-      <c r="F13" s="159" t="s">
+      <c r="F13" s="132" t="s">
         <v>383</v>
       </c>
-      <c r="G13" s="159">
+      <c r="G13" s="132">
         <v>9</v>
       </c>
-      <c r="H13" s="159" t="s">
+      <c r="H13" s="132" t="s">
         <v>404</v>
       </c>
-      <c r="I13" s="159" t="s">
+      <c r="I13" s="132" t="s">
         <v>405</v>
       </c>
-      <c r="J13" s="159" t="s">
+      <c r="J13" s="132" t="s">
         <v>406</v>
       </c>
-      <c r="K13" s="159" t="s">
+      <c r="K13" s="132" t="s">
         <v>362</v>
       </c>
-      <c r="L13" s="159" t="s">
+      <c r="L13" s="132" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="159" t="s">
+      <c r="A14" s="132" t="s">
         <v>518</v>
       </c>
-      <c r="B14" s="159" t="s">
+      <c r="B14" s="132" t="s">
         <v>326</v>
       </c>
-      <c r="C14" s="159" t="s">
+      <c r="C14" s="132" t="s">
         <v>519</v>
       </c>
-      <c r="D14" s="159" t="s">
+      <c r="D14" s="132" t="s">
         <v>149</v>
       </c>
-      <c r="E14" s="159" t="s">
+      <c r="E14" s="132" t="s">
         <v>334</v>
       </c>
-      <c r="F14" s="159" t="s">
+      <c r="F14" s="132" t="s">
         <v>41</v>
       </c>
-      <c r="G14" s="159">
-        <v>2</v>
-      </c>
-      <c r="H14" s="159" t="s">
+      <c r="G14" s="132">
+        <v>2</v>
+      </c>
+      <c r="H14" s="132" t="s">
         <v>335</v>
       </c>
-      <c r="I14" s="159" t="s">
+      <c r="I14" s="132" t="s">
         <v>329</v>
       </c>
-      <c r="J14" s="159" t="s">
+      <c r="J14" s="132" t="s">
         <v>520</v>
       </c>
-      <c r="K14" s="159" t="s">
+      <c r="K14" s="132" t="s">
         <v>362</v>
       </c>
-      <c r="L14" s="159" t="s">
+      <c r="L14" s="132" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="159" t="s">
+      <c r="A15" s="132" t="s">
         <v>366</v>
       </c>
-      <c r="B15" s="159" t="s">
+      <c r="B15" s="132" t="s">
         <v>367</v>
       </c>
-      <c r="C15" s="159" t="s">
+      <c r="C15" s="132" t="s">
         <v>368</v>
       </c>
-      <c r="D15" s="159" t="s">
+      <c r="D15" s="132" t="s">
         <v>149</v>
       </c>
-      <c r="E15" s="159" t="s">
+      <c r="E15" s="132" t="s">
         <v>334</v>
       </c>
-      <c r="F15" s="159" t="s">
+      <c r="F15" s="132" t="s">
         <v>113</v>
       </c>
-      <c r="G15" s="159">
-        <v>4</v>
-      </c>
-      <c r="H15" s="159" t="s">
+      <c r="G15" s="132">
+        <v>4</v>
+      </c>
+      <c r="H15" s="132" t="s">
         <v>369</v>
       </c>
-      <c r="I15" s="159" t="s">
+      <c r="I15" s="132" t="s">
         <v>370</v>
       </c>
-      <c r="J15" s="159" t="s">
+      <c r="J15" s="132" t="s">
         <v>371</v>
       </c>
-      <c r="K15" s="159" t="s">
+      <c r="K15" s="132" t="s">
         <v>330</v>
       </c>
-      <c r="L15" s="159" t="s">
+      <c r="L15" s="132" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="159" t="s">
+      <c r="A16" s="132" t="s">
         <v>407</v>
       </c>
-      <c r="B16" s="159" t="s">
+      <c r="B16" s="132" t="s">
         <v>367</v>
       </c>
-      <c r="C16" s="159" t="s">
+      <c r="C16" s="132" t="s">
         <v>408</v>
       </c>
-      <c r="D16" s="159" t="s">
+      <c r="D16" s="132" t="s">
         <v>402</v>
       </c>
-      <c r="E16" s="159" t="s">
+      <c r="E16" s="132" t="s">
         <v>334</v>
       </c>
-      <c r="F16" s="159" t="s">
+      <c r="F16" s="132" t="s">
         <v>383</v>
       </c>
-      <c r="G16" s="159">
+      <c r="G16" s="132">
         <v>9</v>
       </c>
-      <c r="H16" s="159" t="s">
+      <c r="H16" s="132" t="s">
         <v>404</v>
       </c>
-      <c r="I16" s="159" t="s">
+      <c r="I16" s="132" t="s">
         <v>409</v>
       </c>
-      <c r="J16" s="159" t="s">
+      <c r="J16" s="132" t="s">
         <v>410</v>
       </c>
-      <c r="K16" s="159" t="s">
+      <c r="K16" s="132" t="s">
         <v>362</v>
       </c>
-      <c r="L16" s="159" t="s">
+      <c r="L16" s="132" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="159" t="s">
+      <c r="A17" s="132" t="s">
         <v>386</v>
       </c>
-      <c r="B17" s="159" t="s">
+      <c r="B17" s="132" t="s">
         <v>367</v>
       </c>
-      <c r="C17" s="159" t="s">
+      <c r="C17" s="132" t="s">
         <v>387</v>
       </c>
-      <c r="D17" s="159" t="s">
+      <c r="D17" s="132" t="s">
         <v>154</v>
       </c>
-      <c r="E17" s="159" t="s">
+      <c r="E17" s="132" t="s">
         <v>334</v>
       </c>
-      <c r="F17" s="159" t="s">
+      <c r="F17" s="132" t="s">
         <v>113</v>
       </c>
-      <c r="G17" s="159">
+      <c r="G17" s="132">
         <v>6</v>
       </c>
-      <c r="H17" s="159" t="s">
+      <c r="H17" s="132" t="s">
         <v>376</v>
       </c>
-      <c r="I17" s="159" t="s">
+      <c r="I17" s="132" t="s">
         <v>388</v>
       </c>
-      <c r="J17" s="159" t="s">
+      <c r="J17" s="132" t="s">
         <v>389</v>
       </c>
-      <c r="K17" s="159" t="s">
+      <c r="K17" s="132" t="s">
         <v>390</v>
       </c>
-      <c r="L17" s="159" t="s">
+      <c r="L17" s="132" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="18" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="159" t="s">
+      <c r="A18" s="132" t="s">
         <v>351</v>
       </c>
-      <c r="B18" s="159" t="s">
+      <c r="B18" s="132" t="s">
         <v>352</v>
       </c>
-      <c r="C18" s="159" t="s">
+      <c r="C18" s="132" t="s">
         <v>353</v>
       </c>
-      <c r="D18" s="159" t="s">
+      <c r="D18" s="132" t="s">
         <v>354</v>
       </c>
-      <c r="E18" s="159" t="s">
+      <c r="E18" s="132" t="s">
         <v>334</v>
       </c>
-      <c r="F18" s="159" t="s">
+      <c r="F18" s="132" t="s">
         <v>113</v>
       </c>
-      <c r="G18" s="159">
-        <v>3</v>
-      </c>
-      <c r="H18" s="159" t="s">
+      <c r="G18" s="132">
+        <v>3</v>
+      </c>
+      <c r="H18" s="132" t="s">
         <v>348</v>
       </c>
-      <c r="I18" s="159" t="s">
+      <c r="I18" s="132" t="s">
         <v>355</v>
       </c>
-      <c r="J18" s="159" t="s">
+      <c r="J18" s="132" t="s">
         <v>356</v>
       </c>
-      <c r="K18" s="159" t="s">
+      <c r="K18" s="132" t="s">
         <v>330</v>
       </c>
-      <c r="L18" s="159" t="s">
+      <c r="L18" s="132" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="19" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="159" t="s">
+      <c r="A19" s="132" t="s">
         <v>411</v>
       </c>
-      <c r="B19" s="159" t="s">
+      <c r="B19" s="132" t="s">
         <v>352</v>
       </c>
-      <c r="C19" s="159" t="s">
+      <c r="C19" s="132" t="s">
         <v>412</v>
       </c>
-      <c r="D19" s="159" t="s">
+      <c r="D19" s="132" t="s">
         <v>354</v>
       </c>
-      <c r="E19" s="159" t="s">
+      <c r="E19" s="132" t="s">
         <v>375</v>
       </c>
-      <c r="F19" s="159" t="s">
+      <c r="F19" s="132" t="s">
         <v>383</v>
       </c>
-      <c r="G19" s="159">
+      <c r="G19" s="132">
         <v>12</v>
       </c>
-      <c r="H19" s="159" t="s">
+      <c r="H19" s="132" t="s">
         <v>413</v>
       </c>
-      <c r="I19" s="159" t="s">
+      <c r="I19" s="132" t="s">
         <v>414</v>
       </c>
-      <c r="J19" s="159" t="s">
+      <c r="J19" s="132" t="s">
         <v>415</v>
       </c>
-      <c r="K19" s="159" t="s">
+      <c r="K19" s="132" t="s">
         <v>362</v>
       </c>
-      <c r="L19" s="159" t="s">
+      <c r="L19" s="132" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="159" t="s">
+      <c r="A20" s="132" t="s">
         <v>391</v>
       </c>
-      <c r="B20" s="159" t="s">
+      <c r="B20" s="132" t="s">
         <v>352</v>
       </c>
-      <c r="C20" s="159" t="s">
+      <c r="C20" s="132" t="s">
         <v>392</v>
       </c>
-      <c r="D20" s="159" t="s">
+      <c r="D20" s="132" t="s">
         <v>393</v>
       </c>
-      <c r="E20" s="159" t="s">
+      <c r="E20" s="132" t="s">
         <v>327</v>
       </c>
-      <c r="F20" s="159" t="s">
+      <c r="F20" s="132" t="s">
         <v>41</v>
       </c>
-      <c r="G20" s="159">
+      <c r="G20" s="132">
         <v>6</v>
       </c>
-      <c r="H20" s="159" t="s">
+      <c r="H20" s="132" t="s">
         <v>376</v>
       </c>
-      <c r="I20" s="159" t="s">
+      <c r="I20" s="132" t="s">
         <v>394</v>
       </c>
-      <c r="J20" s="159" t="s">
+      <c r="J20" s="132" t="s">
         <v>395</v>
       </c>
-      <c r="K20" s="159" t="s">
+      <c r="K20" s="132" t="s">
         <v>390</v>
       </c>
-      <c r="L20" s="159" t="s">
+      <c r="L20" s="132" t="s">
         <v>331</v>
       </c>
     </row>
@@ -17008,199 +17026,199 @@
   <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8" style="128" customWidth="1"/>
-    <col min="2" max="2" width="10" style="128" customWidth="1"/>
-    <col min="3" max="3" width="13" style="128" customWidth="1"/>
-    <col min="4" max="4" width="12" style="128" customWidth="1"/>
-    <col min="5" max="5" width="34" style="128" customWidth="1"/>
-    <col min="6" max="6" width="11" style="128" customWidth="1"/>
-    <col min="7" max="7" width="14" style="128" customWidth="1"/>
-    <col min="8" max="8" width="13" style="128" customWidth="1"/>
-    <col min="9" max="9" width="40" style="128" customWidth="1"/>
-    <col min="10" max="16384" width="8.85546875" style="128"/>
+    <col min="1" max="1" width="8" style="125" customWidth="1"/>
+    <col min="2" max="2" width="10" style="125" customWidth="1"/>
+    <col min="3" max="3" width="13" style="125" customWidth="1"/>
+    <col min="4" max="4" width="12" style="125" customWidth="1"/>
+    <col min="5" max="5" width="34" style="125" customWidth="1"/>
+    <col min="6" max="6" width="11" style="125" customWidth="1"/>
+    <col min="7" max="7" width="14" style="125" customWidth="1"/>
+    <col min="8" max="8" width="13" style="125" customWidth="1"/>
+    <col min="9" max="9" width="40" style="125" customWidth="1"/>
+    <col min="10" max="16384" width="8.85546875" style="125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="124" t="s">
         <v>135</v>
       </c>
-      <c r="B1" s="127" t="s">
+      <c r="B1" s="124" t="s">
         <v>416</v>
       </c>
-      <c r="C1" s="127" t="s">
+      <c r="C1" s="124" t="s">
         <v>417</v>
       </c>
-      <c r="D1" s="127" t="s">
+      <c r="D1" s="124" t="s">
         <v>418</v>
       </c>
-      <c r="E1" s="127" t="s">
+      <c r="E1" s="124" t="s">
         <v>419</v>
       </c>
-      <c r="F1" s="127" t="s">
+      <c r="F1" s="124" t="s">
         <v>420</v>
       </c>
-      <c r="G1" s="127" t="s">
+      <c r="G1" s="124" t="s">
         <v>421</v>
       </c>
-      <c r="H1" s="127" t="s">
+      <c r="H1" s="124" t="s">
         <v>422</v>
       </c>
-      <c r="I1" s="127" t="s">
+      <c r="I1" s="124" t="s">
         <v>423</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="129" t="s">
+      <c r="A2" s="126" t="s">
         <v>143</v>
       </c>
-      <c r="B2" s="129" t="s">
+      <c r="B2" s="126" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="129" t="s">
+      <c r="C2" s="126" t="s">
         <v>424</v>
       </c>
-      <c r="D2" s="131" t="s">
+      <c r="D2" s="128" t="s">
         <v>71</v>
       </c>
-      <c r="E2" s="130" t="s">
+      <c r="E2" s="127" t="s">
         <v>425</v>
       </c>
-      <c r="F2" s="129" t="s">
+      <c r="F2" s="126" t="s">
         <v>38</v>
       </c>
-      <c r="G2" s="129" t="s">
+      <c r="G2" s="126" t="s">
         <v>426</v>
       </c>
-      <c r="H2" s="132" t="s">
+      <c r="H2" s="129" t="s">
         <v>66</v>
       </c>
-      <c r="I2" s="130" t="s">
+      <c r="I2" s="127" t="s">
         <v>545</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="129" t="s">
+      <c r="A3" s="126" t="s">
         <v>147</v>
       </c>
-      <c r="B3" s="129" t="s">
+      <c r="B3" s="126" t="s">
         <v>38</v>
       </c>
-      <c r="C3" s="129" t="s">
+      <c r="C3" s="126" t="s">
         <v>426</v>
       </c>
-      <c r="D3" s="132" t="s">
+      <c r="D3" s="129" t="s">
         <v>66</v>
       </c>
-      <c r="E3" s="130" t="s">
+      <c r="E3" s="127" t="s">
         <v>427</v>
       </c>
-      <c r="F3" s="129" t="s">
+      <c r="F3" s="126" t="s">
         <v>38</v>
       </c>
-      <c r="G3" s="129" t="s">
+      <c r="G3" s="126" t="s">
         <v>428</v>
       </c>
-      <c r="H3" s="133" t="s">
+      <c r="H3" s="130" t="s">
         <v>53</v>
       </c>
-      <c r="I3" s="130" t="s">
+      <c r="I3" s="127" t="s">
         <v>546</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="129" t="s">
+      <c r="A4" s="126" t="s">
         <v>149</v>
       </c>
-      <c r="B4" s="129" t="s">
+      <c r="B4" s="126" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="129" t="s">
+      <c r="C4" s="126" t="s">
         <v>424</v>
       </c>
-      <c r="D4" s="131" t="s">
+      <c r="D4" s="128" t="s">
         <v>71</v>
       </c>
-      <c r="E4" s="130" t="s">
+      <c r="E4" s="127" t="s">
         <v>521</v>
       </c>
-      <c r="F4" s="129" t="s">
+      <c r="F4" s="126" t="s">
         <v>38</v>
       </c>
-      <c r="G4" s="129" t="s">
+      <c r="G4" s="126" t="s">
         <v>426</v>
       </c>
-      <c r="H4" s="132" t="s">
+      <c r="H4" s="129" t="s">
         <v>66</v>
       </c>
-      <c r="I4" s="130" t="s">
+      <c r="I4" s="127" t="s">
         <v>545</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="129" t="s">
+      <c r="A5" s="126" t="s">
         <v>151</v>
       </c>
-      <c r="B5" s="129" t="s">
+      <c r="B5" s="126" t="s">
         <v>38</v>
       </c>
-      <c r="C5" s="129" t="s">
+      <c r="C5" s="126" t="s">
         <v>424</v>
       </c>
-      <c r="D5" s="132" t="s">
+      <c r="D5" s="129" t="s">
         <v>66</v>
       </c>
-      <c r="E5" s="130" t="s">
+      <c r="E5" s="127" t="s">
         <v>522</v>
       </c>
-      <c r="F5" s="129" t="s">
+      <c r="F5" s="126" t="s">
         <v>38</v>
       </c>
-      <c r="G5" s="129" t="s">
+      <c r="G5" s="126" t="s">
         <v>426</v>
       </c>
-      <c r="H5" s="132" t="s">
+      <c r="H5" s="129" t="s">
         <v>66</v>
       </c>
-      <c r="I5" s="130" t="s">
+      <c r="I5" s="127" t="s">
         <v>545</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="129" t="s">
+      <c r="A6" s="126" t="s">
         <v>154</v>
       </c>
-      <c r="B6" s="129" t="s">
+      <c r="B6" s="126" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="129" t="s">
+      <c r="C6" s="126" t="s">
         <v>424</v>
       </c>
-      <c r="D6" s="132" t="s">
+      <c r="D6" s="129" t="s">
         <v>66</v>
       </c>
-      <c r="E6" s="130" t="s">
+      <c r="E6" s="127" t="s">
         <v>429</v>
       </c>
-      <c r="F6" s="129" t="s">
+      <c r="F6" s="126" t="s">
         <v>38</v>
       </c>
-      <c r="G6" s="129" t="s">
+      <c r="G6" s="126" t="s">
         <v>426</v>
       </c>
-      <c r="H6" s="132" t="s">
+      <c r="H6" s="129" t="s">
         <v>66</v>
       </c>
-      <c r="I6" s="130" t="s">
+      <c r="I6" s="127" t="s">
         <v>545</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="128" t="s">
+      <c r="A8" s="125" t="s">
         <v>523</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="128" t="s">
+      <c r="A9" s="125" t="s">
         <v>524</v>
       </c>
     </row>
@@ -17214,189 +17232,189 @@
   <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="55" style="124" customWidth="1"/>
-    <col min="2" max="2" width="12" style="124" customWidth="1"/>
-    <col min="3" max="3" width="20" style="124" customWidth="1"/>
-    <col min="4" max="4" width="14" style="124" customWidth="1"/>
-    <col min="5" max="5" width="24" style="124" customWidth="1"/>
-    <col min="6" max="16384" width="8.85546875" style="124"/>
+    <col min="1" max="1" width="55" style="121" customWidth="1"/>
+    <col min="2" max="2" width="12" style="121" customWidth="1"/>
+    <col min="3" max="3" width="20" style="121" customWidth="1"/>
+    <col min="4" max="4" width="14" style="121" customWidth="1"/>
+    <col min="5" max="5" width="24" style="121" customWidth="1"/>
+    <col min="6" max="16384" width="8.85546875" style="121"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="123" t="s">
+      <c r="A1" s="120" t="s">
         <v>430</v>
       </c>
-      <c r="B1" s="123" t="s">
+      <c r="B1" s="120" t="s">
         <v>431</v>
       </c>
-      <c r="C1" s="123" t="s">
+      <c r="C1" s="120" t="s">
         <v>432</v>
       </c>
-      <c r="D1" s="123" t="s">
+      <c r="D1" s="120" t="s">
         <v>433</v>
       </c>
-      <c r="E1" s="123" t="s">
+      <c r="E1" s="120" t="s">
         <v>434</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="125" t="s">
+      <c r="A2" s="122" t="s">
         <v>435</v>
       </c>
-      <c r="B2" s="125" t="s">
+      <c r="B2" s="122" t="s">
         <v>332</v>
       </c>
-      <c r="C2" s="125" t="s">
+      <c r="C2" s="122" t="s">
         <v>436</v>
       </c>
-      <c r="D2" s="125" t="s">
+      <c r="D2" s="122" t="s">
         <v>437</v>
       </c>
-      <c r="E2" s="125" t="s">
+      <c r="E2" s="122" t="s">
         <v>438</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="125" t="s">
+      <c r="A3" s="122" t="s">
         <v>439</v>
       </c>
-      <c r="B3" s="125" t="s">
+      <c r="B3" s="122" t="s">
         <v>351</v>
       </c>
-      <c r="C3" s="125" t="s">
+      <c r="C3" s="122" t="s">
         <v>440</v>
       </c>
-      <c r="D3" s="125" t="s">
+      <c r="D3" s="122" t="s">
         <v>441</v>
       </c>
-      <c r="E3" s="125" t="s">
+      <c r="E3" s="122" t="s">
         <v>438</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="125" t="s">
+      <c r="A4" s="122" t="s">
         <v>442</v>
       </c>
-      <c r="B4" s="125" t="s">
+      <c r="B4" s="122" t="s">
         <v>357</v>
       </c>
-      <c r="C4" s="125" t="s">
+      <c r="C4" s="122" t="s">
         <v>443</v>
       </c>
-      <c r="D4" s="125" t="s">
+      <c r="D4" s="122" t="s">
         <v>444</v>
       </c>
-      <c r="E4" s="125" t="s">
+      <c r="E4" s="122" t="s">
         <v>438</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="125" t="s">
+      <c r="A5" s="122" t="s">
         <v>445</v>
       </c>
-      <c r="B5" s="125" t="s">
+      <c r="B5" s="122" t="s">
         <v>379</v>
       </c>
-      <c r="C5" s="125" t="s">
+      <c r="C5" s="122" t="s">
         <v>446</v>
       </c>
-      <c r="D5" s="125" t="s">
+      <c r="D5" s="122" t="s">
         <v>437</v>
       </c>
-      <c r="E5" s="125" t="s">
+      <c r="E5" s="122" t="s">
         <v>447</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="125" t="s">
+      <c r="A6" s="122" t="s">
         <v>448</v>
       </c>
-      <c r="B6" s="125" t="s">
+      <c r="B6" s="122" t="s">
         <v>449</v>
       </c>
-      <c r="C6" s="125" t="s">
+      <c r="C6" s="122" t="s">
         <v>450</v>
       </c>
-      <c r="D6" s="125" t="s">
+      <c r="D6" s="122" t="s">
         <v>441</v>
       </c>
-      <c r="E6" s="125" t="s">
+      <c r="E6" s="122" t="s">
         <v>451</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="125" t="s">
+      <c r="A7" s="122" t="s">
         <v>525</v>
       </c>
-      <c r="B7" s="125" t="s">
+      <c r="B7" s="122" t="s">
         <v>515</v>
       </c>
-      <c r="C7" s="125" t="s">
+      <c r="C7" s="122" t="s">
         <v>436</v>
       </c>
-      <c r="D7" s="125" t="s">
+      <c r="D7" s="122" t="s">
         <v>437</v>
       </c>
-      <c r="E7" s="125" t="s">
+      <c r="E7" s="122" t="s">
         <v>452</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="125" t="s">
+      <c r="A8" s="122" t="s">
         <v>526</v>
       </c>
-      <c r="B8" s="125" t="s">
+      <c r="B8" s="122" t="s">
         <v>325</v>
       </c>
-      <c r="C8" s="125" t="s">
+      <c r="C8" s="122" t="s">
         <v>436</v>
       </c>
-      <c r="D8" s="125" t="s">
+      <c r="D8" s="122" t="s">
         <v>527</v>
       </c>
-      <c r="E8" s="125" t="s">
+      <c r="E8" s="122" t="s">
         <v>452</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="125" t="s">
+      <c r="A9" s="122" t="s">
         <v>528</v>
       </c>
-      <c r="B9" s="125" t="s">
+      <c r="B9" s="122" t="s">
         <v>518</v>
       </c>
-      <c r="C9" s="125" t="s">
+      <c r="C9" s="122" t="s">
         <v>529</v>
       </c>
-      <c r="D9" s="125" t="s">
+      <c r="D9" s="122" t="s">
         <v>437</v>
       </c>
-      <c r="E9" s="125" t="s">
+      <c r="E9" s="122" t="s">
         <v>438</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="126" t="s">
+      <c r="A11" s="123" t="s">
         <v>453</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="124" t="s">
+      <c r="A12" s="121" t="s">
         <v>454</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="124" t="s">
+      <c r="A13" s="121" t="s">
         <v>455</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="124" t="s">
+      <c r="A14" s="121" t="s">
         <v>456</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="124" t="s">
+      <c r="A15" s="121" t="s">
         <v>457</v>
       </c>
     </row>
@@ -17439,9 +17457,9 @@
       <c r="H1" t="s">
         <v>129</v>
       </c>
-      <c r="J1" s="111"/>
-      <c r="K1" s="111"/>
-      <c r="L1" s="112"/>
+      <c r="J1" s="108"/>
+      <c r="K1" s="108"/>
+      <c r="L1" s="109"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2">
@@ -17476,7 +17494,7 @@
         <f>'Atelier 3 - Carto PP'!J40</f>
         <v>4</v>
       </c>
-      <c r="L2" s="113"/>
+      <c r="L2" s="110"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3">
@@ -29690,34 +29708,34 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A2" s="134" t="s">
+      <c r="A2" s="156" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="134"/>
-      <c r="C2" s="134"/>
-      <c r="D2" s="134"/>
-      <c r="E2" s="134"/>
-      <c r="G2" s="135" t="s">
+      <c r="B2" s="156"/>
+      <c r="C2" s="156"/>
+      <c r="D2" s="156"/>
+      <c r="E2" s="156"/>
+      <c r="G2" s="157" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="135"/>
-      <c r="J2" s="136" t="s">
+      <c r="H2" s="157"/>
+      <c r="J2" s="158" t="s">
         <v>15</v>
       </c>
-      <c r="K2" s="136"/>
-      <c r="L2" s="136"/>
-      <c r="M2" s="136"/>
-      <c r="N2" s="136"/>
-      <c r="O2" s="136"/>
-      <c r="P2" s="136"/>
-      <c r="Q2" s="136"/>
-      <c r="Z2" s="134" t="s">
+      <c r="K2" s="158"/>
+      <c r="L2" s="158"/>
+      <c r="M2" s="158"/>
+      <c r="N2" s="158"/>
+      <c r="O2" s="158"/>
+      <c r="P2" s="158"/>
+      <c r="Q2" s="158"/>
+      <c r="Z2" s="156" t="s">
         <v>16</v>
       </c>
-      <c r="AA2" s="134"/>
-      <c r="AB2" s="134"/>
-      <c r="AC2" s="134"/>
-      <c r="AD2" s="134"/>
+      <c r="AA2" s="156"/>
+      <c r="AB2" s="156"/>
+      <c r="AC2" s="156"/>
+      <c r="AD2" s="156"/>
     </row>
     <row r="3" spans="1:38" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
@@ -29735,7 +29753,7 @@
       <c r="E3" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="F3" s="137" t="s">
+      <c r="F3" s="144" t="s">
         <v>13</v>
       </c>
       <c r="G3" s="15" t="s">
@@ -29744,32 +29762,32 @@
       <c r="H3" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="I3" s="137" t="s">
+      <c r="I3" s="144" t="s">
         <v>14</v>
       </c>
       <c r="J3" s="17">
         <v>1</v>
       </c>
-      <c r="K3" s="138" t="s">
+      <c r="K3" s="146" t="s">
         <v>24</v>
       </c>
-      <c r="L3" s="138"/>
-      <c r="M3" s="138"/>
-      <c r="N3" s="138"/>
-      <c r="O3" s="138"/>
-      <c r="P3" s="138"/>
-      <c r="Q3" s="138"/>
-      <c r="R3" s="137" t="s">
+      <c r="L3" s="146"/>
+      <c r="M3" s="146"/>
+      <c r="N3" s="146"/>
+      <c r="O3" s="146"/>
+      <c r="P3" s="146"/>
+      <c r="Q3" s="146"/>
+      <c r="R3" s="144" t="s">
         <v>15</v>
       </c>
       <c r="T3" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="U3" s="139" t="s">
+      <c r="U3" s="159" t="s">
         <v>25</v>
       </c>
-      <c r="V3" s="139"/>
-      <c r="Y3" s="137" t="s">
+      <c r="V3" s="159"/>
+      <c r="Y3" s="144" t="s">
         <v>26</v>
       </c>
       <c r="Z3" s="19" t="s">
@@ -29787,17 +29805,17 @@
       <c r="AD3" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="AE3" s="137" t="s">
+      <c r="AE3" s="144" t="s">
         <v>31</v>
       </c>
       <c r="AG3" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="AH3" s="141" t="s">
+      <c r="AH3" s="145" t="s">
         <v>32</v>
       </c>
-      <c r="AI3" s="141"/>
-      <c r="AL3" s="137" t="s">
+      <c r="AI3" s="145"/>
+      <c r="AL3" s="144" t="s">
         <v>33</v>
       </c>
     </row>
@@ -29817,35 +29835,35 @@
       <c r="E4" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="F4" s="137"/>
+      <c r="F4" s="144"/>
       <c r="G4" s="26" t="s">
         <v>38</v>
       </c>
       <c r="H4" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="I4" s="137"/>
+      <c r="I4" s="144"/>
       <c r="J4" s="27">
         <v>2</v>
       </c>
-      <c r="K4" s="138" t="s">
+      <c r="K4" s="146" t="s">
         <v>40</v>
       </c>
-      <c r="L4" s="138"/>
-      <c r="M4" s="138"/>
-      <c r="N4" s="138"/>
-      <c r="O4" s="138"/>
-      <c r="P4" s="138"/>
-      <c r="Q4" s="138"/>
-      <c r="R4" s="137"/>
+      <c r="L4" s="146"/>
+      <c r="M4" s="146"/>
+      <c r="N4" s="146"/>
+      <c r="O4" s="146"/>
+      <c r="P4" s="146"/>
+      <c r="Q4" s="146"/>
+      <c r="R4" s="144"/>
       <c r="T4" s="28">
         <v>1</v>
       </c>
-      <c r="U4" s="142" t="s">
+      <c r="U4" s="147" t="s">
         <v>41</v>
       </c>
-      <c r="V4" s="142"/>
-      <c r="Y4" s="137"/>
+      <c r="V4" s="147"/>
+      <c r="Y4" s="144"/>
       <c r="Z4" s="29">
         <v>1</v>
       </c>
@@ -29861,15 +29879,15 @@
       <c r="AD4" s="31" t="s">
         <v>45</v>
       </c>
-      <c r="AE4" s="137"/>
+      <c r="AE4" s="144"/>
       <c r="AG4" s="32">
         <v>1</v>
       </c>
-      <c r="AH4" s="143" t="s">
+      <c r="AH4" s="148" t="s">
         <v>41</v>
       </c>
-      <c r="AI4" s="143"/>
-      <c r="AL4" s="137"/>
+      <c r="AI4" s="148"/>
+      <c r="AL4" s="144"/>
     </row>
     <row r="5" spans="1:38" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="33">
@@ -29887,35 +29905,35 @@
       <c r="E5" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="F5" s="137"/>
+      <c r="F5" s="144"/>
       <c r="G5" s="34" t="s">
         <v>50</v>
       </c>
       <c r="H5" s="35" t="s">
         <v>51</v>
       </c>
-      <c r="I5" s="137"/>
+      <c r="I5" s="144"/>
       <c r="J5" s="36">
         <v>3</v>
       </c>
-      <c r="K5" s="138" t="s">
+      <c r="K5" s="146" t="s">
         <v>52</v>
       </c>
-      <c r="L5" s="138"/>
-      <c r="M5" s="138"/>
-      <c r="N5" s="138"/>
-      <c r="O5" s="138"/>
-      <c r="P5" s="138"/>
-      <c r="Q5" s="138"/>
-      <c r="R5" s="137"/>
+      <c r="L5" s="146"/>
+      <c r="M5" s="146"/>
+      <c r="N5" s="146"/>
+      <c r="O5" s="146"/>
+      <c r="P5" s="146"/>
+      <c r="Q5" s="146"/>
+      <c r="R5" s="144"/>
       <c r="T5" s="37">
         <v>2</v>
       </c>
-      <c r="U5" s="144" t="s">
+      <c r="U5" s="149" t="s">
         <v>53</v>
       </c>
-      <c r="V5" s="144"/>
-      <c r="Y5" s="137"/>
+      <c r="V5" s="149"/>
+      <c r="Y5" s="144"/>
       <c r="Z5" s="38">
         <v>2</v>
       </c>
@@ -29931,15 +29949,15 @@
       <c r="AD5" s="31" t="s">
         <v>57</v>
       </c>
-      <c r="AE5" s="137"/>
+      <c r="AE5" s="144"/>
       <c r="AG5" s="39">
         <v>2</v>
       </c>
-      <c r="AH5" s="145" t="s">
+      <c r="AH5" s="150" t="s">
         <v>58</v>
       </c>
-      <c r="AI5" s="145"/>
-      <c r="AL5" s="137"/>
+      <c r="AI5" s="150"/>
+      <c r="AL5" s="144"/>
     </row>
     <row r="6" spans="1:38" ht="57" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="40">
@@ -29957,35 +29975,35 @@
       <c r="E6" s="25" t="s">
         <v>62</v>
       </c>
-      <c r="F6" s="137"/>
+      <c r="F6" s="144"/>
       <c r="G6" s="41" t="s">
         <v>63</v>
       </c>
       <c r="H6" s="35" t="s">
         <v>64</v>
       </c>
-      <c r="I6" s="137"/>
+      <c r="I6" s="144"/>
       <c r="J6" s="42">
         <v>4</v>
       </c>
-      <c r="K6" s="138" t="s">
+      <c r="K6" s="146" t="s">
         <v>65</v>
       </c>
-      <c r="L6" s="138"/>
-      <c r="M6" s="138"/>
-      <c r="N6" s="138"/>
-      <c r="O6" s="138"/>
-      <c r="P6" s="138"/>
-      <c r="Q6" s="138"/>
-      <c r="R6" s="137"/>
+      <c r="L6" s="146"/>
+      <c r="M6" s="146"/>
+      <c r="N6" s="146"/>
+      <c r="O6" s="146"/>
+      <c r="P6" s="146"/>
+      <c r="Q6" s="146"/>
+      <c r="R6" s="144"/>
       <c r="T6" s="43">
         <v>3</v>
       </c>
-      <c r="U6" s="146" t="s">
+      <c r="U6" s="151" t="s">
         <v>66</v>
       </c>
-      <c r="V6" s="146"/>
-      <c r="Y6" s="137"/>
+      <c r="V6" s="151"/>
+      <c r="Y6" s="144"/>
       <c r="Z6" s="44">
         <v>3</v>
       </c>
@@ -30001,15 +30019,15 @@
       <c r="AD6" s="31" t="s">
         <v>70</v>
       </c>
-      <c r="AE6" s="137"/>
+      <c r="AE6" s="144"/>
       <c r="AG6" s="45">
         <v>3</v>
       </c>
-      <c r="AH6" s="147" t="s">
+      <c r="AH6" s="152" t="s">
         <v>71</v>
       </c>
-      <c r="AI6" s="147"/>
-      <c r="AL6" s="137"/>
+      <c r="AI6" s="152"/>
+      <c r="AL6" s="144"/>
     </row>
     <row r="7" spans="1:38" ht="71.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="46">
@@ -30027,27 +30045,27 @@
       <c r="E7" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="F7" s="137"/>
-      <c r="G7" s="140"/>
-      <c r="H7" s="140"/>
-      <c r="I7" s="137"/>
-      <c r="J7" s="148"/>
-      <c r="K7" s="148"/>
-      <c r="L7" s="148"/>
-      <c r="M7" s="148"/>
-      <c r="N7" s="148"/>
-      <c r="O7" s="148"/>
-      <c r="P7" s="148"/>
-      <c r="Q7" s="148"/>
-      <c r="R7" s="137"/>
+      <c r="F7" s="144"/>
+      <c r="G7" s="142"/>
+      <c r="H7" s="142"/>
+      <c r="I7" s="144"/>
+      <c r="J7" s="153"/>
+      <c r="K7" s="153"/>
+      <c r="L7" s="153"/>
+      <c r="M7" s="153"/>
+      <c r="N7" s="153"/>
+      <c r="O7" s="153"/>
+      <c r="P7" s="153"/>
+      <c r="Q7" s="153"/>
+      <c r="R7" s="144"/>
       <c r="T7" s="48">
         <v>4</v>
       </c>
-      <c r="U7" s="149" t="s">
+      <c r="U7" s="154" t="s">
         <v>71</v>
       </c>
-      <c r="V7" s="149"/>
-      <c r="Y7" s="137"/>
+      <c r="V7" s="154"/>
+      <c r="Y7" s="144"/>
       <c r="Z7" s="49">
         <v>4</v>
       </c>
@@ -30063,49 +30081,49 @@
       <c r="AD7" s="31" t="s">
         <v>79</v>
       </c>
-      <c r="AE7" s="137"/>
+      <c r="AE7" s="144"/>
       <c r="AG7" s="51"/>
-      <c r="AH7" s="150"/>
-      <c r="AI7" s="150"/>
-      <c r="AL7" s="137"/>
+      <c r="AH7" s="155"/>
+      <c r="AI7" s="155"/>
+      <c r="AL7" s="144"/>
     </row>
     <row r="8" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A8" s="140"/>
-      <c r="B8" s="140"/>
-      <c r="C8" s="140"/>
-      <c r="D8" s="140"/>
-      <c r="E8" s="140"/>
-      <c r="Z8" s="140"/>
-      <c r="AA8" s="140"/>
-      <c r="AB8" s="140"/>
-      <c r="AC8" s="140"/>
-      <c r="AD8" s="140"/>
+      <c r="A8" s="142"/>
+      <c r="B8" s="142"/>
+      <c r="C8" s="142"/>
+      <c r="D8" s="142"/>
+      <c r="E8" s="142"/>
+      <c r="Z8" s="142"/>
+      <c r="AA8" s="142"/>
+      <c r="AB8" s="142"/>
+      <c r="AC8" s="142"/>
+      <c r="AD8" s="142"/>
     </row>
     <row r="10" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="L10" s="151" t="s">
+      <c r="L10" s="140" t="s">
         <v>15</v>
       </c>
-      <c r="M10" s="151"/>
-      <c r="N10" s="153" t="s">
+      <c r="M10" s="140"/>
+      <c r="N10" s="143" t="s">
         <v>80</v>
       </c>
-      <c r="O10" s="153"/>
-      <c r="P10" s="153"/>
-      <c r="Q10" s="153"/>
-      <c r="S10" s="151" t="s">
+      <c r="O10" s="143"/>
+      <c r="P10" s="143"/>
+      <c r="Q10" s="143"/>
+      <c r="S10" s="140" t="s">
         <v>25</v>
       </c>
-      <c r="T10" s="151"/>
-      <c r="U10" s="153" t="s">
+      <c r="T10" s="140"/>
+      <c r="U10" s="143" t="s">
         <v>15</v>
       </c>
-      <c r="V10" s="153"/>
-      <c r="W10" s="153"/>
-      <c r="X10" s="153"/>
-      <c r="AF10" s="151" t="s">
+      <c r="V10" s="143"/>
+      <c r="W10" s="143"/>
+      <c r="X10" s="143"/>
+      <c r="AF10" s="140" t="s">
         <v>81</v>
       </c>
-      <c r="AG10" s="151"/>
+      <c r="AG10" s="140"/>
       <c r="AH10" s="52" t="s">
         <v>82</v>
       </c>
@@ -30113,8 +30131,8 @@
       <c r="AJ10" s="53"/>
     </row>
     <row r="11" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="L11" s="151"/>
-      <c r="M11" s="151"/>
+      <c r="L11" s="140"/>
+      <c r="M11" s="140"/>
       <c r="N11" s="54">
         <v>1</v>
       </c>
@@ -30127,8 +30145,8 @@
       <c r="Q11" s="57">
         <v>4</v>
       </c>
-      <c r="S11" s="151"/>
-      <c r="T11" s="151"/>
+      <c r="S11" s="140"/>
+      <c r="T11" s="140"/>
       <c r="U11" s="58">
         <v>1</v>
       </c>
@@ -30141,8 +30159,8 @@
       <c r="X11" s="58">
         <v>4</v>
       </c>
-      <c r="AF11" s="151"/>
-      <c r="AG11" s="151"/>
+      <c r="AF11" s="140"/>
+      <c r="AG11" s="140"/>
       <c r="AH11" s="58" t="s">
         <v>83</v>
       </c>
@@ -30154,7 +30172,7 @@
       </c>
     </row>
     <row r="12" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="L12" s="152" t="s">
+      <c r="L12" s="141" t="s">
         <v>86</v>
       </c>
       <c r="M12" s="54">
@@ -30172,7 +30190,7 @@
       <c r="Q12" s="61">
         <v>3</v>
       </c>
-      <c r="S12" s="152" t="s">
+      <c r="S12" s="141" t="s">
         <v>14</v>
       </c>
       <c r="T12" s="58">
@@ -30207,7 +30225,7 @@
       </c>
     </row>
     <row r="13" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="L13" s="152"/>
+      <c r="L13" s="141"/>
       <c r="M13" s="55">
         <v>2</v>
       </c>
@@ -30223,7 +30241,7 @@
       <c r="Q13" s="61">
         <v>3</v>
       </c>
-      <c r="S13" s="152"/>
+      <c r="S13" s="141"/>
       <c r="T13" s="58">
         <v>2</v>
       </c>
@@ -30254,7 +30272,7 @@
       </c>
     </row>
     <row r="14" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="L14" s="152"/>
+      <c r="L14" s="141"/>
       <c r="M14" s="56">
         <v>3</v>
       </c>
@@ -30270,7 +30288,7 @@
       <c r="Q14" s="70">
         <v>4</v>
       </c>
-      <c r="S14" s="152"/>
+      <c r="S14" s="141"/>
       <c r="T14" s="58">
         <v>3</v>
       </c>
@@ -30301,7 +30319,7 @@
       </c>
     </row>
     <row r="15" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="L15" s="152"/>
+      <c r="L15" s="141"/>
       <c r="M15" s="57">
         <v>4</v>
       </c>
@@ -30317,7 +30335,7 @@
       <c r="Q15" s="70">
         <v>4</v>
       </c>
-      <c r="S15" s="152"/>
+      <c r="S15" s="141"/>
       <c r="T15" s="58">
         <v>4</v>
       </c>
@@ -30336,15 +30354,17 @@
     </row>
   </sheetData>
   <mergeCells count="35">
-    <mergeCell ref="AF10:AG11"/>
-    <mergeCell ref="L12:L15"/>
-    <mergeCell ref="S12:S15"/>
-    <mergeCell ref="A8:E8"/>
-    <mergeCell ref="Z8:AD8"/>
-    <mergeCell ref="L10:M11"/>
-    <mergeCell ref="N10:Q10"/>
-    <mergeCell ref="S10:T11"/>
-    <mergeCell ref="U10:X10"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="J2:Q2"/>
+    <mergeCell ref="Z2:AD2"/>
+    <mergeCell ref="F3:F7"/>
+    <mergeCell ref="I3:I7"/>
+    <mergeCell ref="K3:Q3"/>
+    <mergeCell ref="R3:R7"/>
+    <mergeCell ref="U3:V3"/>
+    <mergeCell ref="Y3:Y7"/>
+    <mergeCell ref="G7:H7"/>
     <mergeCell ref="AE3:AE7"/>
     <mergeCell ref="AH3:AI3"/>
     <mergeCell ref="AL3:AL7"/>
@@ -30360,17 +30380,15 @@
     <mergeCell ref="J7:Q7"/>
     <mergeCell ref="U7:V7"/>
     <mergeCell ref="AH7:AI7"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="J2:Q2"/>
-    <mergeCell ref="Z2:AD2"/>
-    <mergeCell ref="F3:F7"/>
-    <mergeCell ref="I3:I7"/>
-    <mergeCell ref="K3:Q3"/>
-    <mergeCell ref="R3:R7"/>
-    <mergeCell ref="U3:V3"/>
-    <mergeCell ref="Y3:Y7"/>
-    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="AF10:AG11"/>
+    <mergeCell ref="L12:L15"/>
+    <mergeCell ref="S12:S15"/>
+    <mergeCell ref="A8:E8"/>
+    <mergeCell ref="Z8:AD8"/>
+    <mergeCell ref="L10:M11"/>
+    <mergeCell ref="N10:Q10"/>
+    <mergeCell ref="S10:T11"/>
+    <mergeCell ref="U10:X10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup paperSize="0" scale="0" firstPageNumber="0" orientation="portrait" usePrinterDefaults="0" horizontalDpi="0" verticalDpi="0" copies="0"/>
@@ -30403,246 +30421,246 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="27" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="163" t="s">
+      <c r="A1" s="136" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="169" t="s">
+      <c r="B1" s="166" t="s">
         <v>160</v>
       </c>
-      <c r="C1" s="170"/>
-      <c r="D1" s="170"/>
-      <c r="E1" s="170"/>
-      <c r="F1" s="170"/>
-      <c r="G1" s="170"/>
-      <c r="H1" s="170"/>
-      <c r="I1" s="170"/>
-      <c r="J1" s="170"/>
-      <c r="K1" s="170"/>
-      <c r="L1" s="170"/>
-      <c r="M1" s="170"/>
-      <c r="N1" s="171"/>
+      <c r="C1" s="167"/>
+      <c r="D1" s="167"/>
+      <c r="E1" s="167"/>
+      <c r="F1" s="167"/>
+      <c r="G1" s="167"/>
+      <c r="H1" s="167"/>
+      <c r="I1" s="167"/>
+      <c r="J1" s="167"/>
+      <c r="K1" s="167"/>
+      <c r="L1" s="167"/>
+      <c r="M1" s="167"/>
+      <c r="N1" s="168"/>
     </row>
     <row r="2" spans="1:14" ht="36.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="163" t="s">
+      <c r="A2" s="136" t="s">
         <v>89</v>
       </c>
-      <c r="B2" s="165" t="s">
+      <c r="B2" s="169" t="s">
         <v>161</v>
       </c>
-      <c r="C2" s="167"/>
-      <c r="D2" s="167"/>
-      <c r="E2" s="167"/>
-      <c r="F2" s="168"/>
-      <c r="G2" s="164" t="s">
+      <c r="C2" s="170"/>
+      <c r="D2" s="170"/>
+      <c r="E2" s="170"/>
+      <c r="F2" s="171"/>
+      <c r="G2" s="137" t="s">
         <v>162</v>
       </c>
-      <c r="H2" s="165" t="s">
+      <c r="H2" s="169" t="s">
         <v>163</v>
       </c>
-      <c r="I2" s="168"/>
-      <c r="J2" s="165" t="s">
+      <c r="I2" s="171"/>
+      <c r="J2" s="169" t="s">
         <v>164</v>
       </c>
-      <c r="K2" s="167"/>
-      <c r="L2" s="168"/>
-      <c r="M2" s="165" t="s">
+      <c r="K2" s="170"/>
+      <c r="L2" s="171"/>
+      <c r="M2" s="169" t="s">
         <v>165</v>
       </c>
-      <c r="N2" s="167"/>
+      <c r="N2" s="170"/>
     </row>
     <row r="3" spans="1:14" ht="50.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="163" t="s">
+      <c r="A3" s="136" t="s">
         <v>90</v>
       </c>
-      <c r="B3" s="154" t="s">
+      <c r="B3" s="160" t="s">
         <v>91</v>
       </c>
-      <c r="C3" s="172"/>
-      <c r="D3" s="172"/>
-      <c r="E3" s="172"/>
-      <c r="F3" s="173"/>
+      <c r="C3" s="161"/>
+      <c r="D3" s="161"/>
+      <c r="E3" s="161"/>
+      <c r="F3" s="165"/>
       <c r="G3" s="72" t="s">
         <v>92</v>
       </c>
-      <c r="H3" s="154" t="s">
+      <c r="H3" s="160" t="s">
         <v>91</v>
       </c>
-      <c r="I3" s="173"/>
-      <c r="J3" s="154" t="s">
+      <c r="I3" s="165"/>
+      <c r="J3" s="160" t="s">
         <v>92</v>
       </c>
-      <c r="K3" s="172"/>
-      <c r="L3" s="173"/>
-      <c r="M3" s="154" t="s">
+      <c r="K3" s="161"/>
+      <c r="L3" s="165"/>
+      <c r="M3" s="160" t="s">
         <v>93</v>
       </c>
-      <c r="N3" s="172"/>
+      <c r="N3" s="161"/>
     </row>
     <row r="4" spans="1:14" ht="124.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="163" t="s">
+      <c r="A4" s="136" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="154" t="s">
+      <c r="B4" s="160" t="s">
         <v>166</v>
       </c>
-      <c r="C4" s="172"/>
-      <c r="D4" s="172"/>
-      <c r="E4" s="172"/>
-      <c r="F4" s="173"/>
+      <c r="C4" s="161"/>
+      <c r="D4" s="161"/>
+      <c r="E4" s="161"/>
+      <c r="F4" s="165"/>
       <c r="G4" s="72" t="s">
         <v>167</v>
       </c>
-      <c r="H4" s="154" t="s">
+      <c r="H4" s="160" t="s">
         <v>168</v>
       </c>
-      <c r="I4" s="173"/>
-      <c r="J4" s="154" t="s">
+      <c r="I4" s="165"/>
+      <c r="J4" s="160" t="s">
         <v>169</v>
       </c>
-      <c r="K4" s="172"/>
-      <c r="L4" s="173"/>
-      <c r="M4" s="154" t="s">
+      <c r="K4" s="161"/>
+      <c r="L4" s="165"/>
+      <c r="M4" s="160" t="s">
         <v>170</v>
       </c>
-      <c r="N4" s="172"/>
+      <c r="N4" s="161"/>
     </row>
     <row r="5" spans="1:14" ht="30" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="163" t="s">
+      <c r="A5" s="136" t="s">
         <v>94</v>
       </c>
-      <c r="B5" s="154" t="s">
+      <c r="B5" s="160" t="s">
         <v>196</v>
       </c>
-      <c r="C5" s="172"/>
-      <c r="D5" s="172"/>
-      <c r="E5" s="172"/>
-      <c r="F5" s="172"/>
-      <c r="G5" s="172"/>
-      <c r="H5" s="172"/>
-      <c r="I5" s="172"/>
-      <c r="J5" s="172"/>
-      <c r="K5" s="172"/>
-      <c r="L5" s="172"/>
-      <c r="M5" s="172"/>
-      <c r="N5" s="172"/>
+      <c r="C5" s="161"/>
+      <c r="D5" s="161"/>
+      <c r="E5" s="161"/>
+      <c r="F5" s="161"/>
+      <c r="G5" s="161"/>
+      <c r="H5" s="161"/>
+      <c r="I5" s="161"/>
+      <c r="J5" s="161"/>
+      <c r="K5" s="161"/>
+      <c r="L5" s="161"/>
+      <c r="M5" s="161"/>
+      <c r="N5" s="161"/>
     </row>
     <row r="6" spans="1:14" ht="116.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="163" t="s">
+      <c r="A6" s="136" t="s">
         <v>95</v>
       </c>
-      <c r="B6" s="160" t="s">
+      <c r="B6" s="133" t="s">
         <v>171</v>
       </c>
-      <c r="C6" s="161" t="s">
+      <c r="C6" s="134" t="s">
         <v>172</v>
       </c>
-      <c r="D6" s="174" t="s">
+      <c r="D6" s="162" t="s">
         <v>173</v>
       </c>
-      <c r="E6" s="175"/>
-      <c r="F6" s="176"/>
-      <c r="G6" s="161" t="s">
+      <c r="E6" s="163"/>
+      <c r="F6" s="164"/>
+      <c r="G6" s="134" t="s">
         <v>174</v>
       </c>
-      <c r="H6" s="160" t="s">
+      <c r="H6" s="133" t="s">
         <v>175</v>
       </c>
-      <c r="I6" s="166" t="s">
+      <c r="I6" s="138" t="s">
         <v>176</v>
       </c>
-      <c r="J6" s="166" t="s">
+      <c r="J6" s="138" t="s">
         <v>177</v>
       </c>
-      <c r="K6" s="166" t="s">
+      <c r="K6" s="138" t="s">
         <v>178</v>
       </c>
-      <c r="L6" s="160" t="s">
+      <c r="L6" s="133" t="s">
         <v>179</v>
       </c>
-      <c r="M6" s="161" t="s">
+      <c r="M6" s="134" t="s">
         <v>180</v>
       </c>
-      <c r="N6" s="161" t="s">
+      <c r="N6" s="134" t="s">
         <v>181</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="114" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="163" t="s">
+      <c r="A7" s="136" t="s">
         <v>32</v>
       </c>
-      <c r="B7" s="160" t="s">
+      <c r="B7" s="133" t="s">
         <v>186</v>
       </c>
-      <c r="C7" s="161" t="s">
+      <c r="C7" s="134" t="s">
         <v>188</v>
       </c>
-      <c r="D7" s="174" t="s">
+      <c r="D7" s="162" t="s">
         <v>190</v>
       </c>
-      <c r="E7" s="175"/>
-      <c r="F7" s="176"/>
-      <c r="G7" s="161" t="s">
+      <c r="E7" s="163"/>
+      <c r="F7" s="164"/>
+      <c r="G7" s="134" t="s">
         <v>192</v>
       </c>
-      <c r="H7" s="160" t="s">
+      <c r="H7" s="133" t="s">
         <v>193</v>
       </c>
-      <c r="I7" s="166" t="s">
+      <c r="I7" s="138" t="s">
         <v>182</v>
       </c>
-      <c r="J7" s="166" t="s">
+      <c r="J7" s="138" t="s">
         <v>183</v>
       </c>
-      <c r="K7" s="162" t="s">
+      <c r="K7" s="135" t="s">
         <v>184</v>
       </c>
-      <c r="L7" s="160" t="s">
+      <c r="L7" s="133" t="s">
         <v>185</v>
       </c>
-      <c r="M7" s="161" t="s">
+      <c r="M7" s="134" t="s">
         <v>194</v>
       </c>
-      <c r="N7" s="161" t="s">
+      <c r="N7" s="134" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="61.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="163" t="s">
+      <c r="A8" s="136" t="s">
         <v>94</v>
       </c>
-      <c r="B8" s="160" t="s">
+      <c r="B8" s="133" t="s">
         <v>187</v>
       </c>
-      <c r="C8" s="161" t="s">
+      <c r="C8" s="134" t="s">
         <v>189</v>
       </c>
-      <c r="D8" s="174" t="s">
+      <c r="D8" s="162" t="s">
         <v>191</v>
       </c>
-      <c r="E8" s="175"/>
-      <c r="F8" s="176"/>
-      <c r="G8" s="161" t="s">
+      <c r="E8" s="163"/>
+      <c r="F8" s="164"/>
+      <c r="G8" s="134" t="s">
         <v>189</v>
       </c>
-      <c r="H8" s="160" t="s">
+      <c r="H8" s="133" t="s">
         <v>189</v>
       </c>
-      <c r="I8" s="166" t="s">
+      <c r="I8" s="138" t="s">
         <v>191</v>
       </c>
-      <c r="J8" s="166" t="s">
+      <c r="J8" s="138" t="s">
         <v>191</v>
       </c>
-      <c r="K8" s="160" t="s">
+      <c r="K8" s="133" t="s">
         <v>191</v>
       </c>
-      <c r="L8" s="160" t="s">
+      <c r="L8" s="133" t="s">
         <v>191</v>
       </c>
-      <c r="M8" s="161" t="s">
+      <c r="M8" s="134" t="s">
         <v>189</v>
       </c>
-      <c r="N8" s="161" t="s">
+      <c r="N8" s="134" t="s">
         <v>189</v>
       </c>
     </row>
@@ -30726,6 +30744,11 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="B1:N1"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="M2:N2"/>
     <mergeCell ref="B5:N5"/>
     <mergeCell ref="D6:F6"/>
     <mergeCell ref="D7:F7"/>
@@ -30738,11 +30761,6 @@
     <mergeCell ref="H4:I4"/>
     <mergeCell ref="J4:L4"/>
     <mergeCell ref="M4:N4"/>
-    <mergeCell ref="B1:N1"/>
-    <mergeCell ref="B2:F2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="J2:L2"/>
-    <mergeCell ref="M2:N2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
@@ -30767,172 +30785,174 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="155" t="s">
+      <c r="A1" s="181" t="s">
         <v>96</v>
       </c>
-      <c r="B1" s="155"/>
-      <c r="C1" s="156" t="s">
+      <c r="B1" s="181"/>
+      <c r="C1" s="182" t="s">
         <v>97</v>
       </c>
-      <c r="D1" s="156"/>
+      <c r="D1" s="182"/>
+      <c r="E1" s="183"/>
+      <c r="F1" s="183"/>
     </row>
     <row r="2" spans="1:6" ht="42.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="73" t="s">
+      <c r="A2" s="175" t="s">
         <v>98</v>
       </c>
-      <c r="B2" s="74" t="s">
+      <c r="B2" s="175" t="s">
         <v>99</v>
       </c>
-      <c r="C2" s="73" t="s">
+      <c r="C2" s="175" t="s">
         <v>100</v>
       </c>
-      <c r="D2" s="73" t="s">
+      <c r="D2" s="175" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="73" t="s">
+      <c r="E2" s="175" t="s">
         <v>475</v>
       </c>
-      <c r="F2" s="73" t="s">
+      <c r="F2" s="175" t="s">
         <v>476</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="120" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="75" t="s">
+      <c r="A3" s="176" t="s">
         <v>161</v>
       </c>
-      <c r="B3" s="76" t="s">
+      <c r="B3" s="80" t="s">
         <v>201</v>
       </c>
-      <c r="C3" s="76" t="s">
+      <c r="C3" s="80" t="s">
         <v>490</v>
       </c>
-      <c r="D3" s="77" t="s">
+      <c r="D3" s="177" t="s">
         <v>38</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="183" t="s">
         <v>477</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="183" t="s">
         <v>478</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="75" t="s">
+      <c r="A4" s="176" t="s">
         <v>161</v>
       </c>
-      <c r="B4" s="76" t="s">
+      <c r="B4" s="80" t="s">
         <v>280</v>
       </c>
-      <c r="C4" s="76" t="s">
+      <c r="C4" s="80" t="s">
         <v>281</v>
       </c>
-      <c r="D4" s="77" t="s">
+      <c r="D4" s="177" t="s">
         <v>50</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="183" t="s">
         <v>479</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="183" t="s">
         <v>480</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="75" t="s">
+      <c r="A5" s="176" t="s">
         <v>162</v>
       </c>
-      <c r="B5" s="76" t="s">
+      <c r="B5" s="80" t="s">
         <v>282</v>
       </c>
-      <c r="C5" s="76" t="s">
+      <c r="C5" s="80" t="s">
         <v>283</v>
       </c>
-      <c r="D5" s="78" t="s">
+      <c r="D5" s="178" t="s">
         <v>38</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="183" t="s">
         <v>481</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="183" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="75" t="s">
+      <c r="A6" s="176" t="s">
         <v>163</v>
       </c>
-      <c r="B6" s="76" t="s">
+      <c r="B6" s="80" t="s">
         <v>284</v>
       </c>
-      <c r="C6" s="76" t="s">
+      <c r="C6" s="80" t="s">
         <v>285</v>
       </c>
-      <c r="D6" s="79" t="s">
+      <c r="D6" s="179" t="s">
         <v>50</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="183" t="s">
         <v>483</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="183" t="s">
         <v>484</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="75" t="s">
+      <c r="A7" s="176" t="s">
         <v>163</v>
       </c>
-      <c r="B7" s="76" t="s">
+      <c r="B7" s="80" t="s">
         <v>286</v>
       </c>
-      <c r="C7" s="76" t="s">
+      <c r="C7" s="80" t="s">
         <v>287</v>
       </c>
-      <c r="D7" s="80" t="s">
+      <c r="D7" s="180" t="s">
         <v>38</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="183" t="s">
         <v>485</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="183" t="s">
         <v>486</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="81" t="s">
+      <c r="A8" s="79" t="s">
         <v>164</v>
       </c>
-      <c r="B8" s="82" t="s">
+      <c r="B8" s="80" t="s">
         <v>202</v>
       </c>
-      <c r="C8" s="82" t="s">
+      <c r="C8" s="80" t="s">
         <v>491</v>
       </c>
-      <c r="D8" s="83" t="s">
+      <c r="D8" s="179" t="s">
         <v>22</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="183" t="s">
         <v>487</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="183" t="s">
         <v>488</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="84" t="s">
+      <c r="A9" s="79" t="s">
         <v>165</v>
       </c>
-      <c r="B9" s="76" t="s">
+      <c r="B9" s="80" t="s">
         <v>288</v>
       </c>
-      <c r="C9" s="76" t="s">
+      <c r="C9" s="80" t="s">
         <v>289</v>
       </c>
-      <c r="D9" s="79" t="s">
+      <c r="D9" s="179" t="s">
         <v>50</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="183" t="s">
         <v>483</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="183" t="s">
         <v>489</v>
       </c>
     </row>
@@ -30974,14 +30994,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="155" t="s">
+      <c r="A1" s="172" t="s">
         <v>96</v>
       </c>
-      <c r="B1" s="155"/>
-      <c r="C1" s="156" t="s">
+      <c r="B1" s="172"/>
+      <c r="C1" s="173" t="s">
         <v>97</v>
       </c>
-      <c r="D1" s="156"/>
+      <c r="D1" s="173"/>
     </row>
     <row r="2" spans="1:5" ht="42.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="73" t="s">
@@ -31001,223 +31021,223 @@
       </c>
     </row>
     <row r="3" spans="1:5" ht="79.900000000000006" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="114" t="s">
+      <c r="A3" s="111" t="s">
         <v>250</v>
       </c>
-      <c r="B3" s="115" t="s">
+      <c r="B3" s="112" t="s">
         <v>251</v>
       </c>
-      <c r="C3" s="115" t="s">
+      <c r="C3" s="112" t="s">
         <v>252</v>
       </c>
-      <c r="D3" s="115" t="s">
+      <c r="D3" s="112" t="s">
         <v>253</v>
       </c>
-      <c r="E3" s="116" t="s">
+      <c r="E3" s="113" t="s">
         <v>254</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="79.900000000000006" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="117" t="s">
+      <c r="A4" s="114" t="s">
         <v>250</v>
       </c>
-      <c r="B4" s="118" t="s">
+      <c r="B4" s="115" t="s">
         <v>251</v>
       </c>
-      <c r="C4" s="118" t="s">
+      <c r="C4" s="115" t="s">
         <v>252</v>
       </c>
-      <c r="D4" s="118" t="s">
+      <c r="D4" s="115" t="s">
         <v>255</v>
       </c>
-      <c r="E4" s="119" t="s">
+      <c r="E4" s="116" t="s">
         <v>256</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="79.900000000000006" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="117" t="s">
+      <c r="A5" s="114" t="s">
         <v>250</v>
       </c>
-      <c r="B5" s="118" t="s">
+      <c r="B5" s="115" t="s">
         <v>251</v>
       </c>
-      <c r="C5" s="118" t="s">
+      <c r="C5" s="115" t="s">
         <v>252</v>
       </c>
-      <c r="D5" s="118" t="s">
+      <c r="D5" s="115" t="s">
         <v>492</v>
       </c>
-      <c r="E5" s="119" t="s">
+      <c r="E5" s="116" t="s">
         <v>493</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="79.900000000000006" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="117" t="s">
+      <c r="A6" s="114" t="s">
         <v>250</v>
       </c>
-      <c r="B6" s="118" t="s">
+      <c r="B6" s="115" t="s">
         <v>251</v>
       </c>
-      <c r="C6" s="118" t="s">
+      <c r="C6" s="115" t="s">
         <v>252</v>
       </c>
-      <c r="D6" s="118" t="s">
+      <c r="D6" s="115" t="s">
         <v>257</v>
       </c>
-      <c r="E6" s="119" t="s">
+      <c r="E6" s="116" t="s">
         <v>258</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="79.900000000000006" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="117" t="s">
+      <c r="A7" s="114" t="s">
         <v>250</v>
       </c>
-      <c r="B7" s="118" t="s">
+      <c r="B7" s="115" t="s">
         <v>251</v>
       </c>
-      <c r="C7" s="118" t="s">
+      <c r="C7" s="115" t="s">
         <v>259</v>
       </c>
-      <c r="D7" s="118" t="s">
+      <c r="D7" s="115" t="s">
         <v>260</v>
       </c>
-      <c r="E7" s="119" t="s">
+      <c r="E7" s="116" t="s">
         <v>261</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="79.900000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="120" t="s">
+      <c r="A8" s="117" t="s">
         <v>250</v>
       </c>
-      <c r="B8" s="121" t="s">
+      <c r="B8" s="118" t="s">
         <v>251</v>
       </c>
-      <c r="C8" s="121" t="s">
+      <c r="C8" s="118" t="s">
         <v>262</v>
       </c>
-      <c r="D8" s="121" t="s">
+      <c r="D8" s="118" t="s">
         <v>263</v>
       </c>
-      <c r="E8" s="122" t="s">
+      <c r="E8" s="119" t="s">
         <v>494</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="79.900000000000006" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="120" t="s">
+      <c r="A9" s="117" t="s">
         <v>250</v>
       </c>
-      <c r="B9" s="121" t="s">
+      <c r="B9" s="118" t="s">
         <v>251</v>
       </c>
-      <c r="C9" s="121" t="s">
+      <c r="C9" s="118" t="s">
         <v>259</v>
       </c>
-      <c r="D9" s="121" t="s">
+      <c r="D9" s="118" t="s">
         <v>264</v>
       </c>
-      <c r="E9" s="122" t="s">
+      <c r="E9" s="119" t="s">
         <v>265</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="79.900000000000006" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="120" t="s">
+      <c r="A10" s="117" t="s">
         <v>250</v>
       </c>
-      <c r="B10" s="121" t="s">
+      <c r="B10" s="118" t="s">
         <v>251</v>
       </c>
-      <c r="C10" s="121" t="s">
+      <c r="C10" s="118" t="s">
         <v>252</v>
       </c>
-      <c r="D10" s="121" t="s">
+      <c r="D10" s="118" t="s">
         <v>495</v>
       </c>
-      <c r="E10" s="122" t="s">
+      <c r="E10" s="119" t="s">
         <v>496</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="79.900000000000006" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="120" t="s">
+      <c r="A11" s="117" t="s">
         <v>266</v>
       </c>
-      <c r="B11" s="121" t="s">
+      <c r="B11" s="118" t="s">
         <v>267</v>
       </c>
-      <c r="C11" s="121" t="s">
+      <c r="C11" s="118" t="s">
         <v>252</v>
       </c>
-      <c r="D11" s="121" t="s">
+      <c r="D11" s="118" t="s">
         <v>268</v>
       </c>
-      <c r="E11" s="122" t="s">
+      <c r="E11" s="119" t="s">
         <v>269</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="79.900000000000006" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="120" t="s">
+      <c r="A12" s="117" t="s">
         <v>266</v>
       </c>
-      <c r="B12" s="121" t="s">
+      <c r="B12" s="118" t="s">
         <v>270</v>
       </c>
-      <c r="C12" s="121" t="s">
+      <c r="C12" s="118" t="s">
         <v>271</v>
       </c>
-      <c r="D12" s="121" t="s">
+      <c r="D12" s="118" t="s">
         <v>530</v>
       </c>
-      <c r="E12" s="122" t="s">
+      <c r="E12" s="119" t="s">
         <v>272</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="79.900000000000006" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="120" t="s">
+      <c r="A13" s="117" t="s">
         <v>273</v>
       </c>
-      <c r="B13" s="121" t="s">
+      <c r="B13" s="118" t="s">
         <v>274</v>
       </c>
-      <c r="C13" s="121" t="s">
+      <c r="C13" s="118" t="s">
         <v>252</v>
       </c>
-      <c r="D13" s="121" t="s">
+      <c r="D13" s="118" t="s">
         <v>275</v>
       </c>
-      <c r="E13" s="122" t="s">
+      <c r="E13" s="119" t="s">
         <v>276</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="79.900000000000006" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="120" t="s">
+      <c r="A14" s="117" t="s">
         <v>273</v>
       </c>
-      <c r="B14" s="121" t="s">
+      <c r="B14" s="118" t="s">
         <v>277</v>
       </c>
-      <c r="C14" s="121" t="s">
+      <c r="C14" s="118" t="s">
         <v>262</v>
       </c>
-      <c r="D14" s="121" t="s">
+      <c r="D14" s="118" t="s">
         <v>278</v>
       </c>
-      <c r="E14" s="122" t="s">
+      <c r="E14" s="119" t="s">
         <v>279</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="79.900000000000006" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="120" t="s">
+      <c r="A15" s="117" t="s">
         <v>531</v>
       </c>
-      <c r="B15" s="121" t="s">
+      <c r="B15" s="118" t="s">
         <v>532</v>
       </c>
-      <c r="C15" s="121" t="s">
+      <c r="C15" s="118" t="s">
         <v>259</v>
       </c>
-      <c r="D15" s="121" t="s">
+      <c r="D15" s="118" t="s">
         <v>533</v>
       </c>
-      <c r="E15" s="122" t="s">
+      <c r="E15" s="119" t="s">
         <v>534</v>
       </c>
     </row>
@@ -31250,24 +31270,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="155" t="s">
+      <c r="A1" s="172" t="s">
         <v>96</v>
       </c>
-      <c r="B1" s="155"/>
-      <c r="C1" s="156" t="s">
+      <c r="B1" s="172"/>
+      <c r="C1" s="173" t="s">
         <v>97</v>
       </c>
-      <c r="D1" s="156"/>
-      <c r="E1" s="157" t="s">
+      <c r="D1" s="173"/>
+      <c r="E1" s="174" t="s">
         <v>106</v>
       </c>
-      <c r="F1" s="157"/>
+      <c r="F1" s="174"/>
     </row>
     <row r="2" spans="1:8" ht="42.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="73" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="85" t="s">
+      <c r="B2" s="82" t="s">
         <v>108</v>
       </c>
       <c r="C2" s="73" t="s">
@@ -31293,7 +31313,7 @@
       <c r="A3" s="75" t="s">
         <v>203</v>
       </c>
-      <c r="B3" s="86" t="s">
+      <c r="B3" s="83" t="s">
         <v>204</v>
       </c>
       <c r="C3" s="75" t="s">
@@ -31302,7 +31322,7 @@
       <c r="D3" s="75" t="s">
         <v>84</v>
       </c>
-      <c r="E3" s="79" t="s">
+      <c r="E3" s="78" t="s">
         <v>115</v>
       </c>
       <c r="F3" s="75">
@@ -31317,7 +31337,7 @@
       <c r="A4" s="75" t="s">
         <v>205</v>
       </c>
-      <c r="B4" s="86" t="s">
+      <c r="B4" s="83" t="s">
         <v>206</v>
       </c>
       <c r="C4" s="75" t="s">
@@ -31326,7 +31346,7 @@
       <c r="D4" s="75" t="s">
         <v>83</v>
       </c>
-      <c r="E4" s="78" t="s">
+      <c r="E4" s="77" t="s">
         <v>113</v>
       </c>
       <c r="F4" s="75">
@@ -31341,7 +31361,7 @@
       <c r="A5" s="75" t="s">
         <v>207</v>
       </c>
-      <c r="B5" s="86" t="s">
+      <c r="B5" s="83" t="s">
         <v>208</v>
       </c>
       <c r="C5" s="75" t="s">
@@ -31350,7 +31370,7 @@
       <c r="D5" s="75" t="s">
         <v>84</v>
       </c>
-      <c r="E5" s="87" t="s">
+      <c r="E5" s="84" t="s">
         <v>113</v>
       </c>
       <c r="F5" s="75">
@@ -31365,7 +31385,7 @@
       <c r="A6" s="75" t="s">
         <v>209</v>
       </c>
-      <c r="B6" s="86" t="s">
+      <c r="B6" s="83" t="s">
         <v>210</v>
       </c>
       <c r="C6" s="75" t="s">
@@ -31374,7 +31394,7 @@
       <c r="D6" s="75" t="s">
         <v>83</v>
       </c>
-      <c r="E6" s="87" t="s">
+      <c r="E6" s="84" t="s">
         <v>41</v>
       </c>
       <c r="F6" s="75">
@@ -31391,7 +31411,7 @@
       <c r="A7" s="75" t="s">
         <v>212</v>
       </c>
-      <c r="B7" s="86" t="s">
+      <c r="B7" s="83" t="s">
         <v>213</v>
       </c>
       <c r="C7" s="75" t="s">
@@ -31400,7 +31420,7 @@
       <c r="D7" s="75" t="s">
         <v>85</v>
       </c>
-      <c r="E7" s="87" t="s">
+      <c r="E7" s="84" t="s">
         <v>113</v>
       </c>
       <c r="F7" s="75">
@@ -31417,7 +31437,7 @@
       <c r="A8" s="75" t="s">
         <v>215</v>
       </c>
-      <c r="B8" s="86" t="s">
+      <c r="B8" s="83" t="s">
         <v>216</v>
       </c>
       <c r="C8" s="75" t="s">
@@ -31426,7 +31446,7 @@
       <c r="D8" s="75" t="s">
         <v>84</v>
       </c>
-      <c r="E8" s="87" t="s">
+      <c r="E8" s="84" t="s">
         <v>41</v>
       </c>
       <c r="F8" s="75">
@@ -31443,7 +31463,7 @@
       <c r="A9" s="75" t="s">
         <v>218</v>
       </c>
-      <c r="B9" s="86" t="s">
+      <c r="B9" s="83" t="s">
         <v>219</v>
       </c>
       <c r="C9" s="75" t="s">
@@ -31452,7 +31472,7 @@
       <c r="D9" s="75" t="s">
         <v>83</v>
       </c>
-      <c r="E9" s="87" t="s">
+      <c r="E9" s="84" t="s">
         <v>41</v>
       </c>
       <c r="F9" s="75">
@@ -31469,7 +31489,7 @@
       <c r="A10" s="75" t="s">
         <v>221</v>
       </c>
-      <c r="B10" s="86" t="s">
+      <c r="B10" s="83" t="s">
         <v>222</v>
       </c>
       <c r="C10" s="75" t="s">
@@ -31478,7 +31498,7 @@
       <c r="D10" s="75" t="s">
         <v>83</v>
       </c>
-      <c r="E10" s="87" t="s">
+      <c r="E10" s="84" t="s">
         <v>41</v>
       </c>
       <c r="F10" s="75">
@@ -31553,7 +31573,7 @@
       <c r="A1" s="73" t="s">
         <v>117</v>
       </c>
-      <c r="B1" s="85" t="s">
+      <c r="B1" s="82" t="s">
         <v>31</v>
       </c>
       <c r="C1" s="73" t="s">
@@ -31568,7 +31588,7 @@
       <c r="F1" s="73" t="s">
         <v>30</v>
       </c>
-      <c r="G1" s="85" t="s">
+      <c r="G1" s="82" t="s">
         <v>119</v>
       </c>
       <c r="H1" s="73" t="s">
@@ -31582,33 +31602,33 @@
       </c>
     </row>
     <row r="2" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="84" t="s">
+      <c r="A2" s="81" t="s">
         <v>224</v>
       </c>
-      <c r="B2" s="177" t="s">
+      <c r="B2" s="139" t="s">
         <v>225</v>
       </c>
-      <c r="C2" s="88">
-        <v>4</v>
-      </c>
-      <c r="D2" s="88">
-        <v>4</v>
-      </c>
-      <c r="E2" s="88">
-        <v>2</v>
-      </c>
-      <c r="F2" s="88">
-        <v>2</v>
-      </c>
-      <c r="G2" s="89">
+      <c r="C2" s="85">
+        <v>4</v>
+      </c>
+      <c r="D2" s="85">
+        <v>4</v>
+      </c>
+      <c r="E2" s="85">
+        <v>2</v>
+      </c>
+      <c r="F2" s="85">
+        <v>2</v>
+      </c>
+      <c r="G2" s="86">
         <f t="shared" ref="G2:G10" si="0">C2*D2</f>
         <v>16</v>
       </c>
-      <c r="H2" s="90">
+      <c r="H2" s="87">
         <f t="shared" ref="H2:H10" si="1">E2*F2</f>
         <v>4</v>
       </c>
-      <c r="I2" s="91">
+      <c r="I2" s="88">
         <f t="shared" ref="I2:I10" si="2">G2/H2</f>
         <v>4</v>
       </c>
@@ -31617,33 +31637,33 @@
       </c>
     </row>
     <row r="3" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="84" t="s">
+      <c r="A3" s="81" t="s">
         <v>226</v>
       </c>
-      <c r="B3" s="177" t="s">
+      <c r="B3" s="139" t="s">
         <v>227</v>
       </c>
-      <c r="C3" s="88">
-        <v>4</v>
-      </c>
-      <c r="D3" s="88">
-        <v>4</v>
-      </c>
-      <c r="E3" s="88">
-        <v>3</v>
-      </c>
-      <c r="F3" s="88">
-        <v>3</v>
-      </c>
-      <c r="G3" s="89">
+      <c r="C3" s="85">
+        <v>4</v>
+      </c>
+      <c r="D3" s="85">
+        <v>4</v>
+      </c>
+      <c r="E3" s="85">
+        <v>3</v>
+      </c>
+      <c r="F3" s="85">
+        <v>3</v>
+      </c>
+      <c r="G3" s="86">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="H3" s="90">
+      <c r="H3" s="87">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="I3" s="91">
+      <c r="I3" s="88">
         <f t="shared" si="2"/>
         <v>1.7777777777777777</v>
       </c>
@@ -31652,33 +31672,33 @@
       </c>
     </row>
     <row r="4" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="84" t="s">
+      <c r="A4" s="81" t="s">
         <v>226</v>
       </c>
-      <c r="B4" s="177" t="s">
+      <c r="B4" s="139" t="s">
         <v>228</v>
       </c>
-      <c r="C4" s="88">
-        <v>4</v>
-      </c>
-      <c r="D4" s="88">
-        <v>3</v>
-      </c>
-      <c r="E4" s="88">
-        <v>3</v>
-      </c>
-      <c r="F4" s="88">
-        <v>3</v>
-      </c>
-      <c r="G4" s="89">
+      <c r="C4" s="85">
+        <v>4</v>
+      </c>
+      <c r="D4" s="85">
+        <v>3</v>
+      </c>
+      <c r="E4" s="85">
+        <v>3</v>
+      </c>
+      <c r="F4" s="85">
+        <v>3</v>
+      </c>
+      <c r="G4" s="86">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="H4" s="90">
+      <c r="H4" s="87">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="I4" s="91">
+      <c r="I4" s="88">
         <f t="shared" si="2"/>
         <v>1.3333333333333333</v>
       </c>
@@ -31687,33 +31707,33 @@
       </c>
     </row>
     <row r="5" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="84" t="s">
+      <c r="A5" s="81" t="s">
         <v>224</v>
       </c>
-      <c r="B5" s="177" t="s">
+      <c r="B5" s="139" t="s">
         <v>229</v>
       </c>
-      <c r="C5" s="88">
-        <v>2</v>
-      </c>
-      <c r="D5" s="88">
-        <v>1</v>
-      </c>
-      <c r="E5" s="88">
-        <v>2</v>
-      </c>
-      <c r="F5" s="88">
-        <v>2</v>
-      </c>
-      <c r="G5" s="89">
+      <c r="C5" s="85">
+        <v>2</v>
+      </c>
+      <c r="D5" s="85">
+        <v>1</v>
+      </c>
+      <c r="E5" s="85">
+        <v>2</v>
+      </c>
+      <c r="F5" s="85">
+        <v>2</v>
+      </c>
+      <c r="G5" s="86">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="H5" s="90">
+      <c r="H5" s="87">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="I5" s="91">
+      <c r="I5" s="88">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
@@ -31722,33 +31742,33 @@
       </c>
     </row>
     <row r="6" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="84" t="s">
+      <c r="A6" s="81" t="s">
         <v>230</v>
       </c>
-      <c r="B6" s="177" t="s">
+      <c r="B6" s="139" t="s">
         <v>231</v>
       </c>
-      <c r="C6" s="88">
-        <v>2</v>
-      </c>
-      <c r="D6" s="88">
-        <v>2</v>
-      </c>
-      <c r="E6" s="88">
-        <v>2</v>
-      </c>
-      <c r="F6" s="88">
-        <v>3</v>
-      </c>
-      <c r="G6" s="89">
+      <c r="C6" s="85">
+        <v>2</v>
+      </c>
+      <c r="D6" s="85">
+        <v>2</v>
+      </c>
+      <c r="E6" s="85">
+        <v>2</v>
+      </c>
+      <c r="F6" s="85">
+        <v>3</v>
+      </c>
+      <c r="G6" s="86">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="H6" s="90">
+      <c r="H6" s="87">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="I6" s="91">
+      <c r="I6" s="88">
         <f t="shared" si="2"/>
         <v>0.66666666666666663</v>
       </c>
@@ -31757,33 +31777,33 @@
       </c>
     </row>
     <row r="7" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="84" t="s">
+      <c r="A7" s="81" t="s">
         <v>232</v>
       </c>
-      <c r="B7" s="177" t="s">
+      <c r="B7" s="139" t="s">
         <v>233</v>
       </c>
-      <c r="C7" s="88">
-        <v>3</v>
-      </c>
-      <c r="D7" s="88">
-        <v>1</v>
-      </c>
-      <c r="E7" s="88">
-        <v>2</v>
-      </c>
-      <c r="F7" s="88">
-        <v>3</v>
-      </c>
-      <c r="G7" s="89">
+      <c r="C7" s="85">
+        <v>3</v>
+      </c>
+      <c r="D7" s="85">
+        <v>1</v>
+      </c>
+      <c r="E7" s="85">
+        <v>2</v>
+      </c>
+      <c r="F7" s="85">
+        <v>3</v>
+      </c>
+      <c r="G7" s="86">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="H7" s="90">
+      <c r="H7" s="87">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="I7" s="91">
+      <c r="I7" s="88">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
@@ -31792,33 +31812,33 @@
       </c>
     </row>
     <row r="8" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="84" t="s">
+      <c r="A8" s="81" t="s">
         <v>226</v>
       </c>
-      <c r="B8" s="177" t="s">
+      <c r="B8" s="139" t="s">
         <v>234</v>
       </c>
-      <c r="C8" s="88">
-        <v>3</v>
-      </c>
-      <c r="D8" s="88">
-        <v>1</v>
-      </c>
-      <c r="E8" s="88">
-        <v>3</v>
-      </c>
-      <c r="F8" s="88">
-        <v>3</v>
-      </c>
-      <c r="G8" s="89">
+      <c r="C8" s="85">
+        <v>3</v>
+      </c>
+      <c r="D8" s="85">
+        <v>1</v>
+      </c>
+      <c r="E8" s="85">
+        <v>3</v>
+      </c>
+      <c r="F8" s="85">
+        <v>3</v>
+      </c>
+      <c r="G8" s="86">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="H8" s="90">
+      <c r="H8" s="87">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="I8" s="91">
+      <c r="I8" s="88">
         <f t="shared" si="2"/>
         <v>0.33333333333333331</v>
       </c>
@@ -31827,33 +31847,33 @@
       </c>
     </row>
     <row r="9" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="84" t="s">
+      <c r="A9" s="81" t="s">
         <v>226</v>
       </c>
-      <c r="B9" s="177" t="s">
+      <c r="B9" s="139" t="s">
         <v>235</v>
       </c>
-      <c r="C9" s="88">
-        <v>3</v>
-      </c>
-      <c r="D9" s="88">
-        <v>1</v>
-      </c>
-      <c r="E9" s="88">
-        <v>4</v>
-      </c>
-      <c r="F9" s="88">
-        <v>3</v>
-      </c>
-      <c r="G9" s="89">
+      <c r="C9" s="85">
+        <v>3</v>
+      </c>
+      <c r="D9" s="85">
+        <v>1</v>
+      </c>
+      <c r="E9" s="85">
+        <v>4</v>
+      </c>
+      <c r="F9" s="85">
+        <v>3</v>
+      </c>
+      <c r="G9" s="86">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="H9" s="90">
+      <c r="H9" s="87">
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
-      <c r="I9" s="91">
+      <c r="I9" s="88">
         <f t="shared" si="2"/>
         <v>0.25</v>
       </c>
@@ -31862,33 +31882,33 @@
       </c>
     </row>
     <row r="10" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="84" t="s">
+      <c r="A10" s="81" t="s">
         <v>230</v>
       </c>
-      <c r="B10" s="177" t="s">
+      <c r="B10" s="139" t="s">
         <v>236</v>
       </c>
-      <c r="C10" s="88">
-        <v>3</v>
-      </c>
-      <c r="D10" s="88">
-        <v>1</v>
-      </c>
-      <c r="E10" s="88">
-        <v>4</v>
-      </c>
-      <c r="F10" s="88">
-        <v>4</v>
-      </c>
-      <c r="G10" s="89">
+      <c r="C10" s="85">
+        <v>3</v>
+      </c>
+      <c r="D10" s="85">
+        <v>1</v>
+      </c>
+      <c r="E10" s="85">
+        <v>4</v>
+      </c>
+      <c r="F10" s="85">
+        <v>4</v>
+      </c>
+      <c r="G10" s="86">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="H10" s="90">
+      <c r="H10" s="87">
         <f t="shared" si="1"/>
         <v>16</v>
       </c>
-      <c r="I10" s="91">
+      <c r="I10" s="88">
         <f t="shared" si="2"/>
         <v>0.1875</v>
       </c>
@@ -31932,54 +31952,54 @@
   </cols>
   <sheetData>
     <row r="39" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C39" s="92" t="s">
+      <c r="C39" s="89" t="s">
         <v>122</v>
       </c>
-      <c r="D39" s="92" t="s">
+      <c r="D39" s="89" t="s">
         <v>123</v>
       </c>
-      <c r="E39" s="93" t="s">
+      <c r="E39" s="90" t="s">
         <v>124</v>
       </c>
-      <c r="F39" s="94" t="s">
+      <c r="F39" s="91" t="s">
         <v>125</v>
       </c>
-      <c r="G39" s="94" t="s">
+      <c r="G39" s="91" t="s">
         <v>126</v>
       </c>
-      <c r="H39" s="94" t="s">
+      <c r="H39" s="91" t="s">
         <v>127</v>
       </c>
-      <c r="I39" s="94" t="s">
+      <c r="I39" s="91" t="s">
         <v>128</v>
       </c>
-      <c r="J39" s="94" t="s">
+      <c r="J39" s="91" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="40" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C40" s="95">
-        <v>0</v>
-      </c>
-      <c r="D40" s="95">
-        <v>0.9</v>
-      </c>
-      <c r="E40" s="96">
-        <v>3</v>
-      </c>
-      <c r="F40" s="95">
-        <v>0</v>
-      </c>
-      <c r="G40" s="95">
-        <v>1</v>
-      </c>
-      <c r="H40" s="95">
-        <v>2</v>
-      </c>
-      <c r="I40" s="95">
-        <v>3</v>
-      </c>
-      <c r="J40" s="95">
+      <c r="C40" s="92">
+        <v>0</v>
+      </c>
+      <c r="D40" s="92">
+        <v>0.9</v>
+      </c>
+      <c r="E40" s="93">
+        <v>3</v>
+      </c>
+      <c r="F40" s="92">
+        <v>0</v>
+      </c>
+      <c r="G40" s="92">
+        <v>1</v>
+      </c>
+      <c r="H40" s="92">
+        <v>2</v>
+      </c>
+      <c r="I40" s="92">
+        <v>3</v>
+      </c>
+      <c r="J40" s="92">
         <v>4</v>
       </c>
     </row>
@@ -32011,7 +32031,7 @@
       <c r="A1" s="73" t="s">
         <v>130</v>
       </c>
-      <c r="B1" s="85" t="s">
+      <c r="B1" s="82" t="s">
         <v>108</v>
       </c>
       <c r="C1" s="73" t="s">
@@ -32031,7 +32051,7 @@
       <c r="C2" s="76" t="s">
         <v>239</v>
       </c>
-      <c r="D2" s="97" t="s">
+      <c r="D2" s="94" t="s">
         <v>22</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout de l'atelier 3
</commit_message>
<xml_diff>
--- a/EBIOS_RM_Classeur.xlsx
+++ b/EBIOS_RM_Classeur.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fonda\Documents\1 - Portfolio\BACKUP\1 - Python script backup file tree\2 - Learning\4 - Cours\7 - Cours Cyber\TP2_EBIOS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{332F6E16-9D62-4B48-9FA5-028812EB880D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DCC64DB-1809-421C-B434-CAD43A0C291A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="992" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="15720" tabRatio="992" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Organisation" sheetId="1" r:id="rId1"/>
@@ -2976,9 +2976,6 @@
     <xf numFmtId="0" fontId="0" fillId="13" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="17" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="20" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="75"/>
     </xf>
@@ -3099,26 +3096,59 @@
     <xf numFmtId="0" fontId="0" fillId="21" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="15" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3147,17 +3177,32 @@
     <xf numFmtId="0" fontId="12" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="16" fillId="22" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="22" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="22" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="23" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="23" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="23" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="23" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -3177,59 +3222,14 @@
     <xf numFmtId="0" fontId="0" fillId="23" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="22" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="22" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="22" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="23" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="23" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="23" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -15810,7 +15810,7 @@
   <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="49.140625"/>
+    <col min="1" max="1" width="88.28515625" customWidth="1"/>
     <col min="2" max="2" width="43.5703125"/>
     <col min="3" max="5" width="10.5703125"/>
     <col min="6" max="6" width="12.85546875"/>
@@ -15826,42 +15826,42 @@
       </c>
     </row>
     <row r="2" spans="1:2" ht="180" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="76" t="s">
+      <c r="A2" s="80" t="s">
         <v>290</v>
       </c>
-      <c r="B2" s="95" t="s">
+      <c r="B2" s="183" t="s">
         <v>291</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="180" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="76" t="s">
+      <c r="A3" s="80" t="s">
         <v>292</v>
       </c>
-      <c r="B3" s="76" t="s">
+      <c r="B3" s="80" t="s">
         <v>293</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="180" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="76" t="s">
+      <c r="A4" s="80" t="s">
         <v>294</v>
       </c>
-      <c r="B4" s="76" t="s">
+      <c r="B4" s="80" t="s">
         <v>291</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="180" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="76" t="s">
+      <c r="A5" s="80" t="s">
         <v>548</v>
       </c>
-      <c r="B5" s="76" t="s">
+      <c r="B5" s="80" t="s">
         <v>291</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="180" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="76" t="s">
+      <c r="A6" s="80" t="s">
         <v>295</v>
       </c>
-      <c r="B6" s="76" t="s">
+      <c r="B6" s="80" t="s">
         <v>291</v>
       </c>
     </row>
@@ -15963,40 +15963,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="114" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="96" t="s">
+      <c r="A1" s="95" t="s">
         <v>134</v>
       </c>
-      <c r="B1" s="97" t="s">
+      <c r="B1" s="96" t="s">
         <v>135</v>
       </c>
-      <c r="C1" s="98" t="s">
+      <c r="C1" s="97" t="s">
         <v>135</v>
       </c>
-      <c r="D1" s="98" t="s">
+      <c r="D1" s="97" t="s">
         <v>136</v>
       </c>
-      <c r="E1" s="99" t="s">
+      <c r="E1" s="98" t="s">
         <v>137</v>
       </c>
-      <c r="F1" s="99" t="s">
+      <c r="F1" s="98" t="s">
         <v>108</v>
       </c>
-      <c r="G1" s="100" t="s">
+      <c r="G1" s="99" t="s">
         <v>138</v>
       </c>
-      <c r="H1" s="101" t="s">
+      <c r="H1" s="100" t="s">
         <v>139</v>
       </c>
-      <c r="I1" s="101" t="s">
+      <c r="I1" s="100" t="s">
         <v>140</v>
       </c>
-      <c r="J1" s="101" t="s">
+      <c r="J1" s="100" t="s">
         <v>14</v>
       </c>
-      <c r="K1" s="102" t="s">
+      <c r="K1" s="101" t="s">
         <v>141</v>
       </c>
-      <c r="L1" s="102" t="s">
+      <c r="L1" s="101" t="s">
         <v>142</v>
       </c>
     </row>
@@ -16010,7 +16010,7 @@
       <c r="C2" s="77" t="s">
         <v>71</v>
       </c>
-      <c r="D2" s="103" t="s">
+      <c r="D2" s="102" t="s">
         <v>144</v>
       </c>
       <c r="E2" s="75" t="s">
@@ -16034,7 +16034,7 @@
       <c r="K2" s="75" t="s">
         <v>146</v>
       </c>
-      <c r="L2" s="104">
+      <c r="L2" s="103">
         <v>3</v>
       </c>
     </row>
@@ -16048,7 +16048,7 @@
       <c r="C3" s="78" t="s">
         <v>66</v>
       </c>
-      <c r="D3" s="103" t="s">
+      <c r="D3" s="102" t="s">
         <v>144</v>
       </c>
       <c r="E3" s="75" t="s">
@@ -16072,7 +16072,7 @@
       <c r="K3" s="75" t="s">
         <v>148</v>
       </c>
-      <c r="L3" s="105">
+      <c r="L3" s="104">
         <v>2</v>
       </c>
     </row>
@@ -16086,7 +16086,7 @@
       <c r="C4" s="77" t="s">
         <v>71</v>
       </c>
-      <c r="D4" s="103" t="s">
+      <c r="D4" s="102" t="s">
         <v>144</v>
       </c>
       <c r="E4" s="75" t="s">
@@ -16110,7 +16110,7 @@
       <c r="K4" s="75" t="s">
         <v>150</v>
       </c>
-      <c r="L4" s="106">
+      <c r="L4" s="105">
         <v>3</v>
       </c>
     </row>
@@ -16124,7 +16124,7 @@
       <c r="C5" s="78" t="s">
         <v>66</v>
       </c>
-      <c r="D5" s="103" t="s">
+      <c r="D5" s="102" t="s">
         <v>144</v>
       </c>
       <c r="E5" s="75" t="s">
@@ -16148,7 +16148,7 @@
       <c r="K5" s="75" t="s">
         <v>153</v>
       </c>
-      <c r="L5" s="105">
+      <c r="L5" s="104">
         <v>3</v>
       </c>
     </row>
@@ -16162,7 +16162,7 @@
       <c r="C6" s="78" t="s">
         <v>66</v>
       </c>
-      <c r="D6" s="103" t="s">
+      <c r="D6" s="102" t="s">
         <v>144</v>
       </c>
       <c r="E6" s="75" t="s">
@@ -16186,7 +16186,7 @@
       <c r="K6" s="75" t="s">
         <v>155</v>
       </c>
-      <c r="L6" s="107">
+      <c r="L6" s="106">
         <v>3</v>
       </c>
     </row>
@@ -16238,781 +16238,784 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AE1A74E-732B-433E-B6F2-025A8E71D54D}">
+  <sheetPr>
+    <tabColor theme="2" tint="-0.499984740745262"/>
+  </sheetPr>
   <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6" style="125" customWidth="1"/>
-    <col min="2" max="2" width="13" style="125" customWidth="1"/>
-    <col min="3" max="3" width="60" style="125" customWidth="1"/>
-    <col min="4" max="4" width="12" style="125" customWidth="1"/>
-    <col min="5" max="5" width="24" style="125" customWidth="1"/>
-    <col min="6" max="6" width="11" style="125" customWidth="1"/>
-    <col min="7" max="7" width="17.7109375" style="125" customWidth="1"/>
-    <col min="8" max="8" width="12" style="125" customWidth="1"/>
-    <col min="9" max="9" width="16" style="125" customWidth="1"/>
-    <col min="10" max="10" width="34" style="125" customWidth="1"/>
-    <col min="11" max="11" width="9" style="125" customWidth="1"/>
-    <col min="12" max="12" width="11" style="125" customWidth="1"/>
-    <col min="13" max="16384" width="8.85546875" style="125"/>
+    <col min="1" max="1" width="6" style="124" customWidth="1"/>
+    <col min="2" max="2" width="13" style="124" customWidth="1"/>
+    <col min="3" max="3" width="60" style="124" customWidth="1"/>
+    <col min="4" max="4" width="12" style="124" customWidth="1"/>
+    <col min="5" max="5" width="24" style="124" customWidth="1"/>
+    <col min="6" max="6" width="11" style="124" customWidth="1"/>
+    <col min="7" max="7" width="17.7109375" style="124" customWidth="1"/>
+    <col min="8" max="8" width="12" style="124" customWidth="1"/>
+    <col min="9" max="9" width="16" style="124" customWidth="1"/>
+    <col min="10" max="10" width="34" style="124" customWidth="1"/>
+    <col min="11" max="11" width="9" style="124" customWidth="1"/>
+    <col min="12" max="12" width="11" style="124" customWidth="1"/>
+    <col min="13" max="16384" width="8.85546875" style="124"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="131" t="s">
+      <c r="A1" s="130" t="s">
         <v>314</v>
       </c>
-      <c r="B1" s="131" t="s">
+      <c r="B1" s="130" t="s">
         <v>315</v>
       </c>
-      <c r="C1" s="131" t="s">
+      <c r="C1" s="130" t="s">
         <v>316</v>
       </c>
-      <c r="D1" s="131" t="s">
+      <c r="D1" s="130" t="s">
         <v>317</v>
       </c>
-      <c r="E1" s="131" t="s">
+      <c r="E1" s="130" t="s">
         <v>318</v>
       </c>
-      <c r="F1" s="131" t="s">
+      <c r="F1" s="130" t="s">
         <v>319</v>
       </c>
-      <c r="G1" s="131" t="s">
+      <c r="G1" s="130" t="s">
         <v>320</v>
       </c>
-      <c r="H1" s="131" t="s">
+      <c r="H1" s="130" t="s">
         <v>321</v>
       </c>
-      <c r="I1" s="131" t="s">
+      <c r="I1" s="130" t="s">
         <v>322</v>
       </c>
-      <c r="J1" s="131" t="s">
+      <c r="J1" s="130" t="s">
         <v>323</v>
       </c>
-      <c r="K1" s="131" t="s">
+      <c r="K1" s="130" t="s">
         <v>110</v>
       </c>
-      <c r="L1" s="131" t="s">
+      <c r="L1" s="130" t="s">
         <v>324</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="132" t="s">
+      <c r="A2" s="131" t="s">
         <v>347</v>
       </c>
-      <c r="B2" s="132" t="s">
+      <c r="B2" s="131" t="s">
         <v>339</v>
       </c>
-      <c r="C2" s="132" t="s">
+      <c r="C2" s="131" t="s">
         <v>512</v>
       </c>
-      <c r="D2" s="132" t="s">
+      <c r="D2" s="131" t="s">
         <v>143</v>
       </c>
-      <c r="E2" s="132" t="s">
+      <c r="E2" s="131" t="s">
         <v>327</v>
       </c>
-      <c r="F2" s="132" t="s">
+      <c r="F2" s="131" t="s">
         <v>113</v>
       </c>
-      <c r="G2" s="132">
-        <v>3</v>
-      </c>
-      <c r="H2" s="132" t="s">
+      <c r="G2" s="131">
+        <v>3</v>
+      </c>
+      <c r="H2" s="131" t="s">
         <v>348</v>
       </c>
-      <c r="I2" s="132" t="s">
+      <c r="I2" s="131" t="s">
         <v>349</v>
       </c>
-      <c r="J2" s="132" t="s">
+      <c r="J2" s="131" t="s">
         <v>350</v>
       </c>
-      <c r="K2" s="132" t="s">
+      <c r="K2" s="131" t="s">
         <v>330</v>
       </c>
-      <c r="L2" s="132" t="s">
+      <c r="L2" s="131" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="132" t="s">
+      <c r="A3" s="131" t="s">
         <v>357</v>
       </c>
-      <c r="B3" s="132" t="s">
+      <c r="B3" s="131" t="s">
         <v>339</v>
       </c>
-      <c r="C3" s="132" t="s">
+      <c r="C3" s="131" t="s">
         <v>358</v>
       </c>
-      <c r="D3" s="132" t="s">
+      <c r="D3" s="131" t="s">
         <v>359</v>
       </c>
-      <c r="E3" s="132" t="s">
+      <c r="E3" s="131" t="s">
         <v>334</v>
       </c>
-      <c r="F3" s="132" t="s">
+      <c r="F3" s="131" t="s">
         <v>41</v>
       </c>
-      <c r="G3" s="132">
-        <v>3</v>
-      </c>
-      <c r="H3" s="132" t="s">
+      <c r="G3" s="131">
+        <v>3</v>
+      </c>
+      <c r="H3" s="131" t="s">
         <v>348</v>
       </c>
-      <c r="I3" s="132" t="s">
+      <c r="I3" s="131" t="s">
         <v>360</v>
       </c>
-      <c r="J3" s="132" t="s">
+      <c r="J3" s="131" t="s">
         <v>361</v>
       </c>
-      <c r="K3" s="132" t="s">
+      <c r="K3" s="131" t="s">
         <v>330</v>
       </c>
-      <c r="L3" s="132" t="s">
+      <c r="L3" s="131" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="132" t="s">
+      <c r="A4" s="131" t="s">
         <v>325</v>
       </c>
-      <c r="B4" s="132" t="s">
+      <c r="B4" s="131" t="s">
         <v>339</v>
       </c>
-      <c r="C4" s="132" t="s">
+      <c r="C4" s="131" t="s">
         <v>513</v>
       </c>
-      <c r="D4" s="132" t="s">
+      <c r="D4" s="131" t="s">
         <v>151</v>
       </c>
-      <c r="E4" s="132" t="s">
+      <c r="E4" s="131" t="s">
         <v>327</v>
       </c>
-      <c r="F4" s="132" t="s">
+      <c r="F4" s="131" t="s">
         <v>41</v>
       </c>
-      <c r="G4" s="132">
-        <v>1</v>
-      </c>
-      <c r="H4" s="132" t="s">
+      <c r="G4" s="131">
+        <v>1</v>
+      </c>
+      <c r="H4" s="131" t="s">
         <v>328</v>
       </c>
-      <c r="I4" s="132" t="s">
+      <c r="I4" s="131" t="s">
         <v>329</v>
       </c>
-      <c r="J4" s="132" t="s">
+      <c r="J4" s="131" t="s">
         <v>514</v>
       </c>
-      <c r="K4" s="132" t="s">
+      <c r="K4" s="131" t="s">
         <v>330</v>
       </c>
-      <c r="L4" s="132" t="s">
+      <c r="L4" s="131" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="132" t="s">
+      <c r="A5" s="131" t="s">
         <v>372</v>
       </c>
-      <c r="B5" s="132" t="s">
+      <c r="B5" s="131" t="s">
         <v>339</v>
       </c>
-      <c r="C5" s="132" t="s">
+      <c r="C5" s="131" t="s">
         <v>373</v>
       </c>
-      <c r="D5" s="132" t="s">
+      <c r="D5" s="131" t="s">
         <v>374</v>
       </c>
-      <c r="E5" s="132" t="s">
+      <c r="E5" s="131" t="s">
         <v>375</v>
       </c>
-      <c r="F5" s="132" t="s">
+      <c r="F5" s="131" t="s">
         <v>113</v>
       </c>
-      <c r="G5" s="132">
+      <c r="G5" s="131">
         <v>6</v>
       </c>
-      <c r="H5" s="132" t="s">
+      <c r="H5" s="131" t="s">
         <v>376</v>
       </c>
-      <c r="I5" s="132" t="s">
+      <c r="I5" s="131" t="s">
         <v>377</v>
       </c>
-      <c r="J5" s="132" t="s">
+      <c r="J5" s="131" t="s">
         <v>378</v>
       </c>
-      <c r="K5" s="132" t="s">
+      <c r="K5" s="131" t="s">
         <v>362</v>
       </c>
-      <c r="L5" s="132" t="s">
+      <c r="L5" s="131" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="132" t="s">
+      <c r="A6" s="131" t="s">
         <v>363</v>
       </c>
-      <c r="B6" s="132" t="s">
+      <c r="B6" s="131" t="s">
         <v>339</v>
       </c>
-      <c r="C6" s="132" t="s">
+      <c r="C6" s="131" t="s">
         <v>364</v>
       </c>
-      <c r="D6" s="132" t="s">
+      <c r="D6" s="131" t="s">
         <v>154</v>
       </c>
-      <c r="E6" s="132" t="s">
+      <c r="E6" s="131" t="s">
         <v>327</v>
       </c>
-      <c r="F6" s="132" t="s">
+      <c r="F6" s="131" t="s">
         <v>41</v>
       </c>
-      <c r="G6" s="132">
-        <v>3</v>
-      </c>
-      <c r="H6" s="132" t="s">
+      <c r="G6" s="131">
+        <v>3</v>
+      </c>
+      <c r="H6" s="131" t="s">
         <v>348</v>
       </c>
-      <c r="I6" s="132" t="s">
+      <c r="I6" s="131" t="s">
         <v>329</v>
       </c>
-      <c r="J6" s="132" t="s">
+      <c r="J6" s="131" t="s">
         <v>365</v>
       </c>
-      <c r="K6" s="132" t="s">
+      <c r="K6" s="131" t="s">
         <v>362</v>
       </c>
-      <c r="L6" s="132" t="s">
+      <c r="L6" s="131" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="132" t="s">
+      <c r="A7" s="131" t="s">
         <v>338</v>
       </c>
-      <c r="B7" s="132" t="s">
+      <c r="B7" s="131" t="s">
         <v>339</v>
       </c>
-      <c r="C7" s="132" t="s">
+      <c r="C7" s="131" t="s">
         <v>340</v>
       </c>
-      <c r="D7" s="132" t="s">
+      <c r="D7" s="131" t="s">
         <v>143</v>
       </c>
-      <c r="E7" s="132" t="s">
+      <c r="E7" s="131" t="s">
         <v>327</v>
       </c>
-      <c r="F7" s="132" t="s">
+      <c r="F7" s="131" t="s">
         <v>41</v>
       </c>
-      <c r="G7" s="132">
-        <v>2</v>
-      </c>
-      <c r="H7" s="132" t="s">
+      <c r="G7" s="131">
+        <v>2</v>
+      </c>
+      <c r="H7" s="131" t="s">
         <v>335</v>
       </c>
-      <c r="I7" s="132" t="s">
+      <c r="I7" s="131" t="s">
         <v>329</v>
       </c>
-      <c r="J7" s="132" t="s">
+      <c r="J7" s="131" t="s">
         <v>341</v>
       </c>
-      <c r="K7" s="132" t="s">
+      <c r="K7" s="131" t="s">
         <v>362</v>
       </c>
-      <c r="L7" s="132" t="s">
+      <c r="L7" s="131" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="132" t="s">
+      <c r="A8" s="131" t="s">
         <v>332</v>
       </c>
-      <c r="B8" s="132" t="s">
+      <c r="B8" s="131" t="s">
         <v>326</v>
       </c>
-      <c r="C8" s="132" t="s">
+      <c r="C8" s="131" t="s">
         <v>544</v>
       </c>
-      <c r="D8" s="132" t="s">
+      <c r="D8" s="131" t="s">
         <v>333</v>
       </c>
-      <c r="E8" s="132" t="s">
+      <c r="E8" s="131" t="s">
         <v>334</v>
       </c>
-      <c r="F8" s="132" t="s">
+      <c r="F8" s="131" t="s">
         <v>113</v>
       </c>
-      <c r="G8" s="132">
-        <v>2</v>
-      </c>
-      <c r="H8" s="132" t="s">
+      <c r="G8" s="131">
+        <v>2</v>
+      </c>
+      <c r="H8" s="131" t="s">
         <v>335</v>
       </c>
-      <c r="I8" s="132" t="s">
+      <c r="I8" s="131" t="s">
         <v>336</v>
       </c>
-      <c r="J8" s="132" t="s">
+      <c r="J8" s="131" t="s">
         <v>337</v>
       </c>
-      <c r="K8" s="132" t="s">
+      <c r="K8" s="131" t="s">
         <v>330</v>
       </c>
-      <c r="L8" s="132" t="s">
+      <c r="L8" s="131" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="132" t="s">
+      <c r="A9" s="131" t="s">
         <v>379</v>
       </c>
-      <c r="B9" s="132" t="s">
+      <c r="B9" s="131" t="s">
         <v>326</v>
       </c>
-      <c r="C9" s="132" t="s">
+      <c r="C9" s="131" t="s">
         <v>380</v>
       </c>
-      <c r="D9" s="132" t="s">
+      <c r="D9" s="131" t="s">
         <v>381</v>
       </c>
-      <c r="E9" s="132" t="s">
+      <c r="E9" s="131" t="s">
         <v>382</v>
       </c>
-      <c r="F9" s="132" t="s">
+      <c r="F9" s="131" t="s">
         <v>383</v>
       </c>
-      <c r="G9" s="132">
+      <c r="G9" s="131">
         <v>6</v>
       </c>
-      <c r="H9" s="132" t="s">
+      <c r="H9" s="131" t="s">
         <v>376</v>
       </c>
-      <c r="I9" s="132" t="s">
+      <c r="I9" s="131" t="s">
         <v>384</v>
       </c>
-      <c r="J9" s="132" t="s">
+      <c r="J9" s="131" t="s">
         <v>385</v>
       </c>
-      <c r="K9" s="132" t="s">
+      <c r="K9" s="131" t="s">
         <v>330</v>
       </c>
-      <c r="L9" s="132" t="s">
+      <c r="L9" s="131" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="132" t="s">
+      <c r="A10" s="131" t="s">
         <v>342</v>
       </c>
-      <c r="B10" s="132" t="s">
+      <c r="B10" s="131" t="s">
         <v>326</v>
       </c>
-      <c r="C10" s="132" t="s">
+      <c r="C10" s="131" t="s">
         <v>343</v>
       </c>
-      <c r="D10" s="132" t="s">
+      <c r="D10" s="131" t="s">
         <v>154</v>
       </c>
-      <c r="E10" s="132" t="s">
+      <c r="E10" s="131" t="s">
         <v>344</v>
       </c>
-      <c r="F10" s="132" t="s">
+      <c r="F10" s="131" t="s">
         <v>41</v>
       </c>
-      <c r="G10" s="132">
-        <v>2</v>
-      </c>
-      <c r="H10" s="132" t="s">
+      <c r="G10" s="131">
+        <v>2</v>
+      </c>
+      <c r="H10" s="131" t="s">
         <v>335</v>
       </c>
-      <c r="I10" s="132" t="s">
+      <c r="I10" s="131" t="s">
         <v>345</v>
       </c>
-      <c r="J10" s="132" t="s">
+      <c r="J10" s="131" t="s">
         <v>346</v>
       </c>
-      <c r="K10" s="132" t="s">
+      <c r="K10" s="131" t="s">
         <v>330</v>
       </c>
-      <c r="L10" s="132" t="s">
+      <c r="L10" s="131" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="132" t="s">
+      <c r="A11" s="131" t="s">
         <v>515</v>
       </c>
-      <c r="B11" s="132" t="s">
+      <c r="B11" s="131" t="s">
         <v>326</v>
       </c>
-      <c r="C11" s="132" t="s">
+      <c r="C11" s="131" t="s">
         <v>516</v>
       </c>
-      <c r="D11" s="132" t="s">
+      <c r="D11" s="131" t="s">
         <v>151</v>
       </c>
-      <c r="E11" s="132" t="s">
+      <c r="E11" s="131" t="s">
         <v>327</v>
       </c>
-      <c r="F11" s="132" t="s">
+      <c r="F11" s="131" t="s">
         <v>41</v>
       </c>
-      <c r="G11" s="132">
-        <v>1</v>
-      </c>
-      <c r="H11" s="132" t="s">
+      <c r="G11" s="131">
+        <v>1</v>
+      </c>
+      <c r="H11" s="131" t="s">
         <v>328</v>
       </c>
-      <c r="I11" s="132" t="s">
+      <c r="I11" s="131" t="s">
         <v>329</v>
       </c>
-      <c r="J11" s="132" t="s">
+      <c r="J11" s="131" t="s">
         <v>517</v>
       </c>
-      <c r="K11" s="132" t="s">
+      <c r="K11" s="131" t="s">
         <v>330</v>
       </c>
-      <c r="L11" s="132" t="s">
+      <c r="L11" s="131" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="132" t="s">
+      <c r="A12" s="131" t="s">
         <v>396</v>
       </c>
-      <c r="B12" s="132" t="s">
+      <c r="B12" s="131" t="s">
         <v>326</v>
       </c>
-      <c r="C12" s="132" t="s">
+      <c r="C12" s="131" t="s">
         <v>397</v>
       </c>
-      <c r="D12" s="132" t="s">
+      <c r="D12" s="131" t="s">
         <v>147</v>
       </c>
-      <c r="E12" s="132" t="s">
+      <c r="E12" s="131" t="s">
         <v>334</v>
       </c>
-      <c r="F12" s="132" t="s">
+      <c r="F12" s="131" t="s">
         <v>41</v>
       </c>
-      <c r="G12" s="132">
+      <c r="G12" s="131">
         <v>7</v>
       </c>
-      <c r="H12" s="132" t="s">
+      <c r="H12" s="131" t="s">
         <v>398</v>
       </c>
-      <c r="I12" s="132" t="s">
+      <c r="I12" s="131" t="s">
         <v>329</v>
       </c>
-      <c r="J12" s="132" t="s">
+      <c r="J12" s="131" t="s">
         <v>399</v>
       </c>
-      <c r="K12" s="132" t="s">
+      <c r="K12" s="131" t="s">
         <v>362</v>
       </c>
-      <c r="L12" s="132" t="s">
+      <c r="L12" s="131" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="132" t="s">
+      <c r="A13" s="131" t="s">
         <v>400</v>
       </c>
-      <c r="B13" s="132" t="s">
+      <c r="B13" s="131" t="s">
         <v>326</v>
       </c>
-      <c r="C13" s="132" t="s">
+      <c r="C13" s="131" t="s">
         <v>401</v>
       </c>
-      <c r="D13" s="132" t="s">
+      <c r="D13" s="131" t="s">
         <v>402</v>
       </c>
-      <c r="E13" s="132" t="s">
+      <c r="E13" s="131" t="s">
         <v>403</v>
       </c>
-      <c r="F13" s="132" t="s">
+      <c r="F13" s="131" t="s">
         <v>383</v>
       </c>
-      <c r="G13" s="132">
+      <c r="G13" s="131">
         <v>9</v>
       </c>
-      <c r="H13" s="132" t="s">
+      <c r="H13" s="131" t="s">
         <v>404</v>
       </c>
-      <c r="I13" s="132" t="s">
+      <c r="I13" s="131" t="s">
         <v>405</v>
       </c>
-      <c r="J13" s="132" t="s">
+      <c r="J13" s="131" t="s">
         <v>406</v>
       </c>
-      <c r="K13" s="132" t="s">
+      <c r="K13" s="131" t="s">
         <v>362</v>
       </c>
-      <c r="L13" s="132" t="s">
+      <c r="L13" s="131" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="132" t="s">
+      <c r="A14" s="131" t="s">
         <v>518</v>
       </c>
-      <c r="B14" s="132" t="s">
+      <c r="B14" s="131" t="s">
         <v>326</v>
       </c>
-      <c r="C14" s="132" t="s">
+      <c r="C14" s="131" t="s">
         <v>519</v>
       </c>
-      <c r="D14" s="132" t="s">
+      <c r="D14" s="131" t="s">
         <v>149</v>
       </c>
-      <c r="E14" s="132" t="s">
+      <c r="E14" s="131" t="s">
         <v>334</v>
       </c>
-      <c r="F14" s="132" t="s">
+      <c r="F14" s="131" t="s">
         <v>41</v>
       </c>
-      <c r="G14" s="132">
-        <v>2</v>
-      </c>
-      <c r="H14" s="132" t="s">
+      <c r="G14" s="131">
+        <v>2</v>
+      </c>
+      <c r="H14" s="131" t="s">
         <v>335</v>
       </c>
-      <c r="I14" s="132" t="s">
+      <c r="I14" s="131" t="s">
         <v>329</v>
       </c>
-      <c r="J14" s="132" t="s">
+      <c r="J14" s="131" t="s">
         <v>520</v>
       </c>
-      <c r="K14" s="132" t="s">
+      <c r="K14" s="131" t="s">
         <v>362</v>
       </c>
-      <c r="L14" s="132" t="s">
+      <c r="L14" s="131" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="132" t="s">
+      <c r="A15" s="131" t="s">
         <v>366</v>
       </c>
-      <c r="B15" s="132" t="s">
+      <c r="B15" s="131" t="s">
         <v>367</v>
       </c>
-      <c r="C15" s="132" t="s">
+      <c r="C15" s="131" t="s">
         <v>368</v>
       </c>
-      <c r="D15" s="132" t="s">
+      <c r="D15" s="131" t="s">
         <v>149</v>
       </c>
-      <c r="E15" s="132" t="s">
+      <c r="E15" s="131" t="s">
         <v>334</v>
       </c>
-      <c r="F15" s="132" t="s">
+      <c r="F15" s="131" t="s">
         <v>113</v>
       </c>
-      <c r="G15" s="132">
-        <v>4</v>
-      </c>
-      <c r="H15" s="132" t="s">
+      <c r="G15" s="131">
+        <v>4</v>
+      </c>
+      <c r="H15" s="131" t="s">
         <v>369</v>
       </c>
-      <c r="I15" s="132" t="s">
+      <c r="I15" s="131" t="s">
         <v>370</v>
       </c>
-      <c r="J15" s="132" t="s">
+      <c r="J15" s="131" t="s">
         <v>371</v>
       </c>
-      <c r="K15" s="132" t="s">
+      <c r="K15" s="131" t="s">
         <v>330</v>
       </c>
-      <c r="L15" s="132" t="s">
+      <c r="L15" s="131" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="132" t="s">
+      <c r="A16" s="131" t="s">
         <v>407</v>
       </c>
-      <c r="B16" s="132" t="s">
+      <c r="B16" s="131" t="s">
         <v>367</v>
       </c>
-      <c r="C16" s="132" t="s">
+      <c r="C16" s="131" t="s">
         <v>408</v>
       </c>
-      <c r="D16" s="132" t="s">
+      <c r="D16" s="131" t="s">
         <v>402</v>
       </c>
-      <c r="E16" s="132" t="s">
+      <c r="E16" s="131" t="s">
         <v>334</v>
       </c>
-      <c r="F16" s="132" t="s">
+      <c r="F16" s="131" t="s">
         <v>383</v>
       </c>
-      <c r="G16" s="132">
+      <c r="G16" s="131">
         <v>9</v>
       </c>
-      <c r="H16" s="132" t="s">
+      <c r="H16" s="131" t="s">
         <v>404</v>
       </c>
-      <c r="I16" s="132" t="s">
+      <c r="I16" s="131" t="s">
         <v>409</v>
       </c>
-      <c r="J16" s="132" t="s">
+      <c r="J16" s="131" t="s">
         <v>410</v>
       </c>
-      <c r="K16" s="132" t="s">
+      <c r="K16" s="131" t="s">
         <v>362</v>
       </c>
-      <c r="L16" s="132" t="s">
+      <c r="L16" s="131" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="132" t="s">
+      <c r="A17" s="131" t="s">
         <v>386</v>
       </c>
-      <c r="B17" s="132" t="s">
+      <c r="B17" s="131" t="s">
         <v>367</v>
       </c>
-      <c r="C17" s="132" t="s">
+      <c r="C17" s="131" t="s">
         <v>387</v>
       </c>
-      <c r="D17" s="132" t="s">
+      <c r="D17" s="131" t="s">
         <v>154</v>
       </c>
-      <c r="E17" s="132" t="s">
+      <c r="E17" s="131" t="s">
         <v>334</v>
       </c>
-      <c r="F17" s="132" t="s">
+      <c r="F17" s="131" t="s">
         <v>113</v>
       </c>
-      <c r="G17" s="132">
+      <c r="G17" s="131">
         <v>6</v>
       </c>
-      <c r="H17" s="132" t="s">
+      <c r="H17" s="131" t="s">
         <v>376</v>
       </c>
-      <c r="I17" s="132" t="s">
+      <c r="I17" s="131" t="s">
         <v>388</v>
       </c>
-      <c r="J17" s="132" t="s">
+      <c r="J17" s="131" t="s">
         <v>389</v>
       </c>
-      <c r="K17" s="132" t="s">
+      <c r="K17" s="131" t="s">
         <v>390</v>
       </c>
-      <c r="L17" s="132" t="s">
+      <c r="L17" s="131" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="18" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="132" t="s">
+      <c r="A18" s="131" t="s">
         <v>351</v>
       </c>
-      <c r="B18" s="132" t="s">
+      <c r="B18" s="131" t="s">
         <v>352</v>
       </c>
-      <c r="C18" s="132" t="s">
+      <c r="C18" s="131" t="s">
         <v>353</v>
       </c>
-      <c r="D18" s="132" t="s">
+      <c r="D18" s="131" t="s">
         <v>354</v>
       </c>
-      <c r="E18" s="132" t="s">
+      <c r="E18" s="131" t="s">
         <v>334</v>
       </c>
-      <c r="F18" s="132" t="s">
+      <c r="F18" s="131" t="s">
         <v>113</v>
       </c>
-      <c r="G18" s="132">
-        <v>3</v>
-      </c>
-      <c r="H18" s="132" t="s">
+      <c r="G18" s="131">
+        <v>3</v>
+      </c>
+      <c r="H18" s="131" t="s">
         <v>348</v>
       </c>
-      <c r="I18" s="132" t="s">
+      <c r="I18" s="131" t="s">
         <v>355</v>
       </c>
-      <c r="J18" s="132" t="s">
+      <c r="J18" s="131" t="s">
         <v>356</v>
       </c>
-      <c r="K18" s="132" t="s">
+      <c r="K18" s="131" t="s">
         <v>330</v>
       </c>
-      <c r="L18" s="132" t="s">
+      <c r="L18" s="131" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="19" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="132" t="s">
+      <c r="A19" s="131" t="s">
         <v>411</v>
       </c>
-      <c r="B19" s="132" t="s">
+      <c r="B19" s="131" t="s">
         <v>352</v>
       </c>
-      <c r="C19" s="132" t="s">
+      <c r="C19" s="131" t="s">
         <v>412</v>
       </c>
-      <c r="D19" s="132" t="s">
+      <c r="D19" s="131" t="s">
         <v>354</v>
       </c>
-      <c r="E19" s="132" t="s">
+      <c r="E19" s="131" t="s">
         <v>375</v>
       </c>
-      <c r="F19" s="132" t="s">
+      <c r="F19" s="131" t="s">
         <v>383</v>
       </c>
-      <c r="G19" s="132">
+      <c r="G19" s="131">
         <v>12</v>
       </c>
-      <c r="H19" s="132" t="s">
+      <c r="H19" s="131" t="s">
         <v>413</v>
       </c>
-      <c r="I19" s="132" t="s">
+      <c r="I19" s="131" t="s">
         <v>414</v>
       </c>
-      <c r="J19" s="132" t="s">
+      <c r="J19" s="131" t="s">
         <v>415</v>
       </c>
-      <c r="K19" s="132" t="s">
+      <c r="K19" s="131" t="s">
         <v>362</v>
       </c>
-      <c r="L19" s="132" t="s">
+      <c r="L19" s="131" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="132" t="s">
+      <c r="A20" s="131" t="s">
         <v>391</v>
       </c>
-      <c r="B20" s="132" t="s">
+      <c r="B20" s="131" t="s">
         <v>352</v>
       </c>
-      <c r="C20" s="132" t="s">
+      <c r="C20" s="131" t="s">
         <v>392</v>
       </c>
-      <c r="D20" s="132" t="s">
+      <c r="D20" s="131" t="s">
         <v>393</v>
       </c>
-      <c r="E20" s="132" t="s">
+      <c r="E20" s="131" t="s">
         <v>327</v>
       </c>
-      <c r="F20" s="132" t="s">
+      <c r="F20" s="131" t="s">
         <v>41</v>
       </c>
-      <c r="G20" s="132">
+      <c r="G20" s="131">
         <v>6</v>
       </c>
-      <c r="H20" s="132" t="s">
+      <c r="H20" s="131" t="s">
         <v>376</v>
       </c>
-      <c r="I20" s="132" t="s">
+      <c r="I20" s="131" t="s">
         <v>394</v>
       </c>
-      <c r="J20" s="132" t="s">
+      <c r="J20" s="131" t="s">
         <v>395</v>
       </c>
-      <c r="K20" s="132" t="s">
+      <c r="K20" s="131" t="s">
         <v>390</v>
       </c>
-      <c r="L20" s="132" t="s">
+      <c r="L20" s="131" t="s">
         <v>331</v>
       </c>
     </row>
@@ -17023,202 +17026,205 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8153D206-9F5E-4049-A83B-1BF60BFA436A}">
+  <sheetPr>
+    <tabColor theme="6" tint="-0.499984740745262"/>
+  </sheetPr>
   <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8" style="125" customWidth="1"/>
-    <col min="2" max="2" width="10" style="125" customWidth="1"/>
-    <col min="3" max="3" width="13" style="125" customWidth="1"/>
-    <col min="4" max="4" width="12" style="125" customWidth="1"/>
-    <col min="5" max="5" width="34" style="125" customWidth="1"/>
-    <col min="6" max="6" width="11" style="125" customWidth="1"/>
-    <col min="7" max="7" width="14" style="125" customWidth="1"/>
-    <col min="8" max="8" width="13" style="125" customWidth="1"/>
-    <col min="9" max="9" width="40" style="125" customWidth="1"/>
-    <col min="10" max="16384" width="8.85546875" style="125"/>
+    <col min="1" max="1" width="8" style="124" customWidth="1"/>
+    <col min="2" max="2" width="10" style="124" customWidth="1"/>
+    <col min="3" max="3" width="13" style="124" customWidth="1"/>
+    <col min="4" max="4" width="12" style="124" customWidth="1"/>
+    <col min="5" max="5" width="34" style="124" customWidth="1"/>
+    <col min="6" max="6" width="11" style="124" customWidth="1"/>
+    <col min="7" max="7" width="14" style="124" customWidth="1"/>
+    <col min="8" max="8" width="13" style="124" customWidth="1"/>
+    <col min="9" max="9" width="40" style="124" customWidth="1"/>
+    <col min="10" max="16384" width="8.85546875" style="124"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="124" t="s">
+      <c r="A1" s="123" t="s">
         <v>135</v>
       </c>
-      <c r="B1" s="124" t="s">
+      <c r="B1" s="123" t="s">
         <v>416</v>
       </c>
-      <c r="C1" s="124" t="s">
+      <c r="C1" s="123" t="s">
         <v>417</v>
       </c>
-      <c r="D1" s="124" t="s">
+      <c r="D1" s="123" t="s">
         <v>418</v>
       </c>
-      <c r="E1" s="124" t="s">
+      <c r="E1" s="123" t="s">
         <v>419</v>
       </c>
-      <c r="F1" s="124" t="s">
+      <c r="F1" s="123" t="s">
         <v>420</v>
       </c>
-      <c r="G1" s="124" t="s">
+      <c r="G1" s="123" t="s">
         <v>421</v>
       </c>
-      <c r="H1" s="124" t="s">
+      <c r="H1" s="123" t="s">
         <v>422</v>
       </c>
-      <c r="I1" s="124" t="s">
+      <c r="I1" s="123" t="s">
         <v>423</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="126" t="s">
+      <c r="A2" s="125" t="s">
         <v>143</v>
       </c>
-      <c r="B2" s="126" t="s">
+      <c r="B2" s="125" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="126" t="s">
+      <c r="C2" s="125" t="s">
         <v>424</v>
       </c>
-      <c r="D2" s="128" t="s">
+      <c r="D2" s="127" t="s">
         <v>71</v>
       </c>
-      <c r="E2" s="127" t="s">
+      <c r="E2" s="126" t="s">
         <v>425</v>
       </c>
-      <c r="F2" s="126" t="s">
+      <c r="F2" s="125" t="s">
         <v>38</v>
       </c>
-      <c r="G2" s="126" t="s">
+      <c r="G2" s="125" t="s">
         <v>426</v>
       </c>
-      <c r="H2" s="129" t="s">
+      <c r="H2" s="128" t="s">
         <v>66</v>
       </c>
-      <c r="I2" s="127" t="s">
+      <c r="I2" s="126" t="s">
         <v>545</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="126" t="s">
+      <c r="A3" s="125" t="s">
         <v>147</v>
       </c>
-      <c r="B3" s="126" t="s">
+      <c r="B3" s="125" t="s">
         <v>38</v>
       </c>
-      <c r="C3" s="126" t="s">
+      <c r="C3" s="125" t="s">
         <v>426</v>
       </c>
-      <c r="D3" s="129" t="s">
+      <c r="D3" s="128" t="s">
         <v>66</v>
       </c>
-      <c r="E3" s="127" t="s">
+      <c r="E3" s="126" t="s">
         <v>427</v>
       </c>
-      <c r="F3" s="126" t="s">
+      <c r="F3" s="125" t="s">
         <v>38</v>
       </c>
-      <c r="G3" s="126" t="s">
+      <c r="G3" s="125" t="s">
         <v>428</v>
       </c>
-      <c r="H3" s="130" t="s">
+      <c r="H3" s="129" t="s">
         <v>53</v>
       </c>
-      <c r="I3" s="127" t="s">
+      <c r="I3" s="126" t="s">
         <v>546</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="126" t="s">
+      <c r="A4" s="125" t="s">
         <v>149</v>
       </c>
-      <c r="B4" s="126" t="s">
+      <c r="B4" s="125" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="126" t="s">
+      <c r="C4" s="125" t="s">
         <v>424</v>
       </c>
-      <c r="D4" s="128" t="s">
+      <c r="D4" s="127" t="s">
         <v>71</v>
       </c>
-      <c r="E4" s="127" t="s">
+      <c r="E4" s="126" t="s">
         <v>521</v>
       </c>
-      <c r="F4" s="126" t="s">
+      <c r="F4" s="125" t="s">
         <v>38</v>
       </c>
-      <c r="G4" s="126" t="s">
+      <c r="G4" s="125" t="s">
         <v>426</v>
       </c>
-      <c r="H4" s="129" t="s">
+      <c r="H4" s="128" t="s">
         <v>66</v>
       </c>
-      <c r="I4" s="127" t="s">
+      <c r="I4" s="126" t="s">
         <v>545</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="126" t="s">
+      <c r="A5" s="125" t="s">
         <v>151</v>
       </c>
-      <c r="B5" s="126" t="s">
+      <c r="B5" s="125" t="s">
         <v>38</v>
       </c>
-      <c r="C5" s="126" t="s">
+      <c r="C5" s="125" t="s">
         <v>424</v>
       </c>
-      <c r="D5" s="129" t="s">
+      <c r="D5" s="128" t="s">
         <v>66</v>
       </c>
-      <c r="E5" s="127" t="s">
+      <c r="E5" s="126" t="s">
         <v>522</v>
       </c>
-      <c r="F5" s="126" t="s">
+      <c r="F5" s="125" t="s">
         <v>38</v>
       </c>
-      <c r="G5" s="126" t="s">
+      <c r="G5" s="125" t="s">
         <v>426</v>
       </c>
-      <c r="H5" s="129" t="s">
+      <c r="H5" s="128" t="s">
         <v>66</v>
       </c>
-      <c r="I5" s="127" t="s">
+      <c r="I5" s="126" t="s">
         <v>545</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="126" t="s">
+      <c r="A6" s="125" t="s">
         <v>154</v>
       </c>
-      <c r="B6" s="126" t="s">
+      <c r="B6" s="125" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="126" t="s">
+      <c r="C6" s="125" t="s">
         <v>424</v>
       </c>
-      <c r="D6" s="129" t="s">
+      <c r="D6" s="128" t="s">
         <v>66</v>
       </c>
-      <c r="E6" s="127" t="s">
+      <c r="E6" s="126" t="s">
         <v>429</v>
       </c>
-      <c r="F6" s="126" t="s">
+      <c r="F6" s="125" t="s">
         <v>38</v>
       </c>
-      <c r="G6" s="126" t="s">
+      <c r="G6" s="125" t="s">
         <v>426</v>
       </c>
-      <c r="H6" s="129" t="s">
+      <c r="H6" s="128" t="s">
         <v>66</v>
       </c>
-      <c r="I6" s="127" t="s">
+      <c r="I6" s="126" t="s">
         <v>545</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="125" t="s">
+      <c r="A8" s="124" t="s">
         <v>523</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="125" t="s">
+      <c r="A9" s="124" t="s">
         <v>524</v>
       </c>
     </row>
@@ -17229,192 +17235,195 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{390F47A4-D957-42BB-AF94-65A9499B46AB}">
+  <sheetPr>
+    <tabColor theme="8"/>
+  </sheetPr>
   <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="55" style="121" customWidth="1"/>
-    <col min="2" max="2" width="12" style="121" customWidth="1"/>
-    <col min="3" max="3" width="20" style="121" customWidth="1"/>
-    <col min="4" max="4" width="14" style="121" customWidth="1"/>
-    <col min="5" max="5" width="24" style="121" customWidth="1"/>
-    <col min="6" max="16384" width="8.85546875" style="121"/>
+    <col min="1" max="1" width="55" style="120" customWidth="1"/>
+    <col min="2" max="2" width="12" style="120" customWidth="1"/>
+    <col min="3" max="3" width="20" style="120" customWidth="1"/>
+    <col min="4" max="4" width="14" style="120" customWidth="1"/>
+    <col min="5" max="5" width="24" style="120" customWidth="1"/>
+    <col min="6" max="16384" width="8.85546875" style="120"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="120" t="s">
+      <c r="A1" s="119" t="s">
         <v>430</v>
       </c>
-      <c r="B1" s="120" t="s">
+      <c r="B1" s="119" t="s">
         <v>431</v>
       </c>
-      <c r="C1" s="120" t="s">
+      <c r="C1" s="119" t="s">
         <v>432</v>
       </c>
-      <c r="D1" s="120" t="s">
+      <c r="D1" s="119" t="s">
         <v>433</v>
       </c>
-      <c r="E1" s="120" t="s">
+      <c r="E1" s="119" t="s">
         <v>434</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="122" t="s">
+      <c r="A2" s="121" t="s">
         <v>435</v>
       </c>
-      <c r="B2" s="122" t="s">
+      <c r="B2" s="121" t="s">
         <v>332</v>
       </c>
-      <c r="C2" s="122" t="s">
+      <c r="C2" s="121" t="s">
         <v>436</v>
       </c>
-      <c r="D2" s="122" t="s">
+      <c r="D2" s="121" t="s">
         <v>437</v>
       </c>
-      <c r="E2" s="122" t="s">
+      <c r="E2" s="121" t="s">
         <v>438</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="122" t="s">
+      <c r="A3" s="121" t="s">
         <v>439</v>
       </c>
-      <c r="B3" s="122" t="s">
+      <c r="B3" s="121" t="s">
         <v>351</v>
       </c>
-      <c r="C3" s="122" t="s">
+      <c r="C3" s="121" t="s">
         <v>440</v>
       </c>
-      <c r="D3" s="122" t="s">
+      <c r="D3" s="121" t="s">
         <v>441</v>
       </c>
-      <c r="E3" s="122" t="s">
+      <c r="E3" s="121" t="s">
         <v>438</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="122" t="s">
+      <c r="A4" s="121" t="s">
         <v>442</v>
       </c>
-      <c r="B4" s="122" t="s">
+      <c r="B4" s="121" t="s">
         <v>357</v>
       </c>
-      <c r="C4" s="122" t="s">
+      <c r="C4" s="121" t="s">
         <v>443</v>
       </c>
-      <c r="D4" s="122" t="s">
+      <c r="D4" s="121" t="s">
         <v>444</v>
       </c>
-      <c r="E4" s="122" t="s">
+      <c r="E4" s="121" t="s">
         <v>438</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="122" t="s">
+      <c r="A5" s="121" t="s">
         <v>445</v>
       </c>
-      <c r="B5" s="122" t="s">
+      <c r="B5" s="121" t="s">
         <v>379</v>
       </c>
-      <c r="C5" s="122" t="s">
+      <c r="C5" s="121" t="s">
         <v>446</v>
       </c>
-      <c r="D5" s="122" t="s">
+      <c r="D5" s="121" t="s">
         <v>437</v>
       </c>
-      <c r="E5" s="122" t="s">
+      <c r="E5" s="121" t="s">
         <v>447</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="122" t="s">
+      <c r="A6" s="121" t="s">
         <v>448</v>
       </c>
-      <c r="B6" s="122" t="s">
+      <c r="B6" s="121" t="s">
         <v>449</v>
       </c>
-      <c r="C6" s="122" t="s">
+      <c r="C6" s="121" t="s">
         <v>450</v>
       </c>
-      <c r="D6" s="122" t="s">
+      <c r="D6" s="121" t="s">
         <v>441</v>
       </c>
-      <c r="E6" s="122" t="s">
+      <c r="E6" s="121" t="s">
         <v>451</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="122" t="s">
+      <c r="A7" s="121" t="s">
         <v>525</v>
       </c>
-      <c r="B7" s="122" t="s">
+      <c r="B7" s="121" t="s">
         <v>515</v>
       </c>
-      <c r="C7" s="122" t="s">
+      <c r="C7" s="121" t="s">
         <v>436</v>
       </c>
-      <c r="D7" s="122" t="s">
+      <c r="D7" s="121" t="s">
         <v>437</v>
       </c>
-      <c r="E7" s="122" t="s">
+      <c r="E7" s="121" t="s">
         <v>452</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="122" t="s">
+      <c r="A8" s="121" t="s">
         <v>526</v>
       </c>
-      <c r="B8" s="122" t="s">
+      <c r="B8" s="121" t="s">
         <v>325</v>
       </c>
-      <c r="C8" s="122" t="s">
+      <c r="C8" s="121" t="s">
         <v>436</v>
       </c>
-      <c r="D8" s="122" t="s">
+      <c r="D8" s="121" t="s">
         <v>527</v>
       </c>
-      <c r="E8" s="122" t="s">
+      <c r="E8" s="121" t="s">
         <v>452</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="122" t="s">
+      <c r="A9" s="121" t="s">
         <v>528</v>
       </c>
-      <c r="B9" s="122" t="s">
+      <c r="B9" s="121" t="s">
         <v>518</v>
       </c>
-      <c r="C9" s="122" t="s">
+      <c r="C9" s="121" t="s">
         <v>529</v>
       </c>
-      <c r="D9" s="122" t="s">
+      <c r="D9" s="121" t="s">
         <v>437</v>
       </c>
-      <c r="E9" s="122" t="s">
+      <c r="E9" s="121" t="s">
         <v>438</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="123" t="s">
+      <c r="A11" s="122" t="s">
         <v>453</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="121" t="s">
+      <c r="A12" s="120" t="s">
         <v>454</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="121" t="s">
+      <c r="A13" s="120" t="s">
         <v>455</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="121" t="s">
+      <c r="A14" s="120" t="s">
         <v>456</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="121" t="s">
+      <c r="A15" s="120" t="s">
         <v>457</v>
       </c>
     </row>
@@ -17457,9 +17466,9 @@
       <c r="H1" t="s">
         <v>129</v>
       </c>
-      <c r="J1" s="108"/>
-      <c r="K1" s="108"/>
-      <c r="L1" s="109"/>
+      <c r="J1" s="107"/>
+      <c r="K1" s="107"/>
+      <c r="L1" s="108"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2">
@@ -17494,7 +17503,7 @@
         <f>'Atelier 3 - Carto PP'!J40</f>
         <v>4</v>
       </c>
-      <c r="L2" s="110"/>
+      <c r="L2" s="109"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3">
@@ -29708,34 +29717,34 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A2" s="156" t="s">
+      <c r="A2" s="149" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="156"/>
-      <c r="C2" s="156"/>
-      <c r="D2" s="156"/>
-      <c r="E2" s="156"/>
-      <c r="G2" s="157" t="s">
+      <c r="B2" s="149"/>
+      <c r="C2" s="149"/>
+      <c r="D2" s="149"/>
+      <c r="E2" s="149"/>
+      <c r="G2" s="150" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="157"/>
-      <c r="J2" s="158" t="s">
+      <c r="H2" s="150"/>
+      <c r="J2" s="151" t="s">
         <v>15</v>
       </c>
-      <c r="K2" s="158"/>
-      <c r="L2" s="158"/>
-      <c r="M2" s="158"/>
-      <c r="N2" s="158"/>
-      <c r="O2" s="158"/>
-      <c r="P2" s="158"/>
-      <c r="Q2" s="158"/>
-      <c r="Z2" s="156" t="s">
+      <c r="K2" s="151"/>
+      <c r="L2" s="151"/>
+      <c r="M2" s="151"/>
+      <c r="N2" s="151"/>
+      <c r="O2" s="151"/>
+      <c r="P2" s="151"/>
+      <c r="Q2" s="151"/>
+      <c r="Z2" s="149" t="s">
         <v>16</v>
       </c>
-      <c r="AA2" s="156"/>
-      <c r="AB2" s="156"/>
-      <c r="AC2" s="156"/>
-      <c r="AD2" s="156"/>
+      <c r="AA2" s="149"/>
+      <c r="AB2" s="149"/>
+      <c r="AC2" s="149"/>
+      <c r="AD2" s="149"/>
     </row>
     <row r="3" spans="1:38" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
@@ -29753,7 +29762,7 @@
       <c r="E3" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="F3" s="144" t="s">
+      <c r="F3" s="152" t="s">
         <v>13</v>
       </c>
       <c r="G3" s="15" t="s">
@@ -29762,32 +29771,32 @@
       <c r="H3" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="I3" s="144" t="s">
+      <c r="I3" s="152" t="s">
         <v>14</v>
       </c>
       <c r="J3" s="17">
         <v>1</v>
       </c>
-      <c r="K3" s="146" t="s">
+      <c r="K3" s="153" t="s">
         <v>24</v>
       </c>
-      <c r="L3" s="146"/>
-      <c r="M3" s="146"/>
-      <c r="N3" s="146"/>
-      <c r="O3" s="146"/>
-      <c r="P3" s="146"/>
-      <c r="Q3" s="146"/>
-      <c r="R3" s="144" t="s">
+      <c r="L3" s="153"/>
+      <c r="M3" s="153"/>
+      <c r="N3" s="153"/>
+      <c r="O3" s="153"/>
+      <c r="P3" s="153"/>
+      <c r="Q3" s="153"/>
+      <c r="R3" s="152" t="s">
         <v>15</v>
       </c>
       <c r="T3" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="U3" s="159" t="s">
+      <c r="U3" s="154" t="s">
         <v>25</v>
       </c>
-      <c r="V3" s="159"/>
-      <c r="Y3" s="144" t="s">
+      <c r="V3" s="154"/>
+      <c r="Y3" s="152" t="s">
         <v>26</v>
       </c>
       <c r="Z3" s="19" t="s">
@@ -29805,17 +29814,17 @@
       <c r="AD3" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="AE3" s="144" t="s">
+      <c r="AE3" s="152" t="s">
         <v>31</v>
       </c>
       <c r="AG3" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="AH3" s="145" t="s">
+      <c r="AH3" s="156" t="s">
         <v>32</v>
       </c>
-      <c r="AI3" s="145"/>
-      <c r="AL3" s="144" t="s">
+      <c r="AI3" s="156"/>
+      <c r="AL3" s="152" t="s">
         <v>33</v>
       </c>
     </row>
@@ -29835,35 +29844,35 @@
       <c r="E4" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="F4" s="144"/>
+      <c r="F4" s="152"/>
       <c r="G4" s="26" t="s">
         <v>38</v>
       </c>
       <c r="H4" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="I4" s="144"/>
+      <c r="I4" s="152"/>
       <c r="J4" s="27">
         <v>2</v>
       </c>
-      <c r="K4" s="146" t="s">
+      <c r="K4" s="153" t="s">
         <v>40</v>
       </c>
-      <c r="L4" s="146"/>
-      <c r="M4" s="146"/>
-      <c r="N4" s="146"/>
-      <c r="O4" s="146"/>
-      <c r="P4" s="146"/>
-      <c r="Q4" s="146"/>
-      <c r="R4" s="144"/>
+      <c r="L4" s="153"/>
+      <c r="M4" s="153"/>
+      <c r="N4" s="153"/>
+      <c r="O4" s="153"/>
+      <c r="P4" s="153"/>
+      <c r="Q4" s="153"/>
+      <c r="R4" s="152"/>
       <c r="T4" s="28">
         <v>1</v>
       </c>
-      <c r="U4" s="147" t="s">
+      <c r="U4" s="157" t="s">
         <v>41</v>
       </c>
-      <c r="V4" s="147"/>
-      <c r="Y4" s="144"/>
+      <c r="V4" s="157"/>
+      <c r="Y4" s="152"/>
       <c r="Z4" s="29">
         <v>1</v>
       </c>
@@ -29879,15 +29888,15 @@
       <c r="AD4" s="31" t="s">
         <v>45</v>
       </c>
-      <c r="AE4" s="144"/>
+      <c r="AE4" s="152"/>
       <c r="AG4" s="32">
         <v>1</v>
       </c>
-      <c r="AH4" s="148" t="s">
+      <c r="AH4" s="158" t="s">
         <v>41</v>
       </c>
-      <c r="AI4" s="148"/>
-      <c r="AL4" s="144"/>
+      <c r="AI4" s="158"/>
+      <c r="AL4" s="152"/>
     </row>
     <row r="5" spans="1:38" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="33">
@@ -29905,35 +29914,35 @@
       <c r="E5" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="F5" s="144"/>
+      <c r="F5" s="152"/>
       <c r="G5" s="34" t="s">
         <v>50</v>
       </c>
       <c r="H5" s="35" t="s">
         <v>51</v>
       </c>
-      <c r="I5" s="144"/>
+      <c r="I5" s="152"/>
       <c r="J5" s="36">
         <v>3</v>
       </c>
-      <c r="K5" s="146" t="s">
+      <c r="K5" s="153" t="s">
         <v>52</v>
       </c>
-      <c r="L5" s="146"/>
-      <c r="M5" s="146"/>
-      <c r="N5" s="146"/>
-      <c r="O5" s="146"/>
-      <c r="P5" s="146"/>
-      <c r="Q5" s="146"/>
-      <c r="R5" s="144"/>
+      <c r="L5" s="153"/>
+      <c r="M5" s="153"/>
+      <c r="N5" s="153"/>
+      <c r="O5" s="153"/>
+      <c r="P5" s="153"/>
+      <c r="Q5" s="153"/>
+      <c r="R5" s="152"/>
       <c r="T5" s="37">
         <v>2</v>
       </c>
-      <c r="U5" s="149" t="s">
+      <c r="U5" s="159" t="s">
         <v>53</v>
       </c>
-      <c r="V5" s="149"/>
-      <c r="Y5" s="144"/>
+      <c r="V5" s="159"/>
+      <c r="Y5" s="152"/>
       <c r="Z5" s="38">
         <v>2</v>
       </c>
@@ -29949,15 +29958,15 @@
       <c r="AD5" s="31" t="s">
         <v>57</v>
       </c>
-      <c r="AE5" s="144"/>
+      <c r="AE5" s="152"/>
       <c r="AG5" s="39">
         <v>2</v>
       </c>
-      <c r="AH5" s="150" t="s">
+      <c r="AH5" s="160" t="s">
         <v>58</v>
       </c>
-      <c r="AI5" s="150"/>
-      <c r="AL5" s="144"/>
+      <c r="AI5" s="160"/>
+      <c r="AL5" s="152"/>
     </row>
     <row r="6" spans="1:38" ht="57" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="40">
@@ -29975,35 +29984,35 @@
       <c r="E6" s="25" t="s">
         <v>62</v>
       </c>
-      <c r="F6" s="144"/>
+      <c r="F6" s="152"/>
       <c r="G6" s="41" t="s">
         <v>63</v>
       </c>
       <c r="H6" s="35" t="s">
         <v>64</v>
       </c>
-      <c r="I6" s="144"/>
+      <c r="I6" s="152"/>
       <c r="J6" s="42">
         <v>4</v>
       </c>
-      <c r="K6" s="146" t="s">
+      <c r="K6" s="153" t="s">
         <v>65</v>
       </c>
-      <c r="L6" s="146"/>
-      <c r="M6" s="146"/>
-      <c r="N6" s="146"/>
-      <c r="O6" s="146"/>
-      <c r="P6" s="146"/>
-      <c r="Q6" s="146"/>
-      <c r="R6" s="144"/>
+      <c r="L6" s="153"/>
+      <c r="M6" s="153"/>
+      <c r="N6" s="153"/>
+      <c r="O6" s="153"/>
+      <c r="P6" s="153"/>
+      <c r="Q6" s="153"/>
+      <c r="R6" s="152"/>
       <c r="T6" s="43">
         <v>3</v>
       </c>
-      <c r="U6" s="151" t="s">
+      <c r="U6" s="161" t="s">
         <v>66</v>
       </c>
-      <c r="V6" s="151"/>
-      <c r="Y6" s="144"/>
+      <c r="V6" s="161"/>
+      <c r="Y6" s="152"/>
       <c r="Z6" s="44">
         <v>3</v>
       </c>
@@ -30019,15 +30028,15 @@
       <c r="AD6" s="31" t="s">
         <v>70</v>
       </c>
-      <c r="AE6" s="144"/>
+      <c r="AE6" s="152"/>
       <c r="AG6" s="45">
         <v>3</v>
       </c>
-      <c r="AH6" s="152" t="s">
+      <c r="AH6" s="162" t="s">
         <v>71</v>
       </c>
-      <c r="AI6" s="152"/>
-      <c r="AL6" s="144"/>
+      <c r="AI6" s="162"/>
+      <c r="AL6" s="152"/>
     </row>
     <row r="7" spans="1:38" ht="71.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="46">
@@ -30045,27 +30054,27 @@
       <c r="E7" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="F7" s="144"/>
-      <c r="G7" s="142"/>
-      <c r="H7" s="142"/>
-      <c r="I7" s="144"/>
-      <c r="J7" s="153"/>
-      <c r="K7" s="153"/>
-      <c r="L7" s="153"/>
-      <c r="M7" s="153"/>
-      <c r="N7" s="153"/>
-      <c r="O7" s="153"/>
-      <c r="P7" s="153"/>
-      <c r="Q7" s="153"/>
-      <c r="R7" s="144"/>
+      <c r="F7" s="152"/>
+      <c r="G7" s="155"/>
+      <c r="H7" s="155"/>
+      <c r="I7" s="152"/>
+      <c r="J7" s="163"/>
+      <c r="K7" s="163"/>
+      <c r="L7" s="163"/>
+      <c r="M7" s="163"/>
+      <c r="N7" s="163"/>
+      <c r="O7" s="163"/>
+      <c r="P7" s="163"/>
+      <c r="Q7" s="163"/>
+      <c r="R7" s="152"/>
       <c r="T7" s="48">
         <v>4</v>
       </c>
-      <c r="U7" s="154" t="s">
+      <c r="U7" s="164" t="s">
         <v>71</v>
       </c>
-      <c r="V7" s="154"/>
-      <c r="Y7" s="144"/>
+      <c r="V7" s="164"/>
+      <c r="Y7" s="152"/>
       <c r="Z7" s="49">
         <v>4</v>
       </c>
@@ -30081,49 +30090,49 @@
       <c r="AD7" s="31" t="s">
         <v>79</v>
       </c>
-      <c r="AE7" s="144"/>
+      <c r="AE7" s="152"/>
       <c r="AG7" s="51"/>
-      <c r="AH7" s="155"/>
-      <c r="AI7" s="155"/>
-      <c r="AL7" s="144"/>
+      <c r="AH7" s="165"/>
+      <c r="AI7" s="165"/>
+      <c r="AL7" s="152"/>
     </row>
     <row r="8" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A8" s="142"/>
-      <c r="B8" s="142"/>
-      <c r="C8" s="142"/>
-      <c r="D8" s="142"/>
-      <c r="E8" s="142"/>
-      <c r="Z8" s="142"/>
-      <c r="AA8" s="142"/>
-      <c r="AB8" s="142"/>
-      <c r="AC8" s="142"/>
-      <c r="AD8" s="142"/>
+      <c r="A8" s="155"/>
+      <c r="B8" s="155"/>
+      <c r="C8" s="155"/>
+      <c r="D8" s="155"/>
+      <c r="E8" s="155"/>
+      <c r="Z8" s="155"/>
+      <c r="AA8" s="155"/>
+      <c r="AB8" s="155"/>
+      <c r="AC8" s="155"/>
+      <c r="AD8" s="155"/>
     </row>
     <row r="10" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="L10" s="140" t="s">
+      <c r="L10" s="166" t="s">
         <v>15</v>
       </c>
-      <c r="M10" s="140"/>
-      <c r="N10" s="143" t="s">
+      <c r="M10" s="166"/>
+      <c r="N10" s="168" t="s">
         <v>80</v>
       </c>
-      <c r="O10" s="143"/>
-      <c r="P10" s="143"/>
-      <c r="Q10" s="143"/>
-      <c r="S10" s="140" t="s">
+      <c r="O10" s="168"/>
+      <c r="P10" s="168"/>
+      <c r="Q10" s="168"/>
+      <c r="S10" s="166" t="s">
         <v>25</v>
       </c>
-      <c r="T10" s="140"/>
-      <c r="U10" s="143" t="s">
+      <c r="T10" s="166"/>
+      <c r="U10" s="168" t="s">
         <v>15</v>
       </c>
-      <c r="V10" s="143"/>
-      <c r="W10" s="143"/>
-      <c r="X10" s="143"/>
-      <c r="AF10" s="140" t="s">
+      <c r="V10" s="168"/>
+      <c r="W10" s="168"/>
+      <c r="X10" s="168"/>
+      <c r="AF10" s="166" t="s">
         <v>81</v>
       </c>
-      <c r="AG10" s="140"/>
+      <c r="AG10" s="166"/>
       <c r="AH10" s="52" t="s">
         <v>82</v>
       </c>
@@ -30131,8 +30140,8 @@
       <c r="AJ10" s="53"/>
     </row>
     <row r="11" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="L11" s="140"/>
-      <c r="M11" s="140"/>
+      <c r="L11" s="166"/>
+      <c r="M11" s="166"/>
       <c r="N11" s="54">
         <v>1</v>
       </c>
@@ -30145,8 +30154,8 @@
       <c r="Q11" s="57">
         <v>4</v>
       </c>
-      <c r="S11" s="140"/>
-      <c r="T11" s="140"/>
+      <c r="S11" s="166"/>
+      <c r="T11" s="166"/>
       <c r="U11" s="58">
         <v>1</v>
       </c>
@@ -30159,8 +30168,8 @@
       <c r="X11" s="58">
         <v>4</v>
       </c>
-      <c r="AF11" s="140"/>
-      <c r="AG11" s="140"/>
+      <c r="AF11" s="166"/>
+      <c r="AG11" s="166"/>
       <c r="AH11" s="58" t="s">
         <v>83</v>
       </c>
@@ -30172,7 +30181,7 @@
       </c>
     </row>
     <row r="12" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="L12" s="141" t="s">
+      <c r="L12" s="167" t="s">
         <v>86</v>
       </c>
       <c r="M12" s="54">
@@ -30190,7 +30199,7 @@
       <c r="Q12" s="61">
         <v>3</v>
       </c>
-      <c r="S12" s="141" t="s">
+      <c r="S12" s="167" t="s">
         <v>14</v>
       </c>
       <c r="T12" s="58">
@@ -30225,7 +30234,7 @@
       </c>
     </row>
     <row r="13" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="L13" s="141"/>
+      <c r="L13" s="167"/>
       <c r="M13" s="55">
         <v>2</v>
       </c>
@@ -30241,7 +30250,7 @@
       <c r="Q13" s="61">
         <v>3</v>
       </c>
-      <c r="S13" s="141"/>
+      <c r="S13" s="167"/>
       <c r="T13" s="58">
         <v>2</v>
       </c>
@@ -30272,7 +30281,7 @@
       </c>
     </row>
     <row r="14" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="L14" s="141"/>
+      <c r="L14" s="167"/>
       <c r="M14" s="56">
         <v>3</v>
       </c>
@@ -30288,7 +30297,7 @@
       <c r="Q14" s="70">
         <v>4</v>
       </c>
-      <c r="S14" s="141"/>
+      <c r="S14" s="167"/>
       <c r="T14" s="58">
         <v>3</v>
       </c>
@@ -30319,7 +30328,7 @@
       </c>
     </row>
     <row r="15" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="L15" s="141"/>
+      <c r="L15" s="167"/>
       <c r="M15" s="57">
         <v>4</v>
       </c>
@@ -30335,7 +30344,7 @@
       <c r="Q15" s="70">
         <v>4</v>
       </c>
-      <c r="S15" s="141"/>
+      <c r="S15" s="167"/>
       <c r="T15" s="58">
         <v>4</v>
       </c>
@@ -30354,17 +30363,15 @@
     </row>
   </sheetData>
   <mergeCells count="35">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="J2:Q2"/>
-    <mergeCell ref="Z2:AD2"/>
-    <mergeCell ref="F3:F7"/>
-    <mergeCell ref="I3:I7"/>
-    <mergeCell ref="K3:Q3"/>
-    <mergeCell ref="R3:R7"/>
-    <mergeCell ref="U3:V3"/>
-    <mergeCell ref="Y3:Y7"/>
-    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="AF10:AG11"/>
+    <mergeCell ref="L12:L15"/>
+    <mergeCell ref="S12:S15"/>
+    <mergeCell ref="A8:E8"/>
+    <mergeCell ref="Z8:AD8"/>
+    <mergeCell ref="L10:M11"/>
+    <mergeCell ref="N10:Q10"/>
+    <mergeCell ref="S10:T11"/>
+    <mergeCell ref="U10:X10"/>
     <mergeCell ref="AE3:AE7"/>
     <mergeCell ref="AH3:AI3"/>
     <mergeCell ref="AL3:AL7"/>
@@ -30380,15 +30387,17 @@
     <mergeCell ref="J7:Q7"/>
     <mergeCell ref="U7:V7"/>
     <mergeCell ref="AH7:AI7"/>
-    <mergeCell ref="AF10:AG11"/>
-    <mergeCell ref="L12:L15"/>
-    <mergeCell ref="S12:S15"/>
-    <mergeCell ref="A8:E8"/>
-    <mergeCell ref="Z8:AD8"/>
-    <mergeCell ref="L10:M11"/>
-    <mergeCell ref="N10:Q10"/>
-    <mergeCell ref="S10:T11"/>
-    <mergeCell ref="U10:X10"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="J2:Q2"/>
+    <mergeCell ref="Z2:AD2"/>
+    <mergeCell ref="F3:F7"/>
+    <mergeCell ref="I3:I7"/>
+    <mergeCell ref="K3:Q3"/>
+    <mergeCell ref="R3:R7"/>
+    <mergeCell ref="U3:V3"/>
+    <mergeCell ref="Y3:Y7"/>
+    <mergeCell ref="G7:H7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup paperSize="0" scale="0" firstPageNumber="0" orientation="portrait" usePrinterDefaults="0" horizontalDpi="0" verticalDpi="0" copies="0"/>
@@ -30421,246 +30430,246 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="27" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="136" t="s">
+      <c r="A1" s="135" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="166" t="s">
+      <c r="B1" s="169" t="s">
         <v>160</v>
       </c>
-      <c r="C1" s="167"/>
-      <c r="D1" s="167"/>
-      <c r="E1" s="167"/>
-      <c r="F1" s="167"/>
-      <c r="G1" s="167"/>
-      <c r="H1" s="167"/>
-      <c r="I1" s="167"/>
-      <c r="J1" s="167"/>
-      <c r="K1" s="167"/>
-      <c r="L1" s="167"/>
-      <c r="M1" s="167"/>
-      <c r="N1" s="168"/>
+      <c r="C1" s="170"/>
+      <c r="D1" s="170"/>
+      <c r="E1" s="170"/>
+      <c r="F1" s="170"/>
+      <c r="G1" s="170"/>
+      <c r="H1" s="170"/>
+      <c r="I1" s="170"/>
+      <c r="J1" s="170"/>
+      <c r="K1" s="170"/>
+      <c r="L1" s="170"/>
+      <c r="M1" s="170"/>
+      <c r="N1" s="171"/>
     </row>
     <row r="2" spans="1:14" ht="36.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="136" t="s">
+      <c r="A2" s="135" t="s">
         <v>89</v>
       </c>
-      <c r="B2" s="169" t="s">
+      <c r="B2" s="172" t="s">
         <v>161</v>
       </c>
-      <c r="C2" s="170"/>
-      <c r="D2" s="170"/>
-      <c r="E2" s="170"/>
-      <c r="F2" s="171"/>
-      <c r="G2" s="137" t="s">
+      <c r="C2" s="173"/>
+      <c r="D2" s="173"/>
+      <c r="E2" s="173"/>
+      <c r="F2" s="174"/>
+      <c r="G2" s="136" t="s">
         <v>162</v>
       </c>
-      <c r="H2" s="169" t="s">
+      <c r="H2" s="172" t="s">
         <v>163</v>
       </c>
-      <c r="I2" s="171"/>
-      <c r="J2" s="169" t="s">
+      <c r="I2" s="174"/>
+      <c r="J2" s="172" t="s">
         <v>164</v>
       </c>
-      <c r="K2" s="170"/>
-      <c r="L2" s="171"/>
-      <c r="M2" s="169" t="s">
+      <c r="K2" s="173"/>
+      <c r="L2" s="174"/>
+      <c r="M2" s="172" t="s">
         <v>165</v>
       </c>
-      <c r="N2" s="170"/>
+      <c r="N2" s="173"/>
     </row>
     <row r="3" spans="1:14" ht="50.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="136" t="s">
+      <c r="A3" s="135" t="s">
         <v>90</v>
       </c>
-      <c r="B3" s="160" t="s">
+      <c r="B3" s="175" t="s">
         <v>91</v>
       </c>
-      <c r="C3" s="161"/>
-      <c r="D3" s="161"/>
-      <c r="E3" s="161"/>
-      <c r="F3" s="165"/>
+      <c r="C3" s="176"/>
+      <c r="D3" s="176"/>
+      <c r="E3" s="176"/>
+      <c r="F3" s="180"/>
       <c r="G3" s="72" t="s">
         <v>92</v>
       </c>
-      <c r="H3" s="160" t="s">
+      <c r="H3" s="175" t="s">
         <v>91</v>
       </c>
-      <c r="I3" s="165"/>
-      <c r="J3" s="160" t="s">
+      <c r="I3" s="180"/>
+      <c r="J3" s="175" t="s">
         <v>92</v>
       </c>
-      <c r="K3" s="161"/>
-      <c r="L3" s="165"/>
-      <c r="M3" s="160" t="s">
+      <c r="K3" s="176"/>
+      <c r="L3" s="180"/>
+      <c r="M3" s="175" t="s">
         <v>93</v>
       </c>
-      <c r="N3" s="161"/>
+      <c r="N3" s="176"/>
     </row>
     <row r="4" spans="1:14" ht="124.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="136" t="s">
+      <c r="A4" s="135" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="160" t="s">
+      <c r="B4" s="175" t="s">
         <v>166</v>
       </c>
-      <c r="C4" s="161"/>
-      <c r="D4" s="161"/>
-      <c r="E4" s="161"/>
-      <c r="F4" s="165"/>
+      <c r="C4" s="176"/>
+      <c r="D4" s="176"/>
+      <c r="E4" s="176"/>
+      <c r="F4" s="180"/>
       <c r="G4" s="72" t="s">
         <v>167</v>
       </c>
-      <c r="H4" s="160" t="s">
+      <c r="H4" s="175" t="s">
         <v>168</v>
       </c>
-      <c r="I4" s="165"/>
-      <c r="J4" s="160" t="s">
+      <c r="I4" s="180"/>
+      <c r="J4" s="175" t="s">
         <v>169</v>
       </c>
-      <c r="K4" s="161"/>
-      <c r="L4" s="165"/>
-      <c r="M4" s="160" t="s">
+      <c r="K4" s="176"/>
+      <c r="L4" s="180"/>
+      <c r="M4" s="175" t="s">
         <v>170</v>
       </c>
-      <c r="N4" s="161"/>
+      <c r="N4" s="176"/>
     </row>
     <row r="5" spans="1:14" ht="30" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="136" t="s">
+      <c r="A5" s="135" t="s">
         <v>94</v>
       </c>
-      <c r="B5" s="160" t="s">
+      <c r="B5" s="175" t="s">
         <v>196</v>
       </c>
-      <c r="C5" s="161"/>
-      <c r="D5" s="161"/>
-      <c r="E5" s="161"/>
-      <c r="F5" s="161"/>
-      <c r="G5" s="161"/>
-      <c r="H5" s="161"/>
-      <c r="I5" s="161"/>
-      <c r="J5" s="161"/>
-      <c r="K5" s="161"/>
-      <c r="L5" s="161"/>
-      <c r="M5" s="161"/>
-      <c r="N5" s="161"/>
+      <c r="C5" s="176"/>
+      <c r="D5" s="176"/>
+      <c r="E5" s="176"/>
+      <c r="F5" s="176"/>
+      <c r="G5" s="176"/>
+      <c r="H5" s="176"/>
+      <c r="I5" s="176"/>
+      <c r="J5" s="176"/>
+      <c r="K5" s="176"/>
+      <c r="L5" s="176"/>
+      <c r="M5" s="176"/>
+      <c r="N5" s="176"/>
     </row>
     <row r="6" spans="1:14" ht="116.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="136" t="s">
+      <c r="A6" s="135" t="s">
         <v>95</v>
       </c>
-      <c r="B6" s="133" t="s">
+      <c r="B6" s="132" t="s">
         <v>171</v>
       </c>
-      <c r="C6" s="134" t="s">
+      <c r="C6" s="133" t="s">
         <v>172</v>
       </c>
-      <c r="D6" s="162" t="s">
+      <c r="D6" s="177" t="s">
         <v>173</v>
       </c>
-      <c r="E6" s="163"/>
-      <c r="F6" s="164"/>
-      <c r="G6" s="134" t="s">
+      <c r="E6" s="178"/>
+      <c r="F6" s="179"/>
+      <c r="G6" s="133" t="s">
         <v>174</v>
       </c>
-      <c r="H6" s="133" t="s">
+      <c r="H6" s="132" t="s">
         <v>175</v>
       </c>
-      <c r="I6" s="138" t="s">
+      <c r="I6" s="137" t="s">
         <v>176</v>
       </c>
-      <c r="J6" s="138" t="s">
+      <c r="J6" s="137" t="s">
         <v>177</v>
       </c>
-      <c r="K6" s="138" t="s">
+      <c r="K6" s="137" t="s">
         <v>178</v>
       </c>
-      <c r="L6" s="133" t="s">
+      <c r="L6" s="132" t="s">
         <v>179</v>
       </c>
-      <c r="M6" s="134" t="s">
+      <c r="M6" s="133" t="s">
         <v>180</v>
       </c>
-      <c r="N6" s="134" t="s">
+      <c r="N6" s="133" t="s">
         <v>181</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="114" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="136" t="s">
+      <c r="A7" s="135" t="s">
         <v>32</v>
       </c>
-      <c r="B7" s="133" t="s">
+      <c r="B7" s="132" t="s">
         <v>186</v>
       </c>
-      <c r="C7" s="134" t="s">
+      <c r="C7" s="133" t="s">
         <v>188</v>
       </c>
-      <c r="D7" s="162" t="s">
+      <c r="D7" s="177" t="s">
         <v>190</v>
       </c>
-      <c r="E7" s="163"/>
-      <c r="F7" s="164"/>
-      <c r="G7" s="134" t="s">
+      <c r="E7" s="178"/>
+      <c r="F7" s="179"/>
+      <c r="G7" s="133" t="s">
         <v>192</v>
       </c>
-      <c r="H7" s="133" t="s">
+      <c r="H7" s="132" t="s">
         <v>193</v>
       </c>
-      <c r="I7" s="138" t="s">
+      <c r="I7" s="137" t="s">
         <v>182</v>
       </c>
-      <c r="J7" s="138" t="s">
+      <c r="J7" s="137" t="s">
         <v>183</v>
       </c>
-      <c r="K7" s="135" t="s">
+      <c r="K7" s="134" t="s">
         <v>184</v>
       </c>
-      <c r="L7" s="133" t="s">
+      <c r="L7" s="132" t="s">
         <v>185</v>
       </c>
-      <c r="M7" s="134" t="s">
+      <c r="M7" s="133" t="s">
         <v>194</v>
       </c>
-      <c r="N7" s="134" t="s">
+      <c r="N7" s="133" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="61.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="136" t="s">
+      <c r="A8" s="135" t="s">
         <v>94</v>
       </c>
-      <c r="B8" s="133" t="s">
+      <c r="B8" s="132" t="s">
         <v>187</v>
       </c>
-      <c r="C8" s="134" t="s">
+      <c r="C8" s="133" t="s">
         <v>189</v>
       </c>
-      <c r="D8" s="162" t="s">
+      <c r="D8" s="177" t="s">
         <v>191</v>
       </c>
-      <c r="E8" s="163"/>
-      <c r="F8" s="164"/>
-      <c r="G8" s="134" t="s">
+      <c r="E8" s="178"/>
+      <c r="F8" s="179"/>
+      <c r="G8" s="133" t="s">
         <v>189</v>
       </c>
-      <c r="H8" s="133" t="s">
+      <c r="H8" s="132" t="s">
         <v>189</v>
       </c>
-      <c r="I8" s="138" t="s">
+      <c r="I8" s="137" t="s">
         <v>191</v>
       </c>
-      <c r="J8" s="138" t="s">
+      <c r="J8" s="137" t="s">
         <v>191</v>
       </c>
-      <c r="K8" s="133" t="s">
+      <c r="K8" s="132" t="s">
         <v>191</v>
       </c>
-      <c r="L8" s="133" t="s">
+      <c r="L8" s="132" t="s">
         <v>191</v>
       </c>
-      <c r="M8" s="134" t="s">
+      <c r="M8" s="133" t="s">
         <v>189</v>
       </c>
-      <c r="N8" s="134" t="s">
+      <c r="N8" s="133" t="s">
         <v>189</v>
       </c>
     </row>
@@ -30744,11 +30753,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="B1:N1"/>
-    <mergeCell ref="B2:F2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="J2:L2"/>
-    <mergeCell ref="M2:N2"/>
     <mergeCell ref="B5:N5"/>
     <mergeCell ref="D6:F6"/>
     <mergeCell ref="D7:F7"/>
@@ -30761,6 +30765,11 @@
     <mergeCell ref="H4:I4"/>
     <mergeCell ref="J4:L4"/>
     <mergeCell ref="M4:N4"/>
+    <mergeCell ref="B1:N1"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="M2:N2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
@@ -30793,31 +30802,31 @@
         <v>97</v>
       </c>
       <c r="D1" s="182"/>
-      <c r="E1" s="183"/>
-      <c r="F1" s="183"/>
+      <c r="E1" s="145"/>
+      <c r="F1" s="145"/>
     </row>
     <row r="2" spans="1:6" ht="42.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="175" t="s">
+      <c r="A2" s="139" t="s">
         <v>98</v>
       </c>
-      <c r="B2" s="175" t="s">
+      <c r="B2" s="139" t="s">
         <v>99</v>
       </c>
-      <c r="C2" s="175" t="s">
+      <c r="C2" s="139" t="s">
         <v>100</v>
       </c>
-      <c r="D2" s="175" t="s">
+      <c r="D2" s="139" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="175" t="s">
+      <c r="E2" s="139" t="s">
         <v>475</v>
       </c>
-      <c r="F2" s="175" t="s">
+      <c r="F2" s="139" t="s">
         <v>476</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="120" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="176" t="s">
+      <c r="A3" s="140" t="s">
         <v>161</v>
       </c>
       <c r="B3" s="80" t="s">
@@ -30826,18 +30835,18 @@
       <c r="C3" s="80" t="s">
         <v>490</v>
       </c>
-      <c r="D3" s="177" t="s">
+      <c r="D3" s="141" t="s">
         <v>38</v>
       </c>
-      <c r="E3" s="183" t="s">
+      <c r="E3" s="145" t="s">
         <v>477</v>
       </c>
-      <c r="F3" s="183" t="s">
+      <c r="F3" s="145" t="s">
         <v>478</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="176" t="s">
+      <c r="A4" s="140" t="s">
         <v>161</v>
       </c>
       <c r="B4" s="80" t="s">
@@ -30846,18 +30855,18 @@
       <c r="C4" s="80" t="s">
         <v>281</v>
       </c>
-      <c r="D4" s="177" t="s">
+      <c r="D4" s="141" t="s">
         <v>50</v>
       </c>
-      <c r="E4" s="183" t="s">
+      <c r="E4" s="145" t="s">
         <v>479</v>
       </c>
-      <c r="F4" s="183" t="s">
+      <c r="F4" s="145" t="s">
         <v>480</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="176" t="s">
+      <c r="A5" s="140" t="s">
         <v>162</v>
       </c>
       <c r="B5" s="80" t="s">
@@ -30866,18 +30875,18 @@
       <c r="C5" s="80" t="s">
         <v>283</v>
       </c>
-      <c r="D5" s="178" t="s">
+      <c r="D5" s="142" t="s">
         <v>38</v>
       </c>
-      <c r="E5" s="183" t="s">
+      <c r="E5" s="145" t="s">
         <v>481</v>
       </c>
-      <c r="F5" s="183" t="s">
+      <c r="F5" s="145" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="176" t="s">
+      <c r="A6" s="140" t="s">
         <v>163</v>
       </c>
       <c r="B6" s="80" t="s">
@@ -30886,18 +30895,18 @@
       <c r="C6" s="80" t="s">
         <v>285</v>
       </c>
-      <c r="D6" s="179" t="s">
+      <c r="D6" s="143" t="s">
         <v>50</v>
       </c>
-      <c r="E6" s="183" t="s">
+      <c r="E6" s="145" t="s">
         <v>483</v>
       </c>
-      <c r="F6" s="183" t="s">
+      <c r="F6" s="145" t="s">
         <v>484</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="176" t="s">
+      <c r="A7" s="140" t="s">
         <v>163</v>
       </c>
       <c r="B7" s="80" t="s">
@@ -30906,13 +30915,13 @@
       <c r="C7" s="80" t="s">
         <v>287</v>
       </c>
-      <c r="D7" s="180" t="s">
+      <c r="D7" s="144" t="s">
         <v>38</v>
       </c>
-      <c r="E7" s="183" t="s">
+      <c r="E7" s="145" t="s">
         <v>485</v>
       </c>
-      <c r="F7" s="183" t="s">
+      <c r="F7" s="145" t="s">
         <v>486</v>
       </c>
     </row>
@@ -30926,13 +30935,13 @@
       <c r="C8" s="80" t="s">
         <v>491</v>
       </c>
-      <c r="D8" s="179" t="s">
+      <c r="D8" s="143" t="s">
         <v>22</v>
       </c>
-      <c r="E8" s="183" t="s">
+      <c r="E8" s="145" t="s">
         <v>487</v>
       </c>
-      <c r="F8" s="183" t="s">
+      <c r="F8" s="145" t="s">
         <v>488</v>
       </c>
     </row>
@@ -30946,13 +30955,13 @@
       <c r="C9" s="80" t="s">
         <v>289</v>
       </c>
-      <c r="D9" s="179" t="s">
+      <c r="D9" s="143" t="s">
         <v>50</v>
       </c>
-      <c r="E9" s="183" t="s">
+      <c r="E9" s="145" t="s">
         <v>483</v>
       </c>
-      <c r="F9" s="183" t="s">
+      <c r="F9" s="145" t="s">
         <v>489</v>
       </c>
     </row>
@@ -30994,14 +31003,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="172" t="s">
+      <c r="A1" s="146" t="s">
         <v>96</v>
       </c>
-      <c r="B1" s="172"/>
-      <c r="C1" s="173" t="s">
+      <c r="B1" s="146"/>
+      <c r="C1" s="147" t="s">
         <v>97</v>
       </c>
-      <c r="D1" s="173"/>
+      <c r="D1" s="147"/>
     </row>
     <row r="2" spans="1:5" ht="42.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="73" t="s">
@@ -31021,223 +31030,223 @@
       </c>
     </row>
     <row r="3" spans="1:5" ht="79.900000000000006" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="111" t="s">
+      <c r="A3" s="110" t="s">
         <v>250</v>
       </c>
-      <c r="B3" s="112" t="s">
+      <c r="B3" s="111" t="s">
         <v>251</v>
       </c>
-      <c r="C3" s="112" t="s">
+      <c r="C3" s="111" t="s">
         <v>252</v>
       </c>
-      <c r="D3" s="112" t="s">
+      <c r="D3" s="111" t="s">
         <v>253</v>
       </c>
-      <c r="E3" s="113" t="s">
+      <c r="E3" s="112" t="s">
         <v>254</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="79.900000000000006" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="114" t="s">
+      <c r="A4" s="113" t="s">
         <v>250</v>
       </c>
-      <c r="B4" s="115" t="s">
+      <c r="B4" s="114" t="s">
         <v>251</v>
       </c>
-      <c r="C4" s="115" t="s">
+      <c r="C4" s="114" t="s">
         <v>252</v>
       </c>
-      <c r="D4" s="115" t="s">
+      <c r="D4" s="114" t="s">
         <v>255</v>
       </c>
-      <c r="E4" s="116" t="s">
+      <c r="E4" s="115" t="s">
         <v>256</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="79.900000000000006" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="114" t="s">
+      <c r="A5" s="113" t="s">
         <v>250</v>
       </c>
-      <c r="B5" s="115" t="s">
+      <c r="B5" s="114" t="s">
         <v>251</v>
       </c>
-      <c r="C5" s="115" t="s">
+      <c r="C5" s="114" t="s">
         <v>252</v>
       </c>
-      <c r="D5" s="115" t="s">
+      <c r="D5" s="114" t="s">
         <v>492</v>
       </c>
-      <c r="E5" s="116" t="s">
+      <c r="E5" s="115" t="s">
         <v>493</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="79.900000000000006" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="114" t="s">
+      <c r="A6" s="113" t="s">
         <v>250</v>
       </c>
-      <c r="B6" s="115" t="s">
+      <c r="B6" s="114" t="s">
         <v>251</v>
       </c>
-      <c r="C6" s="115" t="s">
+      <c r="C6" s="114" t="s">
         <v>252</v>
       </c>
-      <c r="D6" s="115" t="s">
+      <c r="D6" s="114" t="s">
         <v>257</v>
       </c>
-      <c r="E6" s="116" t="s">
+      <c r="E6" s="115" t="s">
         <v>258</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="79.900000000000006" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="114" t="s">
+      <c r="A7" s="113" t="s">
         <v>250</v>
       </c>
-      <c r="B7" s="115" t="s">
+      <c r="B7" s="114" t="s">
         <v>251</v>
       </c>
-      <c r="C7" s="115" t="s">
+      <c r="C7" s="114" t="s">
         <v>259</v>
       </c>
-      <c r="D7" s="115" t="s">
+      <c r="D7" s="114" t="s">
         <v>260</v>
       </c>
-      <c r="E7" s="116" t="s">
+      <c r="E7" s="115" t="s">
         <v>261</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="79.900000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="117" t="s">
+      <c r="A8" s="116" t="s">
         <v>250</v>
       </c>
-      <c r="B8" s="118" t="s">
+      <c r="B8" s="117" t="s">
         <v>251</v>
       </c>
-      <c r="C8" s="118" t="s">
+      <c r="C8" s="117" t="s">
         <v>262</v>
       </c>
-      <c r="D8" s="118" t="s">
+      <c r="D8" s="117" t="s">
         <v>263</v>
       </c>
-      <c r="E8" s="119" t="s">
+      <c r="E8" s="118" t="s">
         <v>494</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="79.900000000000006" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="117" t="s">
+      <c r="A9" s="116" t="s">
         <v>250</v>
       </c>
-      <c r="B9" s="118" t="s">
+      <c r="B9" s="117" t="s">
         <v>251</v>
       </c>
-      <c r="C9" s="118" t="s">
+      <c r="C9" s="117" t="s">
         <v>259</v>
       </c>
-      <c r="D9" s="118" t="s">
+      <c r="D9" s="117" t="s">
         <v>264</v>
       </c>
-      <c r="E9" s="119" t="s">
+      <c r="E9" s="118" t="s">
         <v>265</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="79.900000000000006" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="117" t="s">
+      <c r="A10" s="116" t="s">
         <v>250</v>
       </c>
-      <c r="B10" s="118" t="s">
+      <c r="B10" s="117" t="s">
         <v>251</v>
       </c>
-      <c r="C10" s="118" t="s">
+      <c r="C10" s="117" t="s">
         <v>252</v>
       </c>
-      <c r="D10" s="118" t="s">
+      <c r="D10" s="117" t="s">
         <v>495</v>
       </c>
-      <c r="E10" s="119" t="s">
+      <c r="E10" s="118" t="s">
         <v>496</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="79.900000000000006" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="117" t="s">
+      <c r="A11" s="116" t="s">
         <v>266</v>
       </c>
-      <c r="B11" s="118" t="s">
+      <c r="B11" s="117" t="s">
         <v>267</v>
       </c>
-      <c r="C11" s="118" t="s">
+      <c r="C11" s="117" t="s">
         <v>252</v>
       </c>
-      <c r="D11" s="118" t="s">
+      <c r="D11" s="117" t="s">
         <v>268</v>
       </c>
-      <c r="E11" s="119" t="s">
+      <c r="E11" s="118" t="s">
         <v>269</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="79.900000000000006" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="117" t="s">
+      <c r="A12" s="116" t="s">
         <v>266</v>
       </c>
-      <c r="B12" s="118" t="s">
+      <c r="B12" s="117" t="s">
         <v>270</v>
       </c>
-      <c r="C12" s="118" t="s">
+      <c r="C12" s="117" t="s">
         <v>271</v>
       </c>
-      <c r="D12" s="118" t="s">
+      <c r="D12" s="117" t="s">
         <v>530</v>
       </c>
-      <c r="E12" s="119" t="s">
+      <c r="E12" s="118" t="s">
         <v>272</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="79.900000000000006" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="117" t="s">
+      <c r="A13" s="116" t="s">
         <v>273</v>
       </c>
-      <c r="B13" s="118" t="s">
+      <c r="B13" s="117" t="s">
         <v>274</v>
       </c>
-      <c r="C13" s="118" t="s">
+      <c r="C13" s="117" t="s">
         <v>252</v>
       </c>
-      <c r="D13" s="118" t="s">
+      <c r="D13" s="117" t="s">
         <v>275</v>
       </c>
-      <c r="E13" s="119" t="s">
+      <c r="E13" s="118" t="s">
         <v>276</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="79.900000000000006" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="117" t="s">
+      <c r="A14" s="116" t="s">
         <v>273</v>
       </c>
-      <c r="B14" s="118" t="s">
+      <c r="B14" s="117" t="s">
         <v>277</v>
       </c>
-      <c r="C14" s="118" t="s">
+      <c r="C14" s="117" t="s">
         <v>262</v>
       </c>
-      <c r="D14" s="118" t="s">
+      <c r="D14" s="117" t="s">
         <v>278</v>
       </c>
-      <c r="E14" s="119" t="s">
+      <c r="E14" s="118" t="s">
         <v>279</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="79.900000000000006" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="117" t="s">
+      <c r="A15" s="116" t="s">
         <v>531</v>
       </c>
-      <c r="B15" s="118" t="s">
+      <c r="B15" s="117" t="s">
         <v>532</v>
       </c>
-      <c r="C15" s="118" t="s">
+      <c r="C15" s="117" t="s">
         <v>259</v>
       </c>
-      <c r="D15" s="118" t="s">
+      <c r="D15" s="117" t="s">
         <v>533</v>
       </c>
-      <c r="E15" s="119" t="s">
+      <c r="E15" s="118" t="s">
         <v>534</v>
       </c>
     </row>
@@ -31270,18 +31279,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="172" t="s">
+      <c r="A1" s="146" t="s">
         <v>96</v>
       </c>
-      <c r="B1" s="172"/>
-      <c r="C1" s="173" t="s">
+      <c r="B1" s="146"/>
+      <c r="C1" s="147" t="s">
         <v>97</v>
       </c>
-      <c r="D1" s="173"/>
-      <c r="E1" s="174" t="s">
+      <c r="D1" s="147"/>
+      <c r="E1" s="148" t="s">
         <v>106</v>
       </c>
-      <c r="F1" s="174"/>
+      <c r="F1" s="148"/>
     </row>
     <row r="2" spans="1:8" ht="42.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="73" t="s">
@@ -31605,7 +31614,7 @@
       <c r="A2" s="81" t="s">
         <v>224</v>
       </c>
-      <c r="B2" s="139" t="s">
+      <c r="B2" s="138" t="s">
         <v>225</v>
       </c>
       <c r="C2" s="85">
@@ -31640,7 +31649,7 @@
       <c r="A3" s="81" t="s">
         <v>226</v>
       </c>
-      <c r="B3" s="139" t="s">
+      <c r="B3" s="138" t="s">
         <v>227</v>
       </c>
       <c r="C3" s="85">
@@ -31675,7 +31684,7 @@
       <c r="A4" s="81" t="s">
         <v>226</v>
       </c>
-      <c r="B4" s="139" t="s">
+      <c r="B4" s="138" t="s">
         <v>228</v>
       </c>
       <c r="C4" s="85">
@@ -31710,7 +31719,7 @@
       <c r="A5" s="81" t="s">
         <v>224</v>
       </c>
-      <c r="B5" s="139" t="s">
+      <c r="B5" s="138" t="s">
         <v>229</v>
       </c>
       <c r="C5" s="85">
@@ -31745,7 +31754,7 @@
       <c r="A6" s="81" t="s">
         <v>230</v>
       </c>
-      <c r="B6" s="139" t="s">
+      <c r="B6" s="138" t="s">
         <v>231</v>
       </c>
       <c r="C6" s="85">
@@ -31780,7 +31789,7 @@
       <c r="A7" s="81" t="s">
         <v>232</v>
       </c>
-      <c r="B7" s="139" t="s">
+      <c r="B7" s="138" t="s">
         <v>233</v>
       </c>
       <c r="C7" s="85">
@@ -31815,7 +31824,7 @@
       <c r="A8" s="81" t="s">
         <v>226</v>
       </c>
-      <c r="B8" s="139" t="s">
+      <c r="B8" s="138" t="s">
         <v>234</v>
       </c>
       <c r="C8" s="85">
@@ -31850,7 +31859,7 @@
       <c r="A9" s="81" t="s">
         <v>226</v>
       </c>
-      <c r="B9" s="139" t="s">
+      <c r="B9" s="138" t="s">
         <v>235</v>
       </c>
       <c r="C9" s="85">
@@ -31885,7 +31894,7 @@
       <c r="A10" s="81" t="s">
         <v>230</v>
       </c>
-      <c r="B10" s="139" t="s">
+      <c r="B10" s="138" t="s">
         <v>236</v>
       </c>
       <c r="C10" s="85">

</xml_diff>